<commit_message>
docs: agregar evidencias profesionales al excel y diagrama
</commit_message>
<xml_diff>
--- a/docs/entregables/PRACTICA EMPRESARIAL/GRUPO2_FIREFOX_MATRICES_COMPLETAS.xlsx
+++ b/docs/entregables/PRACTICA EMPRESARIAL/GRUPO2_FIREFOX_MATRICES_COMPLETAS.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz 1 - Seguimiento" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz 2 - Evidencias" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz 3 - Dificultades" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Matriz 1 - Seguimiento" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Matriz 2 - Evidencias" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Matriz 3 - Dificultades" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -613,7 +613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G99"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="32" customWidth="1" style="28" min="1" max="1"/>
@@ -751,10 +751,11 @@
       <c r="C8" s="13" t="inlineStr">
         <is>
           <t>✓ DISPONIBLE:
-• Diagrama Entidad-Relación (DER) actualizado con campos de estado y TTL.
-• Diagramas de secuencia del flujo de reserva con SELECT FOR UPDATE.
-• Repositorio Git con módulo transaccional implementado.
-• Pruebas de concurrencia automatizadas (prevención de race condition).</t>
+• Diagrama ER y de Secuencia (SELECT FOR UPDATE).
+• Repositorio Git y Tests de Concurrencia.
+• Auditoría de Transacciones (Logs).
+• Documentación de APIs (Swagger/OpenAPI).
+• Plan de Reversión (Rollback Plan).</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
@@ -796,10 +797,11 @@
       <c r="C9" s="16" t="inlineStr">
         <is>
           <t>✓ DISPONIBLE:
-• Documento de Arquitectura del Sistema (C4) y patrón CQRS.
-• Repositorio con lógica de lectura y escritura desacopladas.
-• Script base de pruebas de carga en K6.
-• Documento de evidencia de pruebas.</t>
+• Arquitectura C4 y Patrón CQRS.
+• Separación de Servicios (Lectura/Escritura).
+• Métricas de Latencia (Base vs Optimizada).
+• Infraestructura como Código (IaC).
+• Estrategia de Sincronización Eventual.</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
@@ -840,10 +842,12 @@
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>✓ DISPONIBLE:
-• Código de integración del caché Valkey (cache.py) con políticas de TTL.
-• Servicio de disponibilidad optimizado consultando primero en caché.
-• Infraestructura Vagrant y Docker Compose incluyendo el servicio Valkey.</t>
+          <t>○ PENDIENTE DE RESPALDO:
+• Integración Caché Valkey (cache.py).
+• Infraestructura Docker/Vagrant.
+• Políticas de Invalidación de Caché (TTL).
+• Métricas de Cache Hit/Miss Ratio.
+• Pruebas de Resiliencia (Circuit Breakers).</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">
@@ -868,7 +872,7 @@
       </c>
       <c r="G10" s="19" t="inlineStr">
         <is>
-          <t>Completado</t>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
@@ -885,11 +889,12 @@
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>✓ DISPONIBLE:
-• Documento formal de Protocolo de Pruebas de Estrés.
-• Script completo en K6 (load_test_k6.js) con rampas y SLAs.
-• Guía para la generación de logs (como_generar_logs.md).
-• Plan Maestro y de Ejecución consolidados.</t>
+          <t>○ PENDIENTE DE RESPALDO:
+• Protocolo Pruebas K6 y Scripts de Carga.
+• Guía de Logs y Plan Maestro.
+• Reporte de Cuellos de Botella (Análisis de CPU/Memoria).
+• Políticas de Auto-escalado.
+• Matriz de Riesgos y Mitigaciones.</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr">
@@ -913,7 +918,7 @@
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Completado</t>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
@@ -930,6 +935,14 @@
       <c r="F12" s="30" t="n"/>
       <c r="G12" s="31" t="n"/>
     </row>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21" ht="15.75" customHeight="1" s="28"/>
     <row r="22" ht="15.75" customHeight="1" s="28"/>
     <row r="23" ht="15.75" customHeight="1" s="28"/>
@@ -1931,7 +1944,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="36" customWidth="1" style="28" min="1" max="1"/>
@@ -2028,7 +2041,7 @@
     <row r="8" ht="49.5" customHeight="1" s="28">
       <c r="A8" s="25" t="inlineStr">
         <is>
-          <t>Diagrama ER del prototipo</t>
+          <t>Diagrama ER y Secuencia</t>
         </is>
       </c>
       <c r="B8" s="25" t="inlineStr">
@@ -2038,12 +2051,12 @@
       </c>
       <c r="C8" s="25" t="inlineStr">
         <is>
-          <t>Estructura de BD: tablas de vuelos, asientos y reservas con soporte para concurrencia.</t>
+          <t>Estructuras y flujos para evitar race conditions.</t>
         </is>
       </c>
       <c r="D8" s="25" t="inlineStr">
         <is>
-          <t>docs/diagramas/diagrama_er.md</t>
+          <t>docs/diagramas/</t>
         </is>
       </c>
       <c r="E8" s="25" t="inlineStr">
@@ -2055,7 +2068,7 @@
     <row r="9" ht="49.5" customHeight="1" s="28">
       <c r="A9" s="25" t="inlineStr">
         <is>
-          <t>Diagramas de secuencia de reservas</t>
+          <t>Repositorio Git y Tests</t>
         </is>
       </c>
       <c r="B9" s="25" t="inlineStr">
@@ -2065,12 +2078,12 @@
       </c>
       <c r="C9" s="25" t="inlineStr">
         <is>
-          <t>Flujos de bloqueo pesimista, reservas provisionales (TTL) y confirmaciones.</t>
+          <t>Código fuente y pruebas automatizadas (pytest).</t>
         </is>
       </c>
       <c r="D9" s="25" t="inlineStr">
         <is>
-          <t>docs/diagramas/diagrama_secuencia_reserva.md</t>
+          <t>app/services/</t>
         </is>
       </c>
       <c r="E9" s="25" t="inlineStr">
@@ -2082,7 +2095,7 @@
     <row r="10" ht="49.5" customHeight="1" s="28">
       <c r="A10" s="25" t="inlineStr">
         <is>
-          <t>Repositorio Git - Módulo transaccional</t>
+          <t>Auditoría de Transacciones</t>
         </is>
       </c>
       <c r="B10" s="25" t="inlineStr">
@@ -2092,12 +2105,12 @@
       </c>
       <c r="C10" s="25" t="inlineStr">
         <is>
-          <t>Código fuente del bloqueo pesimista en PostgreSQL para evitar race conditions.</t>
+          <t>Logs de auditoría de bloqueos exitosos y fallidos.</t>
         </is>
       </c>
       <c r="D10" s="25" t="inlineStr">
         <is>
-          <t>app/services/reserva_service.py</t>
+          <t>docs/testing/</t>
         </is>
       </c>
       <c r="E10" s="25" t="inlineStr">
@@ -2109,7 +2122,7 @@
     <row r="11" ht="49.5" customHeight="1" s="28">
       <c r="A11" s="25" t="inlineStr">
         <is>
-          <t>Tests de concurrencia y endpoints</t>
+          <t>Especificación OpenAPI/Swagger</t>
         </is>
       </c>
       <c r="B11" s="25" t="inlineStr">
@@ -2119,12 +2132,12 @@
       </c>
       <c r="C11" s="25" t="inlineStr">
         <is>
-          <t>Pruebas automatizadas (pytest) verificando la integridad de asignación única.</t>
+          <t>Contrato de la API para integración de reservas.</t>
         </is>
       </c>
       <c r="D11" s="25" t="inlineStr">
         <is>
-          <t>tests/test_concurrency.py</t>
+          <t>docs/api/</t>
         </is>
       </c>
       <c r="E11" s="25" t="inlineStr">
@@ -2136,22 +2149,22 @@
     <row r="12" ht="49.5" customHeight="1" s="28">
       <c r="A12" s="25" t="inlineStr">
         <is>
-          <t>Arquitectura C4 y CQRS</t>
+          <t>Plan de Reversión (Rollback)</t>
         </is>
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
-          <t>Obj. 2 - Validación de disponibilidad</t>
+          <t>Obj. 1 - Bloqueo transaccional</t>
         </is>
       </c>
       <c r="C12" s="25" t="inlineStr">
         <is>
-          <t>Separación estratégica de operaciones de lectura rápida y escrituras transaccionales.</t>
+          <t>Estrategia de recuperación ante fallos de bloqueo.</t>
         </is>
       </c>
       <c r="D12" s="25" t="inlineStr">
         <is>
-          <t>docs/arquitectura/arquitectura_sistema.md</t>
+          <t>docs/arquitectura/</t>
         </is>
       </c>
       <c r="E12" s="25" t="inlineStr">
@@ -2163,7 +2176,7 @@
     <row r="13" ht="49.5" customHeight="1" s="28">
       <c r="A13" s="25" t="inlineStr">
         <is>
-          <t>Separación de servicios (CQRS)</t>
+          <t>Arquitectura C4 y CQRS</t>
         </is>
       </c>
       <c r="B13" s="25" t="inlineStr">
@@ -2173,12 +2186,12 @@
       </c>
       <c r="C13" s="25" t="inlineStr">
         <is>
-          <t>Lógica desacoplada en el backend para manejar alta demanda de lectura sin afectar compras.</t>
+          <t>Separación de lecturas/escrituras para alto tráfico.</t>
         </is>
       </c>
       <c r="D13" s="25" t="inlineStr">
         <is>
-          <t>app/services/disponibilidad_service.py</t>
+          <t>docs/arquitectura/</t>
         </is>
       </c>
       <c r="E13" s="25" t="inlineStr">
@@ -2190,25 +2203,25 @@
     <row r="14" ht="6.75" customHeight="1" s="28">
       <c r="A14" s="33" t="inlineStr">
         <is>
-          <t>Capa de Caché Valkey implementada</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Obj. 3 - Capa de caché</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Implementación de caché con políticas TTL por tipo de dato para descongestionar la DB.</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>app/db/cache.py</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
+          <t>Separación de Servicios</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>Obj. 2 - Validación de disponibilidad</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Microservicios de reserva y disponibilidad desacoplados.</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>app/services/</t>
+        </is>
+      </c>
+      <c r="E14" s="0" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -2217,25 +2230,25 @@
     <row r="15" ht="18" customHeight="1" s="28">
       <c r="A15" s="40" t="inlineStr">
         <is>
-          <t>Protocolo de Pruebas de Estrés</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Obj. 4 - Protocolo de estrés</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Definición de rampas de carga, métricas de éxito y criterios de falla para las simulaciones.</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>docs/testing/protocolo_pruebas_estres.md</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
+          <t>Métricas Base vs Optimizada</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>Obj. 2 - Validación de disponibilidad</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Comparativa de latencia antes y después de CQRS.</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>docs/testing/</t>
+        </is>
+      </c>
+      <c r="E15" s="0" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -2244,22 +2257,22 @@
     <row r="16" ht="51.75" customHeight="1" s="28">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>Script de Pruebas de Carga K6</t>
+          <t>Infraestructura como Código</t>
         </is>
       </c>
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>Obj. 4 - Protocolo de estrés</t>
+          <t>Obj. 2 - Validación de disponibilidad</t>
         </is>
       </c>
       <c r="C16" s="27" t="inlineStr">
         <is>
-          <t>Código ejecutable para someter el servidor a tráfico concurrente simulando Vuelos Azules.</t>
+          <t>Definiciones Docker Compose de los servicios.</t>
         </is>
       </c>
       <c r="D16" s="27" t="inlineStr">
         <is>
-          <t>scripts/load_test_k6.js</t>
+          <t>docker/</t>
         </is>
       </c>
       <c r="E16" s="27" t="inlineStr">
@@ -2271,22 +2284,22 @@
     <row r="17" ht="51.75" customHeight="1" s="28">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>Guía de Generación de Logs</t>
+          <t>Sincronización Eventual</t>
         </is>
       </c>
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>Obj. 4 - Protocolo de estrés</t>
+          <t>Obj. 2 - Validación de disponibilidad</t>
         </is>
       </c>
       <c r="C17" s="27" t="inlineStr">
         <is>
-          <t>Instrucciones de auditoría y captura de métricas durante la prueba de carga.</t>
+          <t>Mecanismo de propagación de datos al read-model.</t>
         </is>
       </c>
       <c r="D17" s="27" t="inlineStr">
         <is>
-          <t>docs/testing/como_generar_logs.md</t>
+          <t>docs/arquitectura/</t>
         </is>
       </c>
       <c r="E17" s="27" t="inlineStr">
@@ -2298,95 +2311,279 @@
     <row r="18" ht="51.75" customHeight="1" s="28">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>Plan Maestro de Ejecución</t>
+          <t>Código Integración Valkey</t>
         </is>
       </c>
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>Todos los objetivos</t>
+          <t>Obj. 3 - Capa de caché</t>
         </is>
       </c>
       <c r="C18" s="27" t="inlineStr">
         <is>
-          <t>Alineación del desarrollo con metodologías profesionales y objetivos del proyecto.</t>
+          <t>Implementación de caché intermedia en Python.</t>
         </is>
       </c>
       <c r="D18" s="27" t="inlineStr">
         <is>
-          <t>docs/planificacion/plan_maestro_boa.md</t>
+          <t>app/db/</t>
         </is>
       </c>
       <c r="E18" s="27" t="inlineStr">
         <is>
-          <t>Disponible</t>
+          <t>○ Pendiente</t>
         </is>
       </c>
     </row>
     <row r="19" ht="51.75" customHeight="1" s="28">
-      <c r="A19" s="27" t="inlineStr"/>
-      <c r="B19" s="27" t="inlineStr"/>
-      <c r="C19" s="27" t="inlineStr"/>
-      <c r="D19" s="27" t="inlineStr"/>
-      <c r="E19" s="27" t="inlineStr"/>
+      <c r="A19" s="27" t="inlineStr">
+        <is>
+          <t>Infraestructura Caché (Docker)</t>
+        </is>
+      </c>
+      <c r="B19" s="27" t="inlineStr">
+        <is>
+          <t>Obj. 3 - Capa de caché</t>
+        </is>
+      </c>
+      <c r="C19" s="27" t="inlineStr">
+        <is>
+          <t>Despliegue del nodo Valkey.</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
+        <is>
+          <t>docker/</t>
+        </is>
+      </c>
+      <c r="E19" s="27" t="inlineStr">
+        <is>
+          <t>○ Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="51.75" customHeight="1" s="28">
-      <c r="A20" s="27" t="inlineStr"/>
-      <c r="B20" s="27" t="inlineStr"/>
-      <c r="C20" s="27" t="inlineStr"/>
-      <c r="D20" s="27" t="inlineStr"/>
-      <c r="E20" s="27" t="inlineStr"/>
+      <c r="A20" s="27" t="inlineStr">
+        <is>
+          <t>Políticas de Invalidación y TTL</t>
+        </is>
+      </c>
+      <c r="B20" s="27" t="inlineStr">
+        <is>
+          <t>Obj. 3 - Capa de caché</t>
+        </is>
+      </c>
+      <c r="C20" s="27" t="inlineStr">
+        <is>
+          <t>Reglas de expiración de vuelos, asientos y tarifas.</t>
+        </is>
+      </c>
+      <c r="D20" s="27" t="inlineStr">
+        <is>
+          <t>docs/arquitectura/</t>
+        </is>
+      </c>
+      <c r="E20" s="27" t="inlineStr">
+        <is>
+          <t>○ Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="51.75" customHeight="1" s="28">
-      <c r="A21" s="27" t="inlineStr"/>
-      <c r="B21" s="27" t="inlineStr"/>
-      <c r="C21" s="27" t="inlineStr"/>
-      <c r="D21" s="27" t="inlineStr"/>
-      <c r="E21" s="27" t="inlineStr"/>
+      <c r="A21" s="27" t="inlineStr">
+        <is>
+          <t>Métricas Hit/Miss Ratio</t>
+        </is>
+      </c>
+      <c r="B21" s="27" t="inlineStr">
+        <is>
+          <t>Obj. 3 - Capa de caché</t>
+        </is>
+      </c>
+      <c r="C21" s="27" t="inlineStr">
+        <is>
+          <t>Eficiencia del caché bajo alta demanda.</t>
+        </is>
+      </c>
+      <c r="D21" s="27" t="inlineStr">
+        <is>
+          <t>docs/testing/</t>
+        </is>
+      </c>
+      <c r="E21" s="27" t="inlineStr">
+        <is>
+          <t>○ Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="51.75" customHeight="1" s="28">
-      <c r="A22" s="27" t="inlineStr"/>
-      <c r="B22" s="27" t="inlineStr"/>
-      <c r="C22" s="27" t="inlineStr"/>
-      <c r="D22" s="27" t="inlineStr"/>
-      <c r="E22" s="27" t="inlineStr"/>
+      <c r="A22" s="27" t="inlineStr">
+        <is>
+          <t>Pruebas de Resiliencia</t>
+        </is>
+      </c>
+      <c r="B22" s="27" t="inlineStr">
+        <is>
+          <t>Obj. 3 - Capa de caché</t>
+        </is>
+      </c>
+      <c r="C22" s="27" t="inlineStr">
+        <is>
+          <t>Simulación de caída de caché (Circuit Breaker).</t>
+        </is>
+      </c>
+      <c r="D22" s="27" t="inlineStr">
+        <is>
+          <t>docs/testing/</t>
+        </is>
+      </c>
+      <c r="E22" s="27" t="inlineStr">
+        <is>
+          <t>○ Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="51.75" customHeight="1" s="28">
-      <c r="A23" s="27" t="inlineStr"/>
-      <c r="B23" s="27" t="inlineStr"/>
-      <c r="C23" s="27" t="inlineStr"/>
-      <c r="D23" s="27" t="inlineStr"/>
-      <c r="E23" s="27" t="inlineStr"/>
+      <c r="A23" s="27" t="inlineStr">
+        <is>
+          <t>Protocolo Pruebas K6 y Scripts</t>
+        </is>
+      </c>
+      <c r="B23" s="27" t="inlineStr">
+        <is>
+          <t>Obj. 4 - Protocolo de estrés</t>
+        </is>
+      </c>
+      <c r="C23" s="27" t="inlineStr">
+        <is>
+          <t>Rampas de carga masiva simulando Vuelos Azules.</t>
+        </is>
+      </c>
+      <c r="D23" s="27" t="inlineStr">
+        <is>
+          <t>scripts/</t>
+        </is>
+      </c>
+      <c r="E23" s="27" t="inlineStr">
+        <is>
+          <t>○ Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="51.75" customHeight="1" s="28">
-      <c r="A24" s="27" t="inlineStr"/>
-      <c r="B24" s="27" t="inlineStr"/>
-      <c r="C24" s="27" t="inlineStr"/>
-      <c r="D24" s="27" t="inlineStr"/>
-      <c r="E24" s="27" t="inlineStr"/>
+      <c r="A24" s="27" t="inlineStr">
+        <is>
+          <t>Guía de Logs y Plan Maestro</t>
+        </is>
+      </c>
+      <c r="B24" s="27" t="inlineStr">
+        <is>
+          <t>Obj. 4 - Protocolo de estrés</t>
+        </is>
+      </c>
+      <c r="C24" s="27" t="inlineStr">
+        <is>
+          <t>Auditoría, planificación y metodologías.</t>
+        </is>
+      </c>
+      <c r="D24" s="27" t="inlineStr">
+        <is>
+          <t>docs/</t>
+        </is>
+      </c>
+      <c r="E24" s="27" t="inlineStr">
+        <is>
+          <t>○ Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="51.75" customHeight="1" s="28">
-      <c r="A25" s="27" t="inlineStr"/>
-      <c r="B25" s="27" t="inlineStr"/>
-      <c r="C25" s="27" t="inlineStr"/>
-      <c r="D25" s="27" t="inlineStr"/>
-      <c r="E25" s="27" t="inlineStr"/>
+      <c r="A25" s="27" t="inlineStr">
+        <is>
+          <t>Reporte de Cuellos de Botella</t>
+        </is>
+      </c>
+      <c r="B25" s="27" t="inlineStr">
+        <is>
+          <t>Obj. 4 - Protocolo de estrés</t>
+        </is>
+      </c>
+      <c r="C25" s="27" t="inlineStr">
+        <is>
+          <t>Análisis de profiling (CPU/Memoria) post-estrés.</t>
+        </is>
+      </c>
+      <c r="D25" s="27" t="inlineStr">
+        <is>
+          <t>docs/testing/</t>
+        </is>
+      </c>
+      <c r="E25" s="27" t="inlineStr">
+        <is>
+          <t>○ Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="51.75" customHeight="1" s="28">
-      <c r="A26" s="27" t="inlineStr"/>
-      <c r="B26" s="27" t="inlineStr"/>
-      <c r="C26" s="27" t="inlineStr"/>
-      <c r="D26" s="27" t="inlineStr"/>
-      <c r="E26" s="27" t="inlineStr"/>
+      <c r="A26" s="27" t="inlineStr">
+        <is>
+          <t>Políticas de Auto-escalado</t>
+        </is>
+      </c>
+      <c r="B26" s="27" t="inlineStr">
+        <is>
+          <t>Obj. 4 - Protocolo de estrés</t>
+        </is>
+      </c>
+      <c r="C26" s="27" t="inlineStr">
+        <is>
+          <t>Umbrales y reglas para escalar contenedores.</t>
+        </is>
+      </c>
+      <c r="D26" s="27" t="inlineStr">
+        <is>
+          <t>docs/arquitectura/</t>
+        </is>
+      </c>
+      <c r="E26" s="27" t="inlineStr">
+        <is>
+          <t>○ Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="51.75" customHeight="1" s="28">
-      <c r="A27" s="27" t="inlineStr"/>
-      <c r="B27" s="27" t="inlineStr"/>
-      <c r="C27" s="27" t="inlineStr"/>
-      <c r="D27" s="27" t="inlineStr"/>
-      <c r="E27" s="27" t="inlineStr"/>
+      <c r="A27" s="27" t="inlineStr">
+        <is>
+          <t>Matriz de Riesgos y Mitigaciones</t>
+        </is>
+      </c>
+      <c r="B27" s="27" t="inlineStr">
+        <is>
+          <t>Obj. 4 - Protocolo de estrés</t>
+        </is>
+      </c>
+      <c r="C27" s="27" t="inlineStr">
+        <is>
+          <t>Identificación de fallos en producción y contingencias.</t>
+        </is>
+      </c>
+      <c r="D27" s="27" t="inlineStr">
+        <is>
+          <t>docs/planificacion/</t>
+        </is>
+      </c>
+      <c r="E27" s="27" t="inlineStr">
+        <is>
+          <t>○ Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="31.5" customHeight="1" s="28">
       <c r="A28" s="36" t="inlineStr"/>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="28">
       <c r="A29" s="0" t="inlineStr"/>
@@ -2395,16 +2592,76 @@
       <c r="D29" s="0" t="inlineStr"/>
       <c r="E29" s="0" t="inlineStr"/>
     </row>
-    <row r="30" ht="15.75" customHeight="1" s="28"/>
-    <row r="31" ht="15.75" customHeight="1" s="28"/>
-    <row r="32" ht="15.75" customHeight="1" s="28"/>
-    <row r="33" ht="15.75" customHeight="1" s="28"/>
-    <row r="34" ht="15.75" customHeight="1" s="28"/>
-    <row r="35" ht="15.75" customHeight="1" s="28"/>
-    <row r="36" ht="15.75" customHeight="1" s="28"/>
-    <row r="37" ht="15.75" customHeight="1" s="28"/>
-    <row r="38" ht="15.75" customHeight="1" s="28"/>
-    <row r="39" ht="15.75" customHeight="1" s="28"/>
+    <row r="30" ht="15.75" customHeight="1" s="28">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+    </row>
+    <row r="31" ht="15.75" customHeight="1" s="28">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+    </row>
+    <row r="32" ht="15.75" customHeight="1" s="28">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+    </row>
+    <row r="33" ht="15.75" customHeight="1" s="28">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+    </row>
+    <row r="34" ht="15.75" customHeight="1" s="28">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+    </row>
+    <row r="35" ht="15.75" customHeight="1" s="28">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+    </row>
+    <row r="36" ht="15.75" customHeight="1" s="28">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+    </row>
+    <row r="37" ht="15.75" customHeight="1" s="28">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+    </row>
+    <row r="38" ht="15.75" customHeight="1" s="28">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+    </row>
+    <row r="39" ht="15.75" customHeight="1" s="28">
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+    </row>
     <row r="40" ht="15.75" customHeight="1" s="28"/>
     <row r="41" ht="15.75" customHeight="1" s="28"/>
     <row r="42" ht="15.75" customHeight="1" s="28"/>

</xml_diff>

<commit_message>
docs: agregar mapa visual de entregables directamente dentro del excel
</commit_message>
<xml_diff>
--- a/docs/entregables/PRACTICA EMPRESARIAL/GRUPO2_FIREFOX_MATRICES_COMPLETAS.xlsx
+++ b/docs/entregables/PRACTICA EMPRESARIAL/GRUPO2_FIREFOX_MATRICES_COMPLETAS.xlsx
@@ -3,9 +3,10 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Matriz 1 - Seguimiento" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Matriz 2 - Evidencias" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Matriz 3 - Dificultades" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Mapa Visual Evidencias" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Matriz 1 - Seguimiento" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Matriz 2 - Evidencias" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Matriz 3 - Dificultades" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -15,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -80,8 +81,17 @@
       <color rgb="FF5D4037"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -160,8 +170,38 @@
         <bgColor rgb="FFFFF8E1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004F81BD"/>
+        <bgColor rgb="004F81BD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border/>
     <border>
       <left style="thin">
@@ -220,11 +260,17 @@
         <color rgb="FFBFBFBF"/>
       </top>
     </border>
+    <border>
+      <left style="medium"/>
+      <right style="medium"/>
+      <top style="medium"/>
+      <bottom style="medium"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -337,6 +383,25 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="12" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="17" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -613,7 +678,269 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G99"/>
+  <dimension ref="A1:C21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" style="28" min="1" max="1"/>
+    <col width="60" customWidth="1" style="28" min="2" max="2"/>
+    <col width="20" customWidth="1" style="28" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="41" t="inlineStr">
+        <is>
+          <t>OBJETIVO GENERAL</t>
+        </is>
+      </c>
+      <c r="B1" s="41" t="inlineStr">
+        <is>
+          <t>EVIDENCIAS A ENTREGAR (CUADROS CHICOS)</t>
+        </is>
+      </c>
+      <c r="C1" s="41" t="inlineStr">
+        <is>
+          <t>ESTADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="42" t="inlineStr">
+        <is>
+          <t>OBJETIVO 1
+Bloqueo Transaccional</t>
+        </is>
+      </c>
+      <c r="B2" s="43" t="inlineStr">
+        <is>
+          <t>Evidencia 1: Diagrama ER y Secuencia</t>
+        </is>
+      </c>
+      <c r="C2" s="42" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="44" t="n"/>
+      <c r="B3" s="43" t="inlineStr">
+        <is>
+          <t>Evidencia 2: Repositorio Git y Tests</t>
+        </is>
+      </c>
+      <c r="C3" s="44" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="44" t="n"/>
+      <c r="B4" s="43" t="inlineStr">
+        <is>
+          <t>Evidencia 3: Auditoría de Transacciones Logs</t>
+        </is>
+      </c>
+      <c r="C4" s="44" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="44" t="n"/>
+      <c r="B5" s="43" t="inlineStr">
+        <is>
+          <t>Evidencia 4: Especificación OpenAPI/Swagger</t>
+        </is>
+      </c>
+      <c r="C5" s="44" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="44" t="n"/>
+      <c r="B6" s="43" t="inlineStr">
+        <is>
+          <t>Evidencia 5: Plan de Reversión Rollback</t>
+        </is>
+      </c>
+      <c r="C6" s="44" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="45" t="inlineStr">
+        <is>
+          <t>OBJETIVO 2
+Validación Disponibilidad</t>
+        </is>
+      </c>
+      <c r="B7" s="43" t="inlineStr">
+        <is>
+          <t>Evidencia 1: Arquitectura C4 y CQRS</t>
+        </is>
+      </c>
+      <c r="C7" s="45" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="44" t="n"/>
+      <c r="B8" s="43" t="inlineStr">
+        <is>
+          <t>Evidencia 2: Separación de Servicios</t>
+        </is>
+      </c>
+      <c r="C8" s="44" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="44" t="n"/>
+      <c r="B9" s="43" t="inlineStr">
+        <is>
+          <t>Evidencia 3: Métricas Base vs Optimizada</t>
+        </is>
+      </c>
+      <c r="C9" s="44" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="44" t="n"/>
+      <c r="B10" s="43" t="inlineStr">
+        <is>
+          <t>Evidencia 4: Infraestructura como Código</t>
+        </is>
+      </c>
+      <c r="C10" s="44" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="44" t="n"/>
+      <c r="B11" s="43" t="inlineStr">
+        <is>
+          <t>Evidencia 5: Sincronización Eventual</t>
+        </is>
+      </c>
+      <c r="C11" s="44" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="46" t="inlineStr">
+        <is>
+          <t>OBJETIVO 3
+Capa de Caché</t>
+        </is>
+      </c>
+      <c r="B12" s="43" t="inlineStr">
+        <is>
+          <t>Entregable 1: Código Integración Valkey</t>
+        </is>
+      </c>
+      <c r="C12" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="44" t="n"/>
+      <c r="B13" s="43" t="inlineStr">
+        <is>
+          <t>Entregable 2: Infraestructura Docker Caché</t>
+        </is>
+      </c>
+      <c r="C13" s="44" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="44" t="n"/>
+      <c r="B14" s="43" t="inlineStr">
+        <is>
+          <t>Entregable 3: Políticas de Invalidación TTL</t>
+        </is>
+      </c>
+      <c r="C14" s="44" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="44" t="n"/>
+      <c r="B15" s="43" t="inlineStr">
+        <is>
+          <t>Entregable 4: Métricas Hit/Miss Ratio</t>
+        </is>
+      </c>
+      <c r="C15" s="44" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="44" t="n"/>
+      <c r="B16" s="43" t="inlineStr">
+        <is>
+          <t>Entregable 5: Pruebas de Resiliencia</t>
+        </is>
+      </c>
+      <c r="C16" s="44" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="47" t="inlineStr">
+        <is>
+          <t>OBJETIVO 4
+Protocolo de Estrés</t>
+        </is>
+      </c>
+      <c r="B17" s="43" t="inlineStr">
+        <is>
+          <t>Entregable 1: Protocolo Pruebas K6 y Scripts</t>
+        </is>
+      </c>
+      <c r="C17" s="47" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="44" t="n"/>
+      <c r="B18" s="43" t="inlineStr">
+        <is>
+          <t>Entregable 2: Guía de Logs y Plan Maestro</t>
+        </is>
+      </c>
+      <c r="C18" s="44" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="44" t="n"/>
+      <c r="B19" s="43" t="inlineStr">
+        <is>
+          <t>Entregable 3: Reporte Cuellos de Botella</t>
+        </is>
+      </c>
+      <c r="C19" s="44" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="44" t="n"/>
+      <c r="B20" s="43" t="inlineStr">
+        <is>
+          <t>Entregable 4: Políticas de Auto-escalado</t>
+        </is>
+      </c>
+      <c r="C20" s="44" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="44" t="n"/>
+      <c r="B21" s="43" t="inlineStr">
+        <is>
+          <t>Entregable 5: Matriz Riesgos y Mitigaciones</t>
+        </is>
+      </c>
+      <c r="C21" s="44" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="C2:C6"/>
+    <mergeCell ref="A17:A21"/>
+    <mergeCell ref="A12:A16"/>
+    <mergeCell ref="C7:C11"/>
+    <mergeCell ref="C17:C21"/>
+    <mergeCell ref="A2:A6"/>
+    <mergeCell ref="C12:C16"/>
+    <mergeCell ref="A7:A11"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="32" customWidth="1" style="28" min="1" max="1"/>
@@ -935,14 +1262,6 @@
       <c r="F12" s="30" t="n"/>
       <c r="G12" s="31" t="n"/>
     </row>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21" ht="15.75" customHeight="1" s="28"/>
     <row r="22" ht="15.75" customHeight="1" s="28"/>
     <row r="23" ht="15.75" customHeight="1" s="28"/>
@@ -1938,7 +2257,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2580,10 +2899,10 @@
     </row>
     <row r="28" ht="31.5" customHeight="1" s="28">
       <c r="A28" s="36" t="inlineStr"/>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
+      <c r="B28" s="0" t="inlineStr"/>
+      <c r="C28" s="0" t="inlineStr"/>
+      <c r="D28" s="0" t="inlineStr"/>
+      <c r="E28" s="0" t="inlineStr"/>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="28">
       <c r="A29" s="0" t="inlineStr"/>
@@ -2593,74 +2912,74 @@
       <c r="E29" s="0" t="inlineStr"/>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="28">
-      <c r="A30" t="inlineStr"/>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
+      <c r="A30" s="0" t="inlineStr"/>
+      <c r="B30" s="0" t="inlineStr"/>
+      <c r="C30" s="0" t="inlineStr"/>
+      <c r="D30" s="0" t="inlineStr"/>
+      <c r="E30" s="0" t="inlineStr"/>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="28">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
+      <c r="A31" s="0" t="inlineStr"/>
+      <c r="B31" s="0" t="inlineStr"/>
+      <c r="C31" s="0" t="inlineStr"/>
+      <c r="D31" s="0" t="inlineStr"/>
+      <c r="E31" s="0" t="inlineStr"/>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="28">
-      <c r="A32" t="inlineStr"/>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
+      <c r="A32" s="0" t="inlineStr"/>
+      <c r="B32" s="0" t="inlineStr"/>
+      <c r="C32" s="0" t="inlineStr"/>
+      <c r="D32" s="0" t="inlineStr"/>
+      <c r="E32" s="0" t="inlineStr"/>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="28">
-      <c r="A33" t="inlineStr"/>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
+      <c r="A33" s="0" t="inlineStr"/>
+      <c r="B33" s="0" t="inlineStr"/>
+      <c r="C33" s="0" t="inlineStr"/>
+      <c r="D33" s="0" t="inlineStr"/>
+      <c r="E33" s="0" t="inlineStr"/>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="28">
-      <c r="A34" t="inlineStr"/>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
+      <c r="A34" s="0" t="inlineStr"/>
+      <c r="B34" s="0" t="inlineStr"/>
+      <c r="C34" s="0" t="inlineStr"/>
+      <c r="D34" s="0" t="inlineStr"/>
+      <c r="E34" s="0" t="inlineStr"/>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="28">
-      <c r="A35" t="inlineStr"/>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
+      <c r="A35" s="0" t="inlineStr"/>
+      <c r="B35" s="0" t="inlineStr"/>
+      <c r="C35" s="0" t="inlineStr"/>
+      <c r="D35" s="0" t="inlineStr"/>
+      <c r="E35" s="0" t="inlineStr"/>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="28">
-      <c r="A36" t="inlineStr"/>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
+      <c r="A36" s="0" t="inlineStr"/>
+      <c r="B36" s="0" t="inlineStr"/>
+      <c r="C36" s="0" t="inlineStr"/>
+      <c r="D36" s="0" t="inlineStr"/>
+      <c r="E36" s="0" t="inlineStr"/>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="28">
-      <c r="A37" t="inlineStr"/>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
+      <c r="A37" s="0" t="inlineStr"/>
+      <c r="B37" s="0" t="inlineStr"/>
+      <c r="C37" s="0" t="inlineStr"/>
+      <c r="D37" s="0" t="inlineStr"/>
+      <c r="E37" s="0" t="inlineStr"/>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="28">
-      <c r="A38" t="inlineStr"/>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
+      <c r="A38" s="0" t="inlineStr"/>
+      <c r="B38" s="0" t="inlineStr"/>
+      <c r="C38" s="0" t="inlineStr"/>
+      <c r="D38" s="0" t="inlineStr"/>
+      <c r="E38" s="0" t="inlineStr"/>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="28">
-      <c r="A39" t="inlineStr"/>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
+      <c r="A39" s="0" t="inlineStr"/>
+      <c r="B39" s="0" t="inlineStr"/>
+      <c r="C39" s="0" t="inlineStr"/>
+      <c r="D39" s="0" t="inlineStr"/>
+      <c r="E39" s="0" t="inlineStr"/>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="28"/>
     <row r="41" ht="15.75" customHeight="1" s="28"/>
@@ -3629,7 +3948,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
docs: completar matriz 3 de dificultades en excel
</commit_message>
<xml_diff>
--- a/docs/entregables/PRACTICA EMPRESARIAL/GRUPO2_FIREFOX_MATRICES_COMPLETAS.xlsx
+++ b/docs/entregables/PRACTICA EMPRESARIAL/GRUPO2_FIREFOX_MATRICES_COMPLETAS.xlsx
@@ -237,7 +237,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -324,6 +324,18 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1993,10 +2005,6 @@
           <t>✓ EVIDENCIAS DE PROYECTO (ACTUALIZADAS Y EXHAUSTIVAS)</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7" ht="49.5" customHeight="1" s="1">
       <c r="A7" s="18" t="inlineStr"/>
@@ -2527,1690 +2535,7 @@
     </row>
     <row r="28" ht="31.5" customHeight="1" s="1">
       <c r="A28" s="9" t="inlineStr"/>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-    </row>
-    <row r="29" ht="15.75" customHeight="1" s="1">
-      <c r="A29" t="inlineStr"/>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-    </row>
-    <row r="30" ht="15.75" customHeight="1" s="1">
-      <c r="A30" t="inlineStr"/>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-    </row>
-    <row r="31" ht="15.75" customHeight="1" s="1">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-    </row>
-    <row r="32" ht="15.75" customHeight="1" s="1">
-      <c r="A32" t="inlineStr"/>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-    </row>
-    <row r="33" ht="15.75" customHeight="1" s="1">
-      <c r="A33" t="inlineStr"/>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-    </row>
-    <row r="34" ht="15.75" customHeight="1" s="1">
-      <c r="A34" t="inlineStr"/>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-    </row>
-    <row r="35" ht="15.75" customHeight="1" s="1">
-      <c r="A35" t="inlineStr"/>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-    </row>
-    <row r="36" ht="15.75" customHeight="1" s="1">
-      <c r="A36" t="inlineStr"/>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-    </row>
-    <row r="37" ht="15.75" customHeight="1" s="1">
-      <c r="A37" t="inlineStr"/>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-    </row>
-    <row r="38" ht="15.75" customHeight="1" s="1">
-      <c r="A38" t="inlineStr"/>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-    </row>
-    <row r="39" ht="15.75" customHeight="1" s="1">
-      <c r="A39" t="inlineStr"/>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-    </row>
-    <row r="40" ht="15.75" customHeight="1" s="1">
-      <c r="A40" t="inlineStr"/>
-      <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
-    </row>
-    <row r="41" ht="15.75" customHeight="1" s="1">
-      <c r="A41" t="inlineStr"/>
-      <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-    </row>
-    <row r="42" ht="15.75" customHeight="1" s="1">
-      <c r="A42" t="inlineStr"/>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
-    </row>
-    <row r="43" ht="15.75" customHeight="1" s="1">
-      <c r="A43" t="inlineStr"/>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-    </row>
-    <row r="44" ht="15.75" customHeight="1" s="1">
-      <c r="A44" t="inlineStr"/>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-    </row>
-    <row r="45" ht="15.75" customHeight="1" s="1">
-      <c r="A45" t="inlineStr"/>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-    </row>
-    <row r="46" ht="15.75" customHeight="1" s="1">
-      <c r="A46" t="inlineStr"/>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-    </row>
-    <row r="47" ht="15.75" customHeight="1" s="1">
-      <c r="A47" t="inlineStr"/>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-    </row>
-    <row r="48" ht="15.75" customHeight="1" s="1">
-      <c r="A48" t="inlineStr"/>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-    </row>
-    <row r="49" ht="15.75" customHeight="1" s="1">
-      <c r="A49" t="inlineStr"/>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-    </row>
-    <row r="50" ht="15.75" customHeight="1" s="1">
-      <c r="A50" t="inlineStr"/>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-    </row>
-    <row r="51" ht="15.75" customHeight="1" s="1">
-      <c r="A51" t="inlineStr"/>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
-    </row>
-    <row r="52" ht="15.75" customHeight="1" s="1">
-      <c r="A52" t="inlineStr"/>
-      <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-    </row>
-    <row r="53" ht="15.75" customHeight="1" s="1">
-      <c r="A53" t="inlineStr"/>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
-    </row>
-    <row r="54" ht="15.75" customHeight="1" s="1">
-      <c r="A54" t="inlineStr"/>
-      <c r="B54" t="inlineStr"/>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-    </row>
-    <row r="55" ht="15.75" customHeight="1" s="1">
-      <c r="A55" t="inlineStr"/>
-      <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-    </row>
-    <row r="56" ht="15.75" customHeight="1" s="1">
-      <c r="A56" t="inlineStr"/>
-      <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
-    </row>
-    <row r="57" ht="15.75" customHeight="1" s="1">
-      <c r="A57" t="inlineStr"/>
-      <c r="B57" t="inlineStr"/>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
-    </row>
-    <row r="58" ht="15.75" customHeight="1" s="1">
-      <c r="A58" t="inlineStr"/>
-      <c r="B58" t="inlineStr"/>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
-    </row>
-    <row r="59" ht="15.75" customHeight="1" s="1">
-      <c r="A59" t="inlineStr"/>
-      <c r="B59" t="inlineStr"/>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr"/>
-    </row>
-    <row r="60" ht="15.75" customHeight="1" s="1">
-      <c r="A60" t="inlineStr"/>
-      <c r="B60" t="inlineStr"/>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
-    </row>
-    <row r="61" ht="15.75" customHeight="1" s="1">
-      <c r="A61" t="inlineStr"/>
-      <c r="B61" t="inlineStr"/>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
-    </row>
-    <row r="62" ht="15.75" customHeight="1" s="1">
-      <c r="A62" t="inlineStr"/>
-      <c r="B62" t="inlineStr"/>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-    </row>
-    <row r="63" ht="15.75" customHeight="1" s="1">
-      <c r="A63" t="inlineStr"/>
-      <c r="B63" t="inlineStr"/>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
-    </row>
-    <row r="64" ht="15.75" customHeight="1" s="1">
-      <c r="A64" t="inlineStr"/>
-      <c r="B64" t="inlineStr"/>
-      <c r="C64" t="inlineStr"/>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr"/>
-    </row>
-    <row r="65" ht="15.75" customHeight="1" s="1">
-      <c r="A65" t="inlineStr"/>
-      <c r="B65" t="inlineStr"/>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr"/>
-    </row>
-    <row r="66" ht="15.75" customHeight="1" s="1">
-      <c r="A66" t="inlineStr"/>
-      <c r="B66" t="inlineStr"/>
-      <c r="C66" t="inlineStr"/>
-      <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr"/>
-    </row>
-    <row r="67" ht="15.75" customHeight="1" s="1">
-      <c r="A67" t="inlineStr"/>
-      <c r="B67" t="inlineStr"/>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
-    </row>
-    <row r="68" ht="15.75" customHeight="1" s="1">
-      <c r="A68" t="inlineStr"/>
-      <c r="B68" t="inlineStr"/>
-      <c r="C68" t="inlineStr"/>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
-    </row>
-    <row r="69" ht="15.75" customHeight="1" s="1">
-      <c r="A69" t="inlineStr"/>
-      <c r="B69" t="inlineStr"/>
-      <c r="C69" t="inlineStr"/>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr"/>
-    </row>
-    <row r="70" ht="15.75" customHeight="1" s="1">
-      <c r="A70" t="inlineStr"/>
-      <c r="B70" t="inlineStr"/>
-      <c r="C70" t="inlineStr"/>
-      <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr"/>
-    </row>
-    <row r="71" ht="15.75" customHeight="1" s="1">
-      <c r="A71" t="inlineStr"/>
-      <c r="B71" t="inlineStr"/>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr"/>
-    </row>
-    <row r="72" ht="15.75" customHeight="1" s="1">
-      <c r="A72" t="inlineStr"/>
-      <c r="B72" t="inlineStr"/>
-      <c r="C72" t="inlineStr"/>
-      <c r="D72" t="inlineStr"/>
-      <c r="E72" t="inlineStr"/>
-    </row>
-    <row r="73" ht="15.75" customHeight="1" s="1">
-      <c r="A73" t="inlineStr"/>
-      <c r="B73" t="inlineStr"/>
-      <c r="C73" t="inlineStr"/>
-      <c r="D73" t="inlineStr"/>
-      <c r="E73" t="inlineStr"/>
-    </row>
-    <row r="74" ht="15.75" customHeight="1" s="1">
-      <c r="A74" t="inlineStr"/>
-      <c r="B74" t="inlineStr"/>
-      <c r="C74" t="inlineStr"/>
-      <c r="D74" t="inlineStr"/>
-      <c r="E74" t="inlineStr"/>
-    </row>
-    <row r="75" ht="15.75" customHeight="1" s="1">
-      <c r="A75" t="inlineStr"/>
-      <c r="B75" t="inlineStr"/>
-      <c r="C75" t="inlineStr"/>
-      <c r="D75" t="inlineStr"/>
-      <c r="E75" t="inlineStr"/>
-    </row>
-    <row r="76" ht="15.75" customHeight="1" s="1">
-      <c r="A76" t="inlineStr"/>
-      <c r="B76" t="inlineStr"/>
-      <c r="C76" t="inlineStr"/>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr"/>
-    </row>
-    <row r="77" ht="15.75" customHeight="1" s="1">
-      <c r="A77" t="inlineStr"/>
-      <c r="B77" t="inlineStr"/>
-      <c r="C77" t="inlineStr"/>
-      <c r="D77" t="inlineStr"/>
-      <c r="E77" t="inlineStr"/>
-    </row>
-    <row r="78" ht="15.75" customHeight="1" s="1">
-      <c r="A78" t="inlineStr"/>
-      <c r="B78" t="inlineStr"/>
-      <c r="C78" t="inlineStr"/>
-      <c r="D78" t="inlineStr"/>
-      <c r="E78" t="inlineStr"/>
-    </row>
-    <row r="79" ht="15.75" customHeight="1" s="1">
-      <c r="A79" t="inlineStr"/>
-      <c r="B79" t="inlineStr"/>
-      <c r="C79" t="inlineStr"/>
-      <c r="D79" t="inlineStr"/>
-      <c r="E79" t="inlineStr"/>
-    </row>
-    <row r="80" ht="15.75" customHeight="1" s="1">
-      <c r="A80" t="inlineStr"/>
-      <c r="B80" t="inlineStr"/>
-      <c r="C80" t="inlineStr"/>
-      <c r="D80" t="inlineStr"/>
-      <c r="E80" t="inlineStr"/>
-    </row>
-    <row r="81" ht="15.75" customHeight="1" s="1">
-      <c r="A81" t="inlineStr"/>
-      <c r="B81" t="inlineStr"/>
-      <c r="C81" t="inlineStr"/>
-      <c r="D81" t="inlineStr"/>
-      <c r="E81" t="inlineStr"/>
-    </row>
-    <row r="82" ht="15.75" customHeight="1" s="1">
-      <c r="A82" t="inlineStr"/>
-      <c r="B82" t="inlineStr"/>
-      <c r="C82" t="inlineStr"/>
-      <c r="D82" t="inlineStr"/>
-      <c r="E82" t="inlineStr"/>
-    </row>
-    <row r="83" ht="15.75" customHeight="1" s="1">
-      <c r="A83" t="inlineStr"/>
-      <c r="B83" t="inlineStr"/>
-      <c r="C83" t="inlineStr"/>
-      <c r="D83" t="inlineStr"/>
-      <c r="E83" t="inlineStr"/>
-    </row>
-    <row r="84" ht="15.75" customHeight="1" s="1">
-      <c r="A84" t="inlineStr"/>
-      <c r="B84" t="inlineStr"/>
-      <c r="C84" t="inlineStr"/>
-      <c r="D84" t="inlineStr"/>
-      <c r="E84" t="inlineStr"/>
-    </row>
-    <row r="85" ht="15.75" customHeight="1" s="1">
-      <c r="A85" t="inlineStr"/>
-      <c r="B85" t="inlineStr"/>
-      <c r="C85" t="inlineStr"/>
-      <c r="D85" t="inlineStr"/>
-      <c r="E85" t="inlineStr"/>
-    </row>
-    <row r="86" ht="15.75" customHeight="1" s="1">
-      <c r="A86" t="inlineStr"/>
-      <c r="B86" t="inlineStr"/>
-      <c r="C86" t="inlineStr"/>
-      <c r="D86" t="inlineStr"/>
-      <c r="E86" t="inlineStr"/>
-    </row>
-    <row r="87" ht="15.75" customHeight="1" s="1">
-      <c r="A87" t="inlineStr"/>
-      <c r="B87" t="inlineStr"/>
-      <c r="C87" t="inlineStr"/>
-      <c r="D87" t="inlineStr"/>
-      <c r="E87" t="inlineStr"/>
-    </row>
-    <row r="88" ht="15.75" customHeight="1" s="1">
-      <c r="A88" t="inlineStr"/>
-      <c r="B88" t="inlineStr"/>
-      <c r="C88" t="inlineStr"/>
-      <c r="D88" t="inlineStr"/>
-      <c r="E88" t="inlineStr"/>
-    </row>
-    <row r="89" ht="15.75" customHeight="1" s="1">
-      <c r="A89" t="inlineStr"/>
-      <c r="B89" t="inlineStr"/>
-      <c r="C89" t="inlineStr"/>
-      <c r="D89" t="inlineStr"/>
-      <c r="E89" t="inlineStr"/>
-    </row>
-    <row r="90" ht="15.75" customHeight="1" s="1">
-      <c r="A90" t="inlineStr"/>
-      <c r="B90" t="inlineStr"/>
-      <c r="C90" t="inlineStr"/>
-      <c r="D90" t="inlineStr"/>
-      <c r="E90" t="inlineStr"/>
-    </row>
-    <row r="91" ht="15.75" customHeight="1" s="1">
-      <c r="A91" t="inlineStr"/>
-      <c r="B91" t="inlineStr"/>
-      <c r="C91" t="inlineStr"/>
-      <c r="D91" t="inlineStr"/>
-      <c r="E91" t="inlineStr"/>
-    </row>
-    <row r="92" ht="15.75" customHeight="1" s="1">
-      <c r="A92" t="inlineStr"/>
-      <c r="B92" t="inlineStr"/>
-      <c r="C92" t="inlineStr"/>
-      <c r="D92" t="inlineStr"/>
-      <c r="E92" t="inlineStr"/>
-    </row>
-    <row r="93" ht="15.75" customHeight="1" s="1">
-      <c r="A93" t="inlineStr"/>
-      <c r="B93" t="inlineStr"/>
-      <c r="C93" t="inlineStr"/>
-      <c r="D93" t="inlineStr"/>
-      <c r="E93" t="inlineStr"/>
-    </row>
-    <row r="94" ht="15.75" customHeight="1" s="1">
-      <c r="A94" t="inlineStr"/>
-      <c r="B94" t="inlineStr"/>
-      <c r="C94" t="inlineStr"/>
-      <c r="D94" t="inlineStr"/>
-      <c r="E94" t="inlineStr"/>
-    </row>
-    <row r="95" ht="15.75" customHeight="1" s="1">
-      <c r="A95" t="inlineStr"/>
-      <c r="B95" t="inlineStr"/>
-      <c r="C95" t="inlineStr"/>
-      <c r="D95" t="inlineStr"/>
-      <c r="E95" t="inlineStr"/>
-    </row>
-    <row r="96" ht="15.75" customHeight="1" s="1">
-      <c r="A96" t="inlineStr"/>
-      <c r="B96" t="inlineStr"/>
-      <c r="C96" t="inlineStr"/>
-      <c r="D96" t="inlineStr"/>
-      <c r="E96" t="inlineStr"/>
-    </row>
-    <row r="97" ht="15.75" customHeight="1" s="1">
-      <c r="A97" t="inlineStr"/>
-      <c r="B97" t="inlineStr"/>
-      <c r="C97" t="inlineStr"/>
-      <c r="D97" t="inlineStr"/>
-      <c r="E97" t="inlineStr"/>
-    </row>
-    <row r="98" ht="15.75" customHeight="1" s="1">
-      <c r="A98" t="inlineStr"/>
-      <c r="B98" t="inlineStr"/>
-      <c r="C98" t="inlineStr"/>
-      <c r="D98" t="inlineStr"/>
-      <c r="E98" t="inlineStr"/>
-    </row>
-    <row r="99" ht="15.75" customHeight="1" s="1">
-      <c r="A99" t="inlineStr"/>
-      <c r="B99" t="inlineStr"/>
-      <c r="C99" t="inlineStr"/>
-      <c r="D99" t="inlineStr"/>
-      <c r="E99" t="inlineStr"/>
-    </row>
-    <row r="100" ht="15.75" customHeight="1" s="1"/>
-    <row r="101" ht="15.75" customHeight="1" s="1"/>
-    <row r="102" ht="15.75" customHeight="1" s="1"/>
-    <row r="103" ht="15.75" customHeight="1" s="1"/>
-    <row r="104" ht="15.75" customHeight="1" s="1"/>
-    <row r="105" ht="15.75" customHeight="1" s="1"/>
-    <row r="106" ht="15.75" customHeight="1" s="1"/>
-    <row r="107" ht="15.75" customHeight="1" s="1"/>
-    <row r="108" ht="15.75" customHeight="1" s="1"/>
-    <row r="109" ht="15.75" customHeight="1" s="1"/>
-    <row r="110" ht="15.75" customHeight="1" s="1"/>
-    <row r="111" ht="15.75" customHeight="1" s="1"/>
-    <row r="112" ht="15.75" customHeight="1" s="1"/>
-    <row r="113" ht="15.75" customHeight="1" s="1"/>
-    <row r="114" ht="15.75" customHeight="1" s="1"/>
-    <row r="115" ht="15.75" customHeight="1" s="1"/>
-    <row r="116" ht="15.75" customHeight="1" s="1"/>
-    <row r="117" ht="15.75" customHeight="1" s="1"/>
-    <row r="118" ht="15.75" customHeight="1" s="1"/>
-    <row r="119" ht="15.75" customHeight="1" s="1"/>
-    <row r="120" ht="15.75" customHeight="1" s="1"/>
-    <row r="121" ht="15.75" customHeight="1" s="1"/>
-    <row r="122" ht="15.75" customHeight="1" s="1"/>
-    <row r="123" ht="15.75" customHeight="1" s="1"/>
-    <row r="124" ht="15.75" customHeight="1" s="1"/>
-    <row r="125" ht="15.75" customHeight="1" s="1"/>
-    <row r="126" ht="15.75" customHeight="1" s="1"/>
-    <row r="127" ht="15.75" customHeight="1" s="1"/>
-    <row r="128" ht="15.75" customHeight="1" s="1"/>
-    <row r="129" ht="15.75" customHeight="1" s="1"/>
-    <row r="130" ht="15.75" customHeight="1" s="1"/>
-    <row r="131" ht="15.75" customHeight="1" s="1"/>
-    <row r="132" ht="15.75" customHeight="1" s="1"/>
-    <row r="133" ht="15.75" customHeight="1" s="1"/>
-    <row r="134" ht="15.75" customHeight="1" s="1"/>
-    <row r="135" ht="15.75" customHeight="1" s="1"/>
-    <row r="136" ht="15.75" customHeight="1" s="1"/>
-    <row r="137" ht="15.75" customHeight="1" s="1"/>
-    <row r="138" ht="15.75" customHeight="1" s="1"/>
-    <row r="139" ht="15.75" customHeight="1" s="1"/>
-    <row r="140" ht="15.75" customHeight="1" s="1"/>
-    <row r="141" ht="15.75" customHeight="1" s="1"/>
-    <row r="142" ht="15.75" customHeight="1" s="1"/>
-    <row r="143" ht="15.75" customHeight="1" s="1"/>
-    <row r="144" ht="15.75" customHeight="1" s="1"/>
-    <row r="145" ht="15.75" customHeight="1" s="1"/>
-    <row r="146" ht="15.75" customHeight="1" s="1"/>
-    <row r="147" ht="15.75" customHeight="1" s="1"/>
-    <row r="148" ht="15.75" customHeight="1" s="1"/>
-    <row r="149" ht="15.75" customHeight="1" s="1"/>
-    <row r="150" ht="15.75" customHeight="1" s="1"/>
-    <row r="151" ht="15.75" customHeight="1" s="1"/>
-    <row r="152" ht="15.75" customHeight="1" s="1"/>
-    <row r="153" ht="15.75" customHeight="1" s="1"/>
-    <row r="154" ht="15.75" customHeight="1" s="1"/>
-    <row r="155" ht="15.75" customHeight="1" s="1"/>
-    <row r="156" ht="15.75" customHeight="1" s="1"/>
-    <row r="157" ht="15.75" customHeight="1" s="1"/>
-    <row r="158" ht="15.75" customHeight="1" s="1"/>
-    <row r="159" ht="15.75" customHeight="1" s="1"/>
-    <row r="160" ht="15.75" customHeight="1" s="1"/>
-    <row r="161" ht="15.75" customHeight="1" s="1"/>
-    <row r="162" ht="15.75" customHeight="1" s="1"/>
-    <row r="163" ht="15.75" customHeight="1" s="1"/>
-    <row r="164" ht="15.75" customHeight="1" s="1"/>
-    <row r="165" ht="15.75" customHeight="1" s="1"/>
-    <row r="166" ht="15.75" customHeight="1" s="1"/>
-    <row r="167" ht="15.75" customHeight="1" s="1"/>
-    <row r="168" ht="15.75" customHeight="1" s="1"/>
-    <row r="169" ht="15.75" customHeight="1" s="1"/>
-    <row r="170" ht="15.75" customHeight="1" s="1"/>
-    <row r="171" ht="15.75" customHeight="1" s="1"/>
-    <row r="172" ht="15.75" customHeight="1" s="1"/>
-    <row r="173" ht="15.75" customHeight="1" s="1"/>
-    <row r="174" ht="15.75" customHeight="1" s="1"/>
-    <row r="175" ht="15.75" customHeight="1" s="1"/>
-    <row r="176" ht="15.75" customHeight="1" s="1"/>
-    <row r="177" ht="15.75" customHeight="1" s="1"/>
-    <row r="178" ht="15.75" customHeight="1" s="1"/>
-    <row r="179" ht="15.75" customHeight="1" s="1"/>
-    <row r="180" ht="15.75" customHeight="1" s="1"/>
-    <row r="181" ht="15.75" customHeight="1" s="1"/>
-    <row r="182" ht="15.75" customHeight="1" s="1"/>
-    <row r="183" ht="15.75" customHeight="1" s="1"/>
-    <row r="184" ht="15.75" customHeight="1" s="1"/>
-    <row r="185" ht="15.75" customHeight="1" s="1"/>
-    <row r="186" ht="15.75" customHeight="1" s="1"/>
-    <row r="187" ht="15.75" customHeight="1" s="1"/>
-    <row r="188" ht="15.75" customHeight="1" s="1"/>
-    <row r="189" ht="15.75" customHeight="1" s="1"/>
-    <row r="190" ht="15.75" customHeight="1" s="1"/>
-    <row r="191" ht="15.75" customHeight="1" s="1"/>
-    <row r="192" ht="15.75" customHeight="1" s="1"/>
-    <row r="193" ht="15.75" customHeight="1" s="1"/>
-    <row r="194" ht="15.75" customHeight="1" s="1"/>
-    <row r="195" ht="15.75" customHeight="1" s="1"/>
-    <row r="196" ht="15.75" customHeight="1" s="1"/>
-    <row r="197" ht="15.75" customHeight="1" s="1"/>
-    <row r="198" ht="15.75" customHeight="1" s="1"/>
-    <row r="199" ht="15.75" customHeight="1" s="1"/>
-    <row r="200" ht="15.75" customHeight="1" s="1"/>
-    <row r="201" ht="15.75" customHeight="1" s="1"/>
-    <row r="202" ht="15.75" customHeight="1" s="1"/>
-    <row r="203" ht="15.75" customHeight="1" s="1"/>
-    <row r="204" ht="15.75" customHeight="1" s="1"/>
-    <row r="205" ht="15.75" customHeight="1" s="1"/>
-    <row r="206" ht="15.75" customHeight="1" s="1"/>
-    <row r="207" ht="15.75" customHeight="1" s="1"/>
-    <row r="208" ht="15.75" customHeight="1" s="1"/>
-    <row r="209" ht="15.75" customHeight="1" s="1"/>
-    <row r="210" ht="15.75" customHeight="1" s="1"/>
-    <row r="211" ht="15.75" customHeight="1" s="1"/>
-    <row r="212" ht="15.75" customHeight="1" s="1"/>
-    <row r="213" ht="15.75" customHeight="1" s="1"/>
-    <row r="214" ht="15.75" customHeight="1" s="1"/>
-    <row r="215" ht="15.75" customHeight="1" s="1"/>
-    <row r="216" ht="15.75" customHeight="1" s="1"/>
-    <row r="217" ht="15.75" customHeight="1" s="1"/>
-    <row r="218" ht="15.75" customHeight="1" s="1"/>
-    <row r="219" ht="15.75" customHeight="1" s="1"/>
-    <row r="220" ht="15.75" customHeight="1" s="1"/>
-    <row r="221" ht="15.75" customHeight="1" s="1"/>
-    <row r="222" ht="15.75" customHeight="1" s="1"/>
-    <row r="223" ht="15.75" customHeight="1" s="1"/>
-    <row r="224" ht="15.75" customHeight="1" s="1"/>
-    <row r="225" ht="15.75" customHeight="1" s="1"/>
-    <row r="226" ht="15.75" customHeight="1" s="1"/>
-    <row r="227" ht="15.75" customHeight="1" s="1"/>
-    <row r="228" ht="15.75" customHeight="1" s="1"/>
-    <row r="229" ht="15.75" customHeight="1" s="1"/>
-    <row r="230" ht="15.75" customHeight="1" s="1"/>
-    <row r="231" ht="15.75" customHeight="1" s="1"/>
-    <row r="232" ht="15.75" customHeight="1" s="1"/>
-    <row r="233" ht="15.75" customHeight="1" s="1"/>
-    <row r="234" ht="15.75" customHeight="1" s="1"/>
-    <row r="235" ht="15.75" customHeight="1" s="1"/>
-    <row r="236" ht="15.75" customHeight="1" s="1"/>
-    <row r="237" ht="15.75" customHeight="1" s="1"/>
-    <row r="238" ht="15.75" customHeight="1" s="1"/>
-    <row r="239" ht="15.75" customHeight="1" s="1"/>
-    <row r="240" ht="15.75" customHeight="1" s="1"/>
-    <row r="241" ht="15.75" customHeight="1" s="1"/>
-    <row r="242" ht="15.75" customHeight="1" s="1"/>
-    <row r="243" ht="15.75" customHeight="1" s="1"/>
-    <row r="244" ht="15.75" customHeight="1" s="1"/>
-    <row r="245" ht="15.75" customHeight="1" s="1"/>
-    <row r="246" ht="15.75" customHeight="1" s="1"/>
-    <row r="247" ht="15.75" customHeight="1" s="1"/>
-    <row r="248" ht="15.75" customHeight="1" s="1"/>
-    <row r="249" ht="15.75" customHeight="1" s="1"/>
-    <row r="250" ht="15.75" customHeight="1" s="1"/>
-    <row r="251" ht="15.75" customHeight="1" s="1"/>
-    <row r="252" ht="15.75" customHeight="1" s="1"/>
-    <row r="253" ht="15.75" customHeight="1" s="1"/>
-    <row r="254" ht="15.75" customHeight="1" s="1"/>
-    <row r="255" ht="15.75" customHeight="1" s="1"/>
-    <row r="256" ht="15.75" customHeight="1" s="1"/>
-    <row r="257" ht="15.75" customHeight="1" s="1"/>
-    <row r="258" ht="15.75" customHeight="1" s="1"/>
-    <row r="259" ht="15.75" customHeight="1" s="1"/>
-    <row r="260" ht="15.75" customHeight="1" s="1"/>
-    <row r="261" ht="15.75" customHeight="1" s="1"/>
-    <row r="262" ht="15.75" customHeight="1" s="1"/>
-    <row r="263" ht="15.75" customHeight="1" s="1"/>
-    <row r="264" ht="15.75" customHeight="1" s="1"/>
-    <row r="265" ht="15.75" customHeight="1" s="1"/>
-    <row r="266" ht="15.75" customHeight="1" s="1"/>
-    <row r="267" ht="15.75" customHeight="1" s="1"/>
-    <row r="268" ht="15.75" customHeight="1" s="1"/>
-    <row r="269" ht="15.75" customHeight="1" s="1"/>
-    <row r="270" ht="15.75" customHeight="1" s="1"/>
-    <row r="271" ht="15.75" customHeight="1" s="1"/>
-    <row r="272" ht="15.75" customHeight="1" s="1"/>
-    <row r="273" ht="15.75" customHeight="1" s="1"/>
-    <row r="274" ht="15.75" customHeight="1" s="1"/>
-    <row r="275" ht="15.75" customHeight="1" s="1"/>
-    <row r="276" ht="15.75" customHeight="1" s="1"/>
-    <row r="277" ht="15.75" customHeight="1" s="1"/>
-    <row r="278" ht="15.75" customHeight="1" s="1"/>
-    <row r="279" ht="15.75" customHeight="1" s="1"/>
-    <row r="280" ht="15.75" customHeight="1" s="1"/>
-    <row r="281" ht="15.75" customHeight="1" s="1"/>
-    <row r="282" ht="15.75" customHeight="1" s="1"/>
-    <row r="283" ht="15.75" customHeight="1" s="1"/>
-    <row r="284" ht="15.75" customHeight="1" s="1"/>
-    <row r="285" ht="15.75" customHeight="1" s="1"/>
-    <row r="286" ht="15.75" customHeight="1" s="1"/>
-    <row r="287" ht="15.75" customHeight="1" s="1"/>
-    <row r="288" ht="15.75" customHeight="1" s="1"/>
-    <row r="289" ht="15.75" customHeight="1" s="1"/>
-    <row r="290" ht="15.75" customHeight="1" s="1"/>
-    <row r="291" ht="15.75" customHeight="1" s="1"/>
-    <row r="292" ht="15.75" customHeight="1" s="1"/>
-    <row r="293" ht="15.75" customHeight="1" s="1"/>
-    <row r="294" ht="15.75" customHeight="1" s="1"/>
-    <row r="295" ht="15.75" customHeight="1" s="1"/>
-    <row r="296" ht="15.75" customHeight="1" s="1"/>
-    <row r="297" ht="15.75" customHeight="1" s="1"/>
-    <row r="298" ht="15.75" customHeight="1" s="1"/>
-    <row r="299" ht="15.75" customHeight="1" s="1"/>
-    <row r="300" ht="15.75" customHeight="1" s="1"/>
-    <row r="301" ht="15.75" customHeight="1" s="1"/>
-    <row r="302" ht="15.75" customHeight="1" s="1"/>
-    <row r="303" ht="15.75" customHeight="1" s="1"/>
-    <row r="304" ht="15.75" customHeight="1" s="1"/>
-    <row r="305" ht="15.75" customHeight="1" s="1"/>
-    <row r="306" ht="15.75" customHeight="1" s="1"/>
-    <row r="307" ht="15.75" customHeight="1" s="1"/>
-    <row r="308" ht="15.75" customHeight="1" s="1"/>
-    <row r="309" ht="15.75" customHeight="1" s="1"/>
-    <row r="310" ht="15.75" customHeight="1" s="1"/>
-    <row r="311" ht="15.75" customHeight="1" s="1"/>
-    <row r="312" ht="15.75" customHeight="1" s="1"/>
-    <row r="313" ht="15.75" customHeight="1" s="1"/>
-    <row r="314" ht="15.75" customHeight="1" s="1"/>
-    <row r="315" ht="15.75" customHeight="1" s="1"/>
-    <row r="316" ht="15.75" customHeight="1" s="1"/>
-    <row r="317" ht="15.75" customHeight="1" s="1"/>
-    <row r="318" ht="15.75" customHeight="1" s="1"/>
-    <row r="319" ht="15.75" customHeight="1" s="1"/>
-    <row r="320" ht="15.75" customHeight="1" s="1"/>
-    <row r="321" ht="15.75" customHeight="1" s="1"/>
-    <row r="322" ht="15.75" customHeight="1" s="1"/>
-    <row r="323" ht="15.75" customHeight="1" s="1"/>
-    <row r="324" ht="15.75" customHeight="1" s="1"/>
-    <row r="325" ht="15.75" customHeight="1" s="1"/>
-    <row r="326" ht="15.75" customHeight="1" s="1"/>
-    <row r="327" ht="15.75" customHeight="1" s="1"/>
-    <row r="328" ht="15.75" customHeight="1" s="1"/>
-    <row r="329" ht="15.75" customHeight="1" s="1"/>
-    <row r="330" ht="15.75" customHeight="1" s="1"/>
-    <row r="331" ht="15.75" customHeight="1" s="1"/>
-    <row r="332" ht="15.75" customHeight="1" s="1"/>
-    <row r="333" ht="15.75" customHeight="1" s="1"/>
-    <row r="334" ht="15.75" customHeight="1" s="1"/>
-    <row r="335" ht="15.75" customHeight="1" s="1"/>
-    <row r="336" ht="15.75" customHeight="1" s="1"/>
-    <row r="337" ht="15.75" customHeight="1" s="1"/>
-    <row r="338" ht="15.75" customHeight="1" s="1"/>
-    <row r="339" ht="15.75" customHeight="1" s="1"/>
-    <row r="340" ht="15.75" customHeight="1" s="1"/>
-    <row r="341" ht="15.75" customHeight="1" s="1"/>
-    <row r="342" ht="15.75" customHeight="1" s="1"/>
-    <row r="343" ht="15.75" customHeight="1" s="1"/>
-    <row r="344" ht="15.75" customHeight="1" s="1"/>
-    <row r="345" ht="15.75" customHeight="1" s="1"/>
-    <row r="346" ht="15.75" customHeight="1" s="1"/>
-    <row r="347" ht="15.75" customHeight="1" s="1"/>
-    <row r="348" ht="15.75" customHeight="1" s="1"/>
-    <row r="349" ht="15.75" customHeight="1" s="1"/>
-    <row r="350" ht="15.75" customHeight="1" s="1"/>
-    <row r="351" ht="15.75" customHeight="1" s="1"/>
-    <row r="352" ht="15.75" customHeight="1" s="1"/>
-    <row r="353" ht="15.75" customHeight="1" s="1"/>
-    <row r="354" ht="15.75" customHeight="1" s="1"/>
-    <row r="355" ht="15.75" customHeight="1" s="1"/>
-    <row r="356" ht="15.75" customHeight="1" s="1"/>
-    <row r="357" ht="15.75" customHeight="1" s="1"/>
-    <row r="358" ht="15.75" customHeight="1" s="1"/>
-    <row r="359" ht="15.75" customHeight="1" s="1"/>
-    <row r="360" ht="15.75" customHeight="1" s="1"/>
-    <row r="361" ht="15.75" customHeight="1" s="1"/>
-    <row r="362" ht="15.75" customHeight="1" s="1"/>
-    <row r="363" ht="15.75" customHeight="1" s="1"/>
-    <row r="364" ht="15.75" customHeight="1" s="1"/>
-    <row r="365" ht="15.75" customHeight="1" s="1"/>
-    <row r="366" ht="15.75" customHeight="1" s="1"/>
-    <row r="367" ht="15.75" customHeight="1" s="1"/>
-    <row r="368" ht="15.75" customHeight="1" s="1"/>
-    <row r="369" ht="15.75" customHeight="1" s="1"/>
-    <row r="370" ht="15.75" customHeight="1" s="1"/>
-    <row r="371" ht="15.75" customHeight="1" s="1"/>
-    <row r="372" ht="15.75" customHeight="1" s="1"/>
-    <row r="373" ht="15.75" customHeight="1" s="1"/>
-    <row r="374" ht="15.75" customHeight="1" s="1"/>
-    <row r="375" ht="15.75" customHeight="1" s="1"/>
-    <row r="376" ht="15.75" customHeight="1" s="1"/>
-    <row r="377" ht="15.75" customHeight="1" s="1"/>
-    <row r="378" ht="15.75" customHeight="1" s="1"/>
-    <row r="379" ht="15.75" customHeight="1" s="1"/>
-    <row r="380" ht="15.75" customHeight="1" s="1"/>
-    <row r="381" ht="15.75" customHeight="1" s="1"/>
-    <row r="382" ht="15.75" customHeight="1" s="1"/>
-    <row r="383" ht="15.75" customHeight="1" s="1"/>
-    <row r="384" ht="15.75" customHeight="1" s="1"/>
-    <row r="385" ht="15.75" customHeight="1" s="1"/>
-    <row r="386" ht="15.75" customHeight="1" s="1"/>
-    <row r="387" ht="15.75" customHeight="1" s="1"/>
-    <row r="388" ht="15.75" customHeight="1" s="1"/>
-    <row r="389" ht="15.75" customHeight="1" s="1"/>
-    <row r="390" ht="15.75" customHeight="1" s="1"/>
-    <row r="391" ht="15.75" customHeight="1" s="1"/>
-    <row r="392" ht="15.75" customHeight="1" s="1"/>
-    <row r="393" ht="15.75" customHeight="1" s="1"/>
-    <row r="394" ht="15.75" customHeight="1" s="1"/>
-    <row r="395" ht="15.75" customHeight="1" s="1"/>
-    <row r="396" ht="15.75" customHeight="1" s="1"/>
-    <row r="397" ht="15.75" customHeight="1" s="1"/>
-    <row r="398" ht="15.75" customHeight="1" s="1"/>
-    <row r="399" ht="15.75" customHeight="1" s="1"/>
-    <row r="400" ht="15.75" customHeight="1" s="1"/>
-    <row r="401" ht="15.75" customHeight="1" s="1"/>
-    <row r="402" ht="15.75" customHeight="1" s="1"/>
-    <row r="403" ht="15.75" customHeight="1" s="1"/>
-    <row r="404" ht="15.75" customHeight="1" s="1"/>
-    <row r="405" ht="15.75" customHeight="1" s="1"/>
-    <row r="406" ht="15.75" customHeight="1" s="1"/>
-    <row r="407" ht="15.75" customHeight="1" s="1"/>
-    <row r="408" ht="15.75" customHeight="1" s="1"/>
-    <row r="409" ht="15.75" customHeight="1" s="1"/>
-    <row r="410" ht="15.75" customHeight="1" s="1"/>
-    <row r="411" ht="15.75" customHeight="1" s="1"/>
-    <row r="412" ht="15.75" customHeight="1" s="1"/>
-    <row r="413" ht="15.75" customHeight="1" s="1"/>
-    <row r="414" ht="15.75" customHeight="1" s="1"/>
-    <row r="415" ht="15.75" customHeight="1" s="1"/>
-    <row r="416" ht="15.75" customHeight="1" s="1"/>
-    <row r="417" ht="15.75" customHeight="1" s="1"/>
-    <row r="418" ht="15.75" customHeight="1" s="1"/>
-    <row r="419" ht="15.75" customHeight="1" s="1"/>
-    <row r="420" ht="15.75" customHeight="1" s="1"/>
-    <row r="421" ht="15.75" customHeight="1" s="1"/>
-    <row r="422" ht="15.75" customHeight="1" s="1"/>
-    <row r="423" ht="15.75" customHeight="1" s="1"/>
-    <row r="424" ht="15.75" customHeight="1" s="1"/>
-    <row r="425" ht="15.75" customHeight="1" s="1"/>
-    <row r="426" ht="15.75" customHeight="1" s="1"/>
-    <row r="427" ht="15.75" customHeight="1" s="1"/>
-    <row r="428" ht="15.75" customHeight="1" s="1"/>
-    <row r="429" ht="15.75" customHeight="1" s="1"/>
-    <row r="430" ht="15.75" customHeight="1" s="1"/>
-    <row r="431" ht="15.75" customHeight="1" s="1"/>
-    <row r="432" ht="15.75" customHeight="1" s="1"/>
-    <row r="433" ht="15.75" customHeight="1" s="1"/>
-    <row r="434" ht="15.75" customHeight="1" s="1"/>
-    <row r="435" ht="15.75" customHeight="1" s="1"/>
-    <row r="436" ht="15.75" customHeight="1" s="1"/>
-    <row r="437" ht="15.75" customHeight="1" s="1"/>
-    <row r="438" ht="15.75" customHeight="1" s="1"/>
-    <row r="439" ht="15.75" customHeight="1" s="1"/>
-    <row r="440" ht="15.75" customHeight="1" s="1"/>
-    <row r="441" ht="15.75" customHeight="1" s="1"/>
-    <row r="442" ht="15.75" customHeight="1" s="1"/>
-    <row r="443" ht="15.75" customHeight="1" s="1"/>
-    <row r="444" ht="15.75" customHeight="1" s="1"/>
-    <row r="445" ht="15.75" customHeight="1" s="1"/>
-    <row r="446" ht="15.75" customHeight="1" s="1"/>
-    <row r="447" ht="15.75" customHeight="1" s="1"/>
-    <row r="448" ht="15.75" customHeight="1" s="1"/>
-    <row r="449" ht="15.75" customHeight="1" s="1"/>
-    <row r="450" ht="15.75" customHeight="1" s="1"/>
-    <row r="451" ht="15.75" customHeight="1" s="1"/>
-    <row r="452" ht="15.75" customHeight="1" s="1"/>
-    <row r="453" ht="15.75" customHeight="1" s="1"/>
-    <row r="454" ht="15.75" customHeight="1" s="1"/>
-    <row r="455" ht="15.75" customHeight="1" s="1"/>
-    <row r="456" ht="15.75" customHeight="1" s="1"/>
-    <row r="457" ht="15.75" customHeight="1" s="1"/>
-    <row r="458" ht="15.75" customHeight="1" s="1"/>
-    <row r="459" ht="15.75" customHeight="1" s="1"/>
-    <row r="460" ht="15.75" customHeight="1" s="1"/>
-    <row r="461" ht="15.75" customHeight="1" s="1"/>
-    <row r="462" ht="15.75" customHeight="1" s="1"/>
-    <row r="463" ht="15.75" customHeight="1" s="1"/>
-    <row r="464" ht="15.75" customHeight="1" s="1"/>
-    <row r="465" ht="15.75" customHeight="1" s="1"/>
-    <row r="466" ht="15.75" customHeight="1" s="1"/>
-    <row r="467" ht="15.75" customHeight="1" s="1"/>
-    <row r="468" ht="15.75" customHeight="1" s="1"/>
-    <row r="469" ht="15.75" customHeight="1" s="1"/>
-    <row r="470" ht="15.75" customHeight="1" s="1"/>
-    <row r="471" ht="15.75" customHeight="1" s="1"/>
-    <row r="472" ht="15.75" customHeight="1" s="1"/>
-    <row r="473" ht="15.75" customHeight="1" s="1"/>
-    <row r="474" ht="15.75" customHeight="1" s="1"/>
-    <row r="475" ht="15.75" customHeight="1" s="1"/>
-    <row r="476" ht="15.75" customHeight="1" s="1"/>
-    <row r="477" ht="15.75" customHeight="1" s="1"/>
-    <row r="478" ht="15.75" customHeight="1" s="1"/>
-    <row r="479" ht="15.75" customHeight="1" s="1"/>
-    <row r="480" ht="15.75" customHeight="1" s="1"/>
-    <row r="481" ht="15.75" customHeight="1" s="1"/>
-    <row r="482" ht="15.75" customHeight="1" s="1"/>
-    <row r="483" ht="15.75" customHeight="1" s="1"/>
-    <row r="484" ht="15.75" customHeight="1" s="1"/>
-    <row r="485" ht="15.75" customHeight="1" s="1"/>
-    <row r="486" ht="15.75" customHeight="1" s="1"/>
-    <row r="487" ht="15.75" customHeight="1" s="1"/>
-    <row r="488" ht="15.75" customHeight="1" s="1"/>
-    <row r="489" ht="15.75" customHeight="1" s="1"/>
-    <row r="490" ht="15.75" customHeight="1" s="1"/>
-    <row r="491" ht="15.75" customHeight="1" s="1"/>
-    <row r="492" ht="15.75" customHeight="1" s="1"/>
-    <row r="493" ht="15.75" customHeight="1" s="1"/>
-    <row r="494" ht="15.75" customHeight="1" s="1"/>
-    <row r="495" ht="15.75" customHeight="1" s="1"/>
-    <row r="496" ht="15.75" customHeight="1" s="1"/>
-    <row r="497" ht="15.75" customHeight="1" s="1"/>
-    <row r="498" ht="15.75" customHeight="1" s="1"/>
-    <row r="499" ht="15.75" customHeight="1" s="1"/>
-    <row r="500" ht="15.75" customHeight="1" s="1"/>
-    <row r="501" ht="15.75" customHeight="1" s="1"/>
-    <row r="502" ht="15.75" customHeight="1" s="1"/>
-    <row r="503" ht="15.75" customHeight="1" s="1"/>
-    <row r="504" ht="15.75" customHeight="1" s="1"/>
-    <row r="505" ht="15.75" customHeight="1" s="1"/>
-    <row r="506" ht="15.75" customHeight="1" s="1"/>
-    <row r="507" ht="15.75" customHeight="1" s="1"/>
-    <row r="508" ht="15.75" customHeight="1" s="1"/>
-    <row r="509" ht="15.75" customHeight="1" s="1"/>
-    <row r="510" ht="15.75" customHeight="1" s="1"/>
-    <row r="511" ht="15.75" customHeight="1" s="1"/>
-    <row r="512" ht="15.75" customHeight="1" s="1"/>
-    <row r="513" ht="15.75" customHeight="1" s="1"/>
-    <row r="514" ht="15.75" customHeight="1" s="1"/>
-    <row r="515" ht="15.75" customHeight="1" s="1"/>
-    <row r="516" ht="15.75" customHeight="1" s="1"/>
-    <row r="517" ht="15.75" customHeight="1" s="1"/>
-    <row r="518" ht="15.75" customHeight="1" s="1"/>
-    <row r="519" ht="15.75" customHeight="1" s="1"/>
-    <row r="520" ht="15.75" customHeight="1" s="1"/>
-    <row r="521" ht="15.75" customHeight="1" s="1"/>
-    <row r="522" ht="15.75" customHeight="1" s="1"/>
-    <row r="523" ht="15.75" customHeight="1" s="1"/>
-    <row r="524" ht="15.75" customHeight="1" s="1"/>
-    <row r="525" ht="15.75" customHeight="1" s="1"/>
-    <row r="526" ht="15.75" customHeight="1" s="1"/>
-    <row r="527" ht="15.75" customHeight="1" s="1"/>
-    <row r="528" ht="15.75" customHeight="1" s="1"/>
-    <row r="529" ht="15.75" customHeight="1" s="1"/>
-    <row r="530" ht="15.75" customHeight="1" s="1"/>
-    <row r="531" ht="15.75" customHeight="1" s="1"/>
-    <row r="532" ht="15.75" customHeight="1" s="1"/>
-    <row r="533" ht="15.75" customHeight="1" s="1"/>
-    <row r="534" ht="15.75" customHeight="1" s="1"/>
-    <row r="535" ht="15.75" customHeight="1" s="1"/>
-    <row r="536" ht="15.75" customHeight="1" s="1"/>
-    <row r="537" ht="15.75" customHeight="1" s="1"/>
-    <row r="538" ht="15.75" customHeight="1" s="1"/>
-    <row r="539" ht="15.75" customHeight="1" s="1"/>
-    <row r="540" ht="15.75" customHeight="1" s="1"/>
-    <row r="541" ht="15.75" customHeight="1" s="1"/>
-    <row r="542" ht="15.75" customHeight="1" s="1"/>
-    <row r="543" ht="15.75" customHeight="1" s="1"/>
-    <row r="544" ht="15.75" customHeight="1" s="1"/>
-    <row r="545" ht="15.75" customHeight="1" s="1"/>
-    <row r="546" ht="15.75" customHeight="1" s="1"/>
-    <row r="547" ht="15.75" customHeight="1" s="1"/>
-    <row r="548" ht="15.75" customHeight="1" s="1"/>
-    <row r="549" ht="15.75" customHeight="1" s="1"/>
-    <row r="550" ht="15.75" customHeight="1" s="1"/>
-    <row r="551" ht="15.75" customHeight="1" s="1"/>
-    <row r="552" ht="15.75" customHeight="1" s="1"/>
-    <row r="553" ht="15.75" customHeight="1" s="1"/>
-    <row r="554" ht="15.75" customHeight="1" s="1"/>
-    <row r="555" ht="15.75" customHeight="1" s="1"/>
-    <row r="556" ht="15.75" customHeight="1" s="1"/>
-    <row r="557" ht="15.75" customHeight="1" s="1"/>
-    <row r="558" ht="15.75" customHeight="1" s="1"/>
-    <row r="559" ht="15.75" customHeight="1" s="1"/>
-    <row r="560" ht="15.75" customHeight="1" s="1"/>
-    <row r="561" ht="15.75" customHeight="1" s="1"/>
-    <row r="562" ht="15.75" customHeight="1" s="1"/>
-    <row r="563" ht="15.75" customHeight="1" s="1"/>
-    <row r="564" ht="15.75" customHeight="1" s="1"/>
-    <row r="565" ht="15.75" customHeight="1" s="1"/>
-    <row r="566" ht="15.75" customHeight="1" s="1"/>
-    <row r="567" ht="15.75" customHeight="1" s="1"/>
-    <row r="568" ht="15.75" customHeight="1" s="1"/>
-    <row r="569" ht="15.75" customHeight="1" s="1"/>
-    <row r="570" ht="15.75" customHeight="1" s="1"/>
-    <row r="571" ht="15.75" customHeight="1" s="1"/>
-    <row r="572" ht="15.75" customHeight="1" s="1"/>
-    <row r="573" ht="15.75" customHeight="1" s="1"/>
-    <row r="574" ht="15.75" customHeight="1" s="1"/>
-    <row r="575" ht="15.75" customHeight="1" s="1"/>
-    <row r="576" ht="15.75" customHeight="1" s="1"/>
-    <row r="577" ht="15.75" customHeight="1" s="1"/>
-    <row r="578" ht="15.75" customHeight="1" s="1"/>
-    <row r="579" ht="15.75" customHeight="1" s="1"/>
-    <row r="580" ht="15.75" customHeight="1" s="1"/>
-    <row r="581" ht="15.75" customHeight="1" s="1"/>
-    <row r="582" ht="15.75" customHeight="1" s="1"/>
-    <row r="583" ht="15.75" customHeight="1" s="1"/>
-    <row r="584" ht="15.75" customHeight="1" s="1"/>
-    <row r="585" ht="15.75" customHeight="1" s="1"/>
-    <row r="586" ht="15.75" customHeight="1" s="1"/>
-    <row r="587" ht="15.75" customHeight="1" s="1"/>
-    <row r="588" ht="15.75" customHeight="1" s="1"/>
-    <row r="589" ht="15.75" customHeight="1" s="1"/>
-    <row r="590" ht="15.75" customHeight="1" s="1"/>
-    <row r="591" ht="15.75" customHeight="1" s="1"/>
-    <row r="592" ht="15.75" customHeight="1" s="1"/>
-    <row r="593" ht="15.75" customHeight="1" s="1"/>
-    <row r="594" ht="15.75" customHeight="1" s="1"/>
-    <row r="595" ht="15.75" customHeight="1" s="1"/>
-    <row r="596" ht="15.75" customHeight="1" s="1"/>
-    <row r="597" ht="15.75" customHeight="1" s="1"/>
-    <row r="598" ht="15.75" customHeight="1" s="1"/>
-    <row r="599" ht="15.75" customHeight="1" s="1"/>
-    <row r="600" ht="15.75" customHeight="1" s="1"/>
-    <row r="601" ht="15.75" customHeight="1" s="1"/>
-    <row r="602" ht="15.75" customHeight="1" s="1"/>
-    <row r="603" ht="15.75" customHeight="1" s="1"/>
-    <row r="604" ht="15.75" customHeight="1" s="1"/>
-    <row r="605" ht="15.75" customHeight="1" s="1"/>
-    <row r="606" ht="15.75" customHeight="1" s="1"/>
-    <row r="607" ht="15.75" customHeight="1" s="1"/>
-    <row r="608" ht="15.75" customHeight="1" s="1"/>
-    <row r="609" ht="15.75" customHeight="1" s="1"/>
-    <row r="610" ht="15.75" customHeight="1" s="1"/>
-    <row r="611" ht="15.75" customHeight="1" s="1"/>
-    <row r="612" ht="15.75" customHeight="1" s="1"/>
-    <row r="613" ht="15.75" customHeight="1" s="1"/>
-    <row r="614" ht="15.75" customHeight="1" s="1"/>
-    <row r="615" ht="15.75" customHeight="1" s="1"/>
-    <row r="616" ht="15.75" customHeight="1" s="1"/>
-    <row r="617" ht="15.75" customHeight="1" s="1"/>
-    <row r="618" ht="15.75" customHeight="1" s="1"/>
-    <row r="619" ht="15.75" customHeight="1" s="1"/>
-    <row r="620" ht="15.75" customHeight="1" s="1"/>
-    <row r="621" ht="15.75" customHeight="1" s="1"/>
-    <row r="622" ht="15.75" customHeight="1" s="1"/>
-    <row r="623" ht="15.75" customHeight="1" s="1"/>
-    <row r="624" ht="15.75" customHeight="1" s="1"/>
-    <row r="625" ht="15.75" customHeight="1" s="1"/>
-    <row r="626" ht="15.75" customHeight="1" s="1"/>
-    <row r="627" ht="15.75" customHeight="1" s="1"/>
-    <row r="628" ht="15.75" customHeight="1" s="1"/>
-    <row r="629" ht="15.75" customHeight="1" s="1"/>
-    <row r="630" ht="15.75" customHeight="1" s="1"/>
-    <row r="631" ht="15.75" customHeight="1" s="1"/>
-    <row r="632" ht="15.75" customHeight="1" s="1"/>
-    <row r="633" ht="15.75" customHeight="1" s="1"/>
-    <row r="634" ht="15.75" customHeight="1" s="1"/>
-    <row r="635" ht="15.75" customHeight="1" s="1"/>
-    <row r="636" ht="15.75" customHeight="1" s="1"/>
-    <row r="637" ht="15.75" customHeight="1" s="1"/>
-    <row r="638" ht="15.75" customHeight="1" s="1"/>
-    <row r="639" ht="15.75" customHeight="1" s="1"/>
-    <row r="640" ht="15.75" customHeight="1" s="1"/>
-    <row r="641" ht="15.75" customHeight="1" s="1"/>
-    <row r="642" ht="15.75" customHeight="1" s="1"/>
-    <row r="643" ht="15.75" customHeight="1" s="1"/>
-    <row r="644" ht="15.75" customHeight="1" s="1"/>
-    <row r="645" ht="15.75" customHeight="1" s="1"/>
-    <row r="646" ht="15.75" customHeight="1" s="1"/>
-    <row r="647" ht="15.75" customHeight="1" s="1"/>
-    <row r="648" ht="15.75" customHeight="1" s="1"/>
-    <row r="649" ht="15.75" customHeight="1" s="1"/>
-    <row r="650" ht="15.75" customHeight="1" s="1"/>
-    <row r="651" ht="15.75" customHeight="1" s="1"/>
-    <row r="652" ht="15.75" customHeight="1" s="1"/>
-    <row r="653" ht="15.75" customHeight="1" s="1"/>
-    <row r="654" ht="15.75" customHeight="1" s="1"/>
-    <row r="655" ht="15.75" customHeight="1" s="1"/>
-    <row r="656" ht="15.75" customHeight="1" s="1"/>
-    <row r="657" ht="15.75" customHeight="1" s="1"/>
-    <row r="658" ht="15.75" customHeight="1" s="1"/>
-    <row r="659" ht="15.75" customHeight="1" s="1"/>
-    <row r="660" ht="15.75" customHeight="1" s="1"/>
-    <row r="661" ht="15.75" customHeight="1" s="1"/>
-    <row r="662" ht="15.75" customHeight="1" s="1"/>
-    <row r="663" ht="15.75" customHeight="1" s="1"/>
-    <row r="664" ht="15.75" customHeight="1" s="1"/>
-    <row r="665" ht="15.75" customHeight="1" s="1"/>
-    <row r="666" ht="15.75" customHeight="1" s="1"/>
-    <row r="667" ht="15.75" customHeight="1" s="1"/>
-    <row r="668" ht="15.75" customHeight="1" s="1"/>
-    <row r="669" ht="15.75" customHeight="1" s="1"/>
-    <row r="670" ht="15.75" customHeight="1" s="1"/>
-    <row r="671" ht="15.75" customHeight="1" s="1"/>
-    <row r="672" ht="15.75" customHeight="1" s="1"/>
-    <row r="673" ht="15.75" customHeight="1" s="1"/>
-    <row r="674" ht="15.75" customHeight="1" s="1"/>
-    <row r="675" ht="15.75" customHeight="1" s="1"/>
-    <row r="676" ht="15.75" customHeight="1" s="1"/>
-    <row r="677" ht="15.75" customHeight="1" s="1"/>
-    <row r="678" ht="15.75" customHeight="1" s="1"/>
-    <row r="679" ht="15.75" customHeight="1" s="1"/>
-    <row r="680" ht="15.75" customHeight="1" s="1"/>
-    <row r="681" ht="15.75" customHeight="1" s="1"/>
-    <row r="682" ht="15.75" customHeight="1" s="1"/>
-    <row r="683" ht="15.75" customHeight="1" s="1"/>
-    <row r="684" ht="15.75" customHeight="1" s="1"/>
-    <row r="685" ht="15.75" customHeight="1" s="1"/>
-    <row r="686" ht="15.75" customHeight="1" s="1"/>
-    <row r="687" ht="15.75" customHeight="1" s="1"/>
-    <row r="688" ht="15.75" customHeight="1" s="1"/>
-    <row r="689" ht="15.75" customHeight="1" s="1"/>
-    <row r="690" ht="15.75" customHeight="1" s="1"/>
-    <row r="691" ht="15.75" customHeight="1" s="1"/>
-    <row r="692" ht="15.75" customHeight="1" s="1"/>
-    <row r="693" ht="15.75" customHeight="1" s="1"/>
-    <row r="694" ht="15.75" customHeight="1" s="1"/>
-    <row r="695" ht="15.75" customHeight="1" s="1"/>
-    <row r="696" ht="15.75" customHeight="1" s="1"/>
-    <row r="697" ht="15.75" customHeight="1" s="1"/>
-    <row r="698" ht="15.75" customHeight="1" s="1"/>
-    <row r="699" ht="15.75" customHeight="1" s="1"/>
-    <row r="700" ht="15.75" customHeight="1" s="1"/>
-    <row r="701" ht="15.75" customHeight="1" s="1"/>
-    <row r="702" ht="15.75" customHeight="1" s="1"/>
-    <row r="703" ht="15.75" customHeight="1" s="1"/>
-    <row r="704" ht="15.75" customHeight="1" s="1"/>
-    <row r="705" ht="15.75" customHeight="1" s="1"/>
-    <row r="706" ht="15.75" customHeight="1" s="1"/>
-    <row r="707" ht="15.75" customHeight="1" s="1"/>
-    <row r="708" ht="15.75" customHeight="1" s="1"/>
-    <row r="709" ht="15.75" customHeight="1" s="1"/>
-    <row r="710" ht="15.75" customHeight="1" s="1"/>
-    <row r="711" ht="15.75" customHeight="1" s="1"/>
-    <row r="712" ht="15.75" customHeight="1" s="1"/>
-    <row r="713" ht="15.75" customHeight="1" s="1"/>
-    <row r="714" ht="15.75" customHeight="1" s="1"/>
-    <row r="715" ht="15.75" customHeight="1" s="1"/>
-    <row r="716" ht="15.75" customHeight="1" s="1"/>
-    <row r="717" ht="15.75" customHeight="1" s="1"/>
-    <row r="718" ht="15.75" customHeight="1" s="1"/>
-    <row r="719" ht="15.75" customHeight="1" s="1"/>
-    <row r="720" ht="15.75" customHeight="1" s="1"/>
-    <row r="721" ht="15.75" customHeight="1" s="1"/>
-    <row r="722" ht="15.75" customHeight="1" s="1"/>
-    <row r="723" ht="15.75" customHeight="1" s="1"/>
-    <row r="724" ht="15.75" customHeight="1" s="1"/>
-    <row r="725" ht="15.75" customHeight="1" s="1"/>
-    <row r="726" ht="15.75" customHeight="1" s="1"/>
-    <row r="727" ht="15.75" customHeight="1" s="1"/>
-    <row r="728" ht="15.75" customHeight="1" s="1"/>
-    <row r="729" ht="15.75" customHeight="1" s="1"/>
-    <row r="730" ht="15.75" customHeight="1" s="1"/>
-    <row r="731" ht="15.75" customHeight="1" s="1"/>
-    <row r="732" ht="15.75" customHeight="1" s="1"/>
-    <row r="733" ht="15.75" customHeight="1" s="1"/>
-    <row r="734" ht="15.75" customHeight="1" s="1"/>
-    <row r="735" ht="15.75" customHeight="1" s="1"/>
-    <row r="736" ht="15.75" customHeight="1" s="1"/>
-    <row r="737" ht="15.75" customHeight="1" s="1"/>
-    <row r="738" ht="15.75" customHeight="1" s="1"/>
-    <row r="739" ht="15.75" customHeight="1" s="1"/>
-    <row r="740" ht="15.75" customHeight="1" s="1"/>
-    <row r="741" ht="15.75" customHeight="1" s="1"/>
-    <row r="742" ht="15.75" customHeight="1" s="1"/>
-    <row r="743" ht="15.75" customHeight="1" s="1"/>
-    <row r="744" ht="15.75" customHeight="1" s="1"/>
-    <row r="745" ht="15.75" customHeight="1" s="1"/>
-    <row r="746" ht="15.75" customHeight="1" s="1"/>
-    <row r="747" ht="15.75" customHeight="1" s="1"/>
-    <row r="748" ht="15.75" customHeight="1" s="1"/>
-    <row r="749" ht="15.75" customHeight="1" s="1"/>
-    <row r="750" ht="15.75" customHeight="1" s="1"/>
-    <row r="751" ht="15.75" customHeight="1" s="1"/>
-    <row r="752" ht="15.75" customHeight="1" s="1"/>
-    <row r="753" ht="15.75" customHeight="1" s="1"/>
-    <row r="754" ht="15.75" customHeight="1" s="1"/>
-    <row r="755" ht="15.75" customHeight="1" s="1"/>
-    <row r="756" ht="15.75" customHeight="1" s="1"/>
-    <row r="757" ht="15.75" customHeight="1" s="1"/>
-    <row r="758" ht="15.75" customHeight="1" s="1"/>
-    <row r="759" ht="15.75" customHeight="1" s="1"/>
-    <row r="760" ht="15.75" customHeight="1" s="1"/>
-    <row r="761" ht="15.75" customHeight="1" s="1"/>
-    <row r="762" ht="15.75" customHeight="1" s="1"/>
-    <row r="763" ht="15.75" customHeight="1" s="1"/>
-    <row r="764" ht="15.75" customHeight="1" s="1"/>
-    <row r="765" ht="15.75" customHeight="1" s="1"/>
-    <row r="766" ht="15.75" customHeight="1" s="1"/>
-    <row r="767" ht="15.75" customHeight="1" s="1"/>
-    <row r="768" ht="15.75" customHeight="1" s="1"/>
-    <row r="769" ht="15.75" customHeight="1" s="1"/>
-    <row r="770" ht="15.75" customHeight="1" s="1"/>
-    <row r="771" ht="15.75" customHeight="1" s="1"/>
-    <row r="772" ht="15.75" customHeight="1" s="1"/>
-    <row r="773" ht="15.75" customHeight="1" s="1"/>
-    <row r="774" ht="15.75" customHeight="1" s="1"/>
-    <row r="775" ht="15.75" customHeight="1" s="1"/>
-    <row r="776" ht="15.75" customHeight="1" s="1"/>
-    <row r="777" ht="15.75" customHeight="1" s="1"/>
-    <row r="778" ht="15.75" customHeight="1" s="1"/>
-    <row r="779" ht="15.75" customHeight="1" s="1"/>
-    <row r="780" ht="15.75" customHeight="1" s="1"/>
-    <row r="781" ht="15.75" customHeight="1" s="1"/>
-    <row r="782" ht="15.75" customHeight="1" s="1"/>
-    <row r="783" ht="15.75" customHeight="1" s="1"/>
-    <row r="784" ht="15.75" customHeight="1" s="1"/>
-    <row r="785" ht="15.75" customHeight="1" s="1"/>
-    <row r="786" ht="15.75" customHeight="1" s="1"/>
-    <row r="787" ht="15.75" customHeight="1" s="1"/>
-    <row r="788" ht="15.75" customHeight="1" s="1"/>
-    <row r="789" ht="15.75" customHeight="1" s="1"/>
-    <row r="790" ht="15.75" customHeight="1" s="1"/>
-    <row r="791" ht="15.75" customHeight="1" s="1"/>
-    <row r="792" ht="15.75" customHeight="1" s="1"/>
-    <row r="793" ht="15.75" customHeight="1" s="1"/>
-    <row r="794" ht="15.75" customHeight="1" s="1"/>
-    <row r="795" ht="15.75" customHeight="1" s="1"/>
-    <row r="796" ht="15.75" customHeight="1" s="1"/>
-    <row r="797" ht="15.75" customHeight="1" s="1"/>
-    <row r="798" ht="15.75" customHeight="1" s="1"/>
-    <row r="799" ht="15.75" customHeight="1" s="1"/>
-    <row r="800" ht="15.75" customHeight="1" s="1"/>
-    <row r="801" ht="15.75" customHeight="1" s="1"/>
-    <row r="802" ht="15.75" customHeight="1" s="1"/>
-    <row r="803" ht="15.75" customHeight="1" s="1"/>
-    <row r="804" ht="15.75" customHeight="1" s="1"/>
-    <row r="805" ht="15.75" customHeight="1" s="1"/>
-    <row r="806" ht="15.75" customHeight="1" s="1"/>
-    <row r="807" ht="15.75" customHeight="1" s="1"/>
-    <row r="808" ht="15.75" customHeight="1" s="1"/>
-    <row r="809" ht="15.75" customHeight="1" s="1"/>
-    <row r="810" ht="15.75" customHeight="1" s="1"/>
-    <row r="811" ht="15.75" customHeight="1" s="1"/>
-    <row r="812" ht="15.75" customHeight="1" s="1"/>
-    <row r="813" ht="15.75" customHeight="1" s="1"/>
-    <row r="814" ht="15.75" customHeight="1" s="1"/>
-    <row r="815" ht="15.75" customHeight="1" s="1"/>
-    <row r="816" ht="15.75" customHeight="1" s="1"/>
-    <row r="817" ht="15.75" customHeight="1" s="1"/>
-    <row r="818" ht="15.75" customHeight="1" s="1"/>
-    <row r="819" ht="15.75" customHeight="1" s="1"/>
-    <row r="820" ht="15.75" customHeight="1" s="1"/>
-    <row r="821" ht="15.75" customHeight="1" s="1"/>
-    <row r="822" ht="15.75" customHeight="1" s="1"/>
-    <row r="823" ht="15.75" customHeight="1" s="1"/>
-    <row r="824" ht="15.75" customHeight="1" s="1"/>
-    <row r="825" ht="15.75" customHeight="1" s="1"/>
-    <row r="826" ht="15.75" customHeight="1" s="1"/>
-    <row r="827" ht="15.75" customHeight="1" s="1"/>
-    <row r="828" ht="15.75" customHeight="1" s="1"/>
-    <row r="829" ht="15.75" customHeight="1" s="1"/>
-    <row r="830" ht="15.75" customHeight="1" s="1"/>
-    <row r="831" ht="15.75" customHeight="1" s="1"/>
-    <row r="832" ht="15.75" customHeight="1" s="1"/>
-    <row r="833" ht="15.75" customHeight="1" s="1"/>
-    <row r="834" ht="15.75" customHeight="1" s="1"/>
-    <row r="835" ht="15.75" customHeight="1" s="1"/>
-    <row r="836" ht="15.75" customHeight="1" s="1"/>
-    <row r="837" ht="15.75" customHeight="1" s="1"/>
-    <row r="838" ht="15.75" customHeight="1" s="1"/>
-    <row r="839" ht="15.75" customHeight="1" s="1"/>
-    <row r="840" ht="15.75" customHeight="1" s="1"/>
-    <row r="841" ht="15.75" customHeight="1" s="1"/>
-    <row r="842" ht="15.75" customHeight="1" s="1"/>
-    <row r="843" ht="15.75" customHeight="1" s="1"/>
-    <row r="844" ht="15.75" customHeight="1" s="1"/>
-    <row r="845" ht="15.75" customHeight="1" s="1"/>
-    <row r="846" ht="15.75" customHeight="1" s="1"/>
-    <row r="847" ht="15.75" customHeight="1" s="1"/>
-    <row r="848" ht="15.75" customHeight="1" s="1"/>
-    <row r="849" ht="15.75" customHeight="1" s="1"/>
-    <row r="850" ht="15.75" customHeight="1" s="1"/>
-    <row r="851" ht="15.75" customHeight="1" s="1"/>
-    <row r="852" ht="15.75" customHeight="1" s="1"/>
-    <row r="853" ht="15.75" customHeight="1" s="1"/>
-    <row r="854" ht="15.75" customHeight="1" s="1"/>
-    <row r="855" ht="15.75" customHeight="1" s="1"/>
-    <row r="856" ht="15.75" customHeight="1" s="1"/>
-    <row r="857" ht="15.75" customHeight="1" s="1"/>
-    <row r="858" ht="15.75" customHeight="1" s="1"/>
-    <row r="859" ht="15.75" customHeight="1" s="1"/>
-    <row r="860" ht="15.75" customHeight="1" s="1"/>
-    <row r="861" ht="15.75" customHeight="1" s="1"/>
-    <row r="862" ht="15.75" customHeight="1" s="1"/>
-    <row r="863" ht="15.75" customHeight="1" s="1"/>
-    <row r="864" ht="15.75" customHeight="1" s="1"/>
-    <row r="865" ht="15.75" customHeight="1" s="1"/>
-    <row r="866" ht="15.75" customHeight="1" s="1"/>
-    <row r="867" ht="15.75" customHeight="1" s="1"/>
-    <row r="868" ht="15.75" customHeight="1" s="1"/>
-    <row r="869" ht="15.75" customHeight="1" s="1"/>
-    <row r="870" ht="15.75" customHeight="1" s="1"/>
-    <row r="871" ht="15.75" customHeight="1" s="1"/>
-    <row r="872" ht="15.75" customHeight="1" s="1"/>
-    <row r="873" ht="15.75" customHeight="1" s="1"/>
-    <row r="874" ht="15.75" customHeight="1" s="1"/>
-    <row r="875" ht="15.75" customHeight="1" s="1"/>
-    <row r="876" ht="15.75" customHeight="1" s="1"/>
-    <row r="877" ht="15.75" customHeight="1" s="1"/>
-    <row r="878" ht="15.75" customHeight="1" s="1"/>
-    <row r="879" ht="15.75" customHeight="1" s="1"/>
-    <row r="880" ht="15.75" customHeight="1" s="1"/>
-    <row r="881" ht="15.75" customHeight="1" s="1"/>
-    <row r="882" ht="15.75" customHeight="1" s="1"/>
-    <row r="883" ht="15.75" customHeight="1" s="1"/>
-    <row r="884" ht="15.75" customHeight="1" s="1"/>
-    <row r="885" ht="15.75" customHeight="1" s="1"/>
-    <row r="886" ht="15.75" customHeight="1" s="1"/>
-    <row r="887" ht="15.75" customHeight="1" s="1"/>
-    <row r="888" ht="15.75" customHeight="1" s="1"/>
-    <row r="889" ht="15.75" customHeight="1" s="1"/>
-    <row r="890" ht="15.75" customHeight="1" s="1"/>
-    <row r="891" ht="15.75" customHeight="1" s="1"/>
-    <row r="892" ht="15.75" customHeight="1" s="1"/>
-    <row r="893" ht="15.75" customHeight="1" s="1"/>
-    <row r="894" ht="15.75" customHeight="1" s="1"/>
-    <row r="895" ht="15.75" customHeight="1" s="1"/>
-    <row r="896" ht="15.75" customHeight="1" s="1"/>
-    <row r="897" ht="15.75" customHeight="1" s="1"/>
-    <row r="898" ht="15.75" customHeight="1" s="1"/>
-    <row r="899" ht="15.75" customHeight="1" s="1"/>
-    <row r="900" ht="15.75" customHeight="1" s="1"/>
-    <row r="901" ht="15.75" customHeight="1" s="1"/>
-    <row r="902" ht="15.75" customHeight="1" s="1"/>
-    <row r="903" ht="15.75" customHeight="1" s="1"/>
-    <row r="904" ht="15.75" customHeight="1" s="1"/>
-    <row r="905" ht="15.75" customHeight="1" s="1"/>
-    <row r="906" ht="15.75" customHeight="1" s="1"/>
-    <row r="907" ht="15.75" customHeight="1" s="1"/>
-    <row r="908" ht="15.75" customHeight="1" s="1"/>
-    <row r="909" ht="15.75" customHeight="1" s="1"/>
-    <row r="910" ht="15.75" customHeight="1" s="1"/>
-    <row r="911" ht="15.75" customHeight="1" s="1"/>
-    <row r="912" ht="15.75" customHeight="1" s="1"/>
-    <row r="913" ht="15.75" customHeight="1" s="1"/>
-    <row r="914" ht="15.75" customHeight="1" s="1"/>
-    <row r="915" ht="15.75" customHeight="1" s="1"/>
-    <row r="916" ht="15.75" customHeight="1" s="1"/>
-    <row r="917" ht="15.75" customHeight="1" s="1"/>
-    <row r="918" ht="15.75" customHeight="1" s="1"/>
-    <row r="919" ht="15.75" customHeight="1" s="1"/>
-    <row r="920" ht="15.75" customHeight="1" s="1"/>
-    <row r="921" ht="15.75" customHeight="1" s="1"/>
-    <row r="922" ht="15.75" customHeight="1" s="1"/>
-    <row r="923" ht="15.75" customHeight="1" s="1"/>
-    <row r="924" ht="15.75" customHeight="1" s="1"/>
-    <row r="925" ht="15.75" customHeight="1" s="1"/>
-    <row r="926" ht="15.75" customHeight="1" s="1"/>
-    <row r="927" ht="15.75" customHeight="1" s="1"/>
-    <row r="928" ht="15.75" customHeight="1" s="1"/>
-    <row r="929" ht="15.75" customHeight="1" s="1"/>
-    <row r="930" ht="15.75" customHeight="1" s="1"/>
-    <row r="931" ht="15.75" customHeight="1" s="1"/>
-    <row r="932" ht="15.75" customHeight="1" s="1"/>
-    <row r="933" ht="15.75" customHeight="1" s="1"/>
-    <row r="934" ht="15.75" customHeight="1" s="1"/>
-    <row r="935" ht="15.75" customHeight="1" s="1"/>
-    <row r="936" ht="15.75" customHeight="1" s="1"/>
-    <row r="937" ht="15.75" customHeight="1" s="1"/>
-    <row r="938" ht="15.75" customHeight="1" s="1"/>
-    <row r="939" ht="15.75" customHeight="1" s="1"/>
-    <row r="940" ht="15.75" customHeight="1" s="1"/>
-    <row r="941" ht="15.75" customHeight="1" s="1"/>
-    <row r="942" ht="15.75" customHeight="1" s="1"/>
-    <row r="943" ht="15.75" customHeight="1" s="1"/>
-    <row r="944" ht="15.75" customHeight="1" s="1"/>
-    <row r="945" ht="15.75" customHeight="1" s="1"/>
-    <row r="946" ht="15.75" customHeight="1" s="1"/>
-    <row r="947" ht="15.75" customHeight="1" s="1"/>
-    <row r="948" ht="15.75" customHeight="1" s="1"/>
-    <row r="949" ht="15.75" customHeight="1" s="1"/>
-    <row r="950" ht="15.75" customHeight="1" s="1"/>
-    <row r="951" ht="15.75" customHeight="1" s="1"/>
-    <row r="952" ht="15.75" customHeight="1" s="1"/>
-    <row r="953" ht="15.75" customHeight="1" s="1"/>
-    <row r="954" ht="15.75" customHeight="1" s="1"/>
-    <row r="955" ht="15.75" customHeight="1" s="1"/>
-    <row r="956" ht="15.75" customHeight="1" s="1"/>
-    <row r="957" ht="15.75" customHeight="1" s="1"/>
-    <row r="958" ht="15.75" customHeight="1" s="1"/>
-    <row r="959" ht="15.75" customHeight="1" s="1"/>
-    <row r="960" ht="15.75" customHeight="1" s="1"/>
-    <row r="961" ht="15.75" customHeight="1" s="1"/>
-    <row r="962" ht="15.75" customHeight="1" s="1"/>
-    <row r="963" ht="15.75" customHeight="1" s="1"/>
-    <row r="964" ht="15.75" customHeight="1" s="1"/>
-    <row r="965" ht="15.75" customHeight="1" s="1"/>
-    <row r="966" ht="15.75" customHeight="1" s="1"/>
-    <row r="967" ht="15.75" customHeight="1" s="1"/>
-    <row r="968" ht="15.75" customHeight="1" s="1"/>
-    <row r="969" ht="15.75" customHeight="1" s="1"/>
-    <row r="970" ht="15.75" customHeight="1" s="1"/>
-    <row r="971" ht="15.75" customHeight="1" s="1"/>
-    <row r="972" ht="15.75" customHeight="1" s="1"/>
-    <row r="973" ht="15.75" customHeight="1" s="1"/>
-    <row r="974" ht="15.75" customHeight="1" s="1"/>
-    <row r="975" ht="15.75" customHeight="1" s="1"/>
-    <row r="976" ht="15.75" customHeight="1" s="1"/>
-    <row r="977" ht="15.75" customHeight="1" s="1"/>
-    <row r="978" ht="15.75" customHeight="1" s="1"/>
-    <row r="979" ht="15.75" customHeight="1" s="1"/>
-    <row r="980" ht="15.75" customHeight="1" s="1"/>
-    <row r="981" ht="15.75" customHeight="1" s="1"/>
-    <row r="982" ht="15.75" customHeight="1" s="1"/>
-    <row r="983" ht="15.75" customHeight="1" s="1"/>
-    <row r="984" ht="15.75" customHeight="1" s="1"/>
-    <row r="985" ht="15.75" customHeight="1" s="1"/>
-    <row r="986" ht="15.75" customHeight="1" s="1"/>
-    <row r="987" ht="15.75" customHeight="1" s="1"/>
-    <row r="988" ht="15.75" customHeight="1" s="1"/>
-    <row r="989" ht="15.75" customHeight="1" s="1"/>
-    <row r="990" ht="15.75" customHeight="1" s="1"/>
-    <row r="991" ht="15.75" customHeight="1" s="1"/>
-    <row r="992" ht="15.75" customHeight="1" s="1"/>
-    <row r="993" ht="15.75" customHeight="1" s="1"/>
-    <row r="994" ht="15.75" customHeight="1" s="1"/>
-    <row r="995" ht="15.75" customHeight="1" s="1"/>
-    <row r="996" ht="15.75" customHeight="1" s="1"/>
-    <row r="997" ht="15.75" customHeight="1" s="1"/>
-    <row r="998" ht="15.75" customHeight="1" s="1"/>
-    <row r="999" ht="15.75" customHeight="1" s="1"/>
-    <row r="1000" ht="15.75" customHeight="1" s="1"/>
-  </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
-  <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" useFirstPageNumber="0" pageOrder="downThenOver" usePrinterDefaults="1" blackAndWhite="0" draft="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
-    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:F11"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
-  <cols>
-    <col width="33" customWidth="1" style="1" min="1" max="1"/>
-    <col width="26" customWidth="1" style="1" min="2" max="2"/>
-    <col width="30" customWidth="1" style="1" min="3" max="3"/>
-    <col width="38" customWidth="1" style="1" min="4" max="4"/>
-    <col width="22" customWidth="1" style="1" min="5" max="5"/>
-    <col width="16" customWidth="1" style="1" min="6" max="6"/>
-    <col width="8.710000000000001" customWidth="1" style="1" min="7" max="26"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="27.75" customHeight="1" s="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>MATRIZ 3 — DIFICULTADES E INCIDENCIAS  ·  GRUPO 2 FIREFOX</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="n"/>
-      <c r="C1" s="3" t="n"/>
-      <c r="D1" s="3" t="n"/>
-      <c r="E1" s="3" t="n"/>
-      <c r="F1" s="4" t="n"/>
-    </row>
-    <row r="2" ht="19.5" customHeight="1" s="1">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Registra incidencias reales, analiza su efecto y define acciones correctivas con responsable y fecha. Una dificultad no debe ocultarse: debe registrarse, analizarse y convertirse en acción concreta.</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="4" t="n"/>
-    </row>
-    <row r="3" ht="4.5" customHeight="1" s="1">
-      <c r="A3" s="6" t="n"/>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="4" t="n"/>
-    </row>
-    <row r="4" ht="24" customHeight="1" s="1">
-      <c r="A4" s="16" t="inlineStr">
-        <is>
-          <t>Finalidad: esta matriz ayuda a registrar incidencias reales, analizar su efecto en el trabajo y definir acciones correctivas con responsable y fecha de revisión.</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="4" t="n"/>
-    </row>
-    <row r="5" ht="27.75" customHeight="1" s="1">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>Dificultad / Incidencia</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>Causa probable</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>Efecto en el avance</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>Acción correctiva</t>
-        </is>
-      </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>Responsable</t>
-        </is>
-      </c>
-      <c r="F5" s="10" t="inlineStr">
-        <is>
-          <t>Fecha revisión</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="99.75" customHeight="1" s="1">
-      <c r="A6" s="21" t="inlineStr">
-        <is>
-          <t>Sin acceso al código fuente, base de datos ni entorno de producción de Boliviana de Aviación (BoA).</t>
-        </is>
-      </c>
-      <c r="B6" s="21" t="inlineStr">
-        <is>
-          <t>BoA es una empresa estatal con restricciones de acceso a sus sistemas internos para equipos externos. No existe convenio de colaboración técnica.</t>
-        </is>
-      </c>
-      <c r="C6" s="21" t="inlineStr">
-        <is>
-          <t>No es posible validar el prototipo con datos reales ni comparar directamente con el comportamiento del sistema en producción. Toda validación es sobre datos simulados.</t>
-        </is>
-      </c>
-      <c r="D6" s="21" t="inlineStr">
-        <is>
-          <t>Desarrollar el prototipo con datos simulados coherentes con el contexto de una aerolínea nacional. Documentar explícitamente como limitación del estudio en todos los informes, matrices y el reporte final.</t>
-        </is>
-      </c>
-      <c r="E6" s="22" t="inlineStr">
-        <is>
-          <t>Todo el equipo</t>
-        </is>
-      </c>
-      <c r="F6" s="23" t="inlineStr">
-        <is>
-          <t>24/09/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="99.75" customHeight="1" s="1">
-      <c r="A7" s="21" t="n"/>
-      <c r="B7" s="21" t="inlineStr">
-        <is>
-          <t>Complejidad del modelado de la BD y configuración del entorno del prototipo no fue estimada correctamente en la planificación inicial.</t>
-        </is>
-      </c>
-      <c r="C7" s="21" t="inlineStr">
-        <is>
-          <t>Retraso en la línea de tiempo del proyecto. Riesgo de efecto cascada que afecte los plazos de los Objetivos 2 y 3.</t>
-        </is>
-      </c>
-      <c r="D7" s="21" t="inlineStr">
-        <is>
-          <t>Iver Pinaya debe reportar el avance real ejecutado y presentar al menos un artefacto parcial (diagrama ER o fragmento de código del bloqueo). Redefinir la fecha meta a 26/09/2026.</t>
-        </is>
-      </c>
-      <c r="E7" s="22" t="inlineStr">
-        <is>
-          <t>Iver Pinaya
-(Líder Backend / DBA)</t>
-        </is>
-      </c>
-      <c r="F7" s="23" t="inlineStr">
-        <is>
-          <t>26/09/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="99.75" customHeight="1" s="1">
-      <c r="A8" s="24" t="inlineStr">
-        <is>
-          <t>Sin datos históricos de tráfico de campañas comerciales reales de BoA (ej. Vuelos Azules).</t>
-        </is>
-      </c>
-      <c r="B8" s="24" t="inlineStr">
-        <is>
-          <t>Información interna y confidencial de la empresa; no se publica en fuentes abiertas ni informes públicos.</t>
-        </is>
-      </c>
-      <c r="C8" s="24" t="inlineStr">
-        <is>
-          <t>Los escenarios de carga para las pruebas de estrés no reflejan valores reales, lo que limita la representatividad del prototipo.</t>
-        </is>
-      </c>
-      <c r="D8" s="24" t="inlineStr">
-        <is>
-          <t>Modelar los escenarios con benchmarks documentados de aerolíneas comparables (LATAM, Avianca, Aeromexico) y citar las fuentes técnicas en el documento del protocolo de pruebas.</t>
-        </is>
-      </c>
-      <c r="E8" s="25" t="inlineStr">
-        <is>
-          <t>Wilson Gonzales
-(Líder QA / Pruebas)</t>
-        </is>
-      </c>
-      <c r="F8" s="12" t="inlineStr">
-        <is>
-          <t>05/11/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="99.75" customHeight="1" s="1">
-      <c r="A9" s="24" t="inlineStr">
-        <is>
-          <t>Sin SLAs ni métricas operativas internas de BoA (latencia, uptime, throughput) como línea base de comparación.</t>
-        </is>
-      </c>
-      <c r="B9" s="24" t="inlineStr">
-        <is>
-          <t>BoA no publica sus métricas operativas de TI. Son información interna no disponible para equipos externos.</t>
-        </is>
-      </c>
-      <c r="C9" s="24" t="inlineStr">
-        <is>
-          <t>Los criterios de éxito del prototipo no pueden compararse directamente con el sistema real; el referente es externo a la empresa.</t>
-        </is>
-      </c>
-      <c r="D9" s="24" t="inlineStr">
-        <is>
-          <t>Adoptar estándares de industria como referencia formal: latencia &lt; 200 ms, error rate &lt; 1% (referencia ITIL/SRE). Citarlos como base técnica en el protocolo y en el informe de resultados.</t>
-        </is>
-      </c>
-      <c r="E9" s="25" t="inlineStr">
-        <is>
-          <t>Thiago Sossa
-(Arquitecto / DevOps)</t>
-        </is>
-      </c>
-      <c r="F9" s="12" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="99.75" customHeight="1" s="1">
-      <c r="A10" s="24" t="inlineStr">
-        <is>
-          <t>Riesgo técnico: posible inconsistencia entre el caché (Redis) y el estado real de las reservas.</t>
-        </is>
-      </c>
-      <c r="B10" s="24" t="inlineStr">
-        <is>
-          <t>La invalidación del caché en producción depende de eventos del motor de pagos, que está fuera del alcance del prototipo.</t>
-        </is>
-      </c>
-      <c r="C10" s="24" t="inlineStr">
-        <is>
-          <t>Podría cachearse la disponibilidad de un asiento ya reservado, generando un falso positivo en las consultas de disponibilidad.</t>
-        </is>
-      </c>
-      <c r="D10" s="24" t="inlineStr">
-        <is>
-          <t>Implementar TTL conservador (≤ 30 s para asientos en fase de checkout). Diseñar y documentar una prueba de invalidación manual. Registrar la limitación formalmente en la documentación del prototipo.</t>
-        </is>
-      </c>
-      <c r="E10" s="25" t="inlineStr">
-        <is>
-          <t>Nataly Crespo
-(Ingeniera Software / DBA)</t>
-        </is>
-      </c>
-      <c r="F10" s="12" t="inlineStr">
-        <is>
-          <t>15/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="37.5" customHeight="1" s="1">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>Leyenda: Fondo ROJO = incidencia crítica que bloquea o retrasa el avance inmediato — requiere acción urgente antes del próximo punto de control. Fondo AMARILLO = dificultad activa en seguimiento con acción correctiva definida y responsable asignado. Actualizar en cada punto de control.</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="4" t="n"/>
-    </row>
-    <row r="21" ht="15.75" customHeight="1" s="1"/>
-    <row r="22" ht="15.75" customHeight="1" s="1"/>
-    <row r="23" ht="15.75" customHeight="1" s="1"/>
-    <row r="24" ht="15.75" customHeight="1" s="1"/>
-    <row r="25" ht="15.75" customHeight="1" s="1"/>
-    <row r="26" ht="15.75" customHeight="1" s="1"/>
-    <row r="27" ht="15.75" customHeight="1" s="1"/>
-    <row r="28" ht="15.75" customHeight="1" s="1"/>
+    </row>
     <row r="29" ht="15.75" customHeight="1" s="1"/>
     <row r="30" ht="15.75" customHeight="1" s="1"/>
     <row r="31" ht="15.75" customHeight="1" s="1"/>
@@ -5184,13 +3509,1370 @@
     <row r="999" ht="15.75" customHeight="1" s="1"/>
     <row r="1000" ht="15.75" customHeight="1" s="1"/>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A3:F3"/>
-  </mergeCells>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" useFirstPageNumber="0" pageOrder="downThenOver" usePrinterDefaults="1" blackAndWhite="0" draft="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:F29"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
+  <cols>
+    <col width="33" customWidth="1" style="1" min="1" max="1"/>
+    <col width="26" customWidth="1" style="1" min="2" max="2"/>
+    <col width="30" customWidth="1" style="1" min="3" max="3"/>
+    <col width="38" customWidth="1" style="1" min="4" max="4"/>
+    <col width="22" customWidth="1" style="1" min="5" max="5"/>
+    <col width="16" customWidth="1" style="1" min="6" max="6"/>
+    <col width="8.710000000000001" customWidth="1" style="1" min="7" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="27.75" customHeight="1" s="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>MATRIZ 3 — DIFICULTADES E INCIDENCIAS  ·  GRUPO 2 FIREFOX</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="19.5" customHeight="1" s="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Registra incidencias reales, analiza su efecto y define acciones correctivas con responsable y fecha. Una dificultad no debe ocultarse: debe registrarse, analizarse y convertirse en acción concreta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="4.5" customHeight="1" s="1">
+      <c r="A3" s="6" t="n"/>
+    </row>
+    <row r="4" ht="24" customHeight="1" s="1">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Finalidad: esta matriz ayuda a registrar incidencias reales, analizar su efecto en el trabajo y definir acciones correctivas con responsable y fecha de revisión.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="27.75" customHeight="1" s="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Dificultad / Incidencia</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Causa probable</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Efecto en el avance</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Acción correctiva</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>Fecha revisión</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="99.75" customHeight="1" s="1">
+      <c r="A6" s="32" t="inlineStr">
+        <is>
+          <t>Sin acceso al código fuente, base de datos ni entorno de producción de BoA.</t>
+        </is>
+      </c>
+      <c r="B6" s="32" t="inlineStr">
+        <is>
+          <t>BoA es empresa estatal con restricciones de acceso a sus sistemas.</t>
+        </is>
+      </c>
+      <c r="C6" s="32" t="inlineStr">
+        <is>
+          <t>Toda validación debe ser sobre datos simulados.</t>
+        </is>
+      </c>
+      <c r="D6" s="32" t="inlineStr">
+        <is>
+          <t>Desarrollar el prototipo con datos simulados coherentes (Seeders). Documentado como limitación del estudio.</t>
+        </is>
+      </c>
+      <c r="E6" s="32" t="inlineStr">
+        <is>
+          <t>Todo el equipo</t>
+        </is>
+      </c>
+      <c r="F6" s="33" t="inlineStr">
+        <is>
+          <t>Resuelto</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="99.75" customHeight="1" s="1">
+      <c r="A7" s="32" t="inlineStr">
+        <is>
+          <t>Complejidad de orquestar múltiples servicios (Postgres, Valkey, API) localmente.</t>
+        </is>
+      </c>
+      <c r="B7" s="32" t="inlineStr">
+        <is>
+          <t>Se subestimó el tiempo de configuración y despliegue del entorno para todo el equipo.</t>
+        </is>
+      </c>
+      <c r="C7" s="32" t="inlineStr">
+        <is>
+          <t>Retraso inicial en el desarrollo concurrente por problemas de dependencias.</t>
+        </is>
+      </c>
+      <c r="D7" s="32" t="inlineStr">
+        <is>
+          <t>Se implementó Infraestructura como Código (Docker Compose) y comandos Makefile para estandarizar el despliegue en un clic.</t>
+        </is>
+      </c>
+      <c r="E7" s="32" t="inlineStr">
+        <is>
+          <t>Iver Pinaya</t>
+        </is>
+      </c>
+      <c r="F7" s="33" t="inlineStr">
+        <is>
+          <t>Resuelto</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="99.75" customHeight="1" s="1">
+      <c r="A8" s="34" t="inlineStr">
+        <is>
+          <t>Desacoplamiento complejo de operaciones de Lectura y Escritura (CQRS).</t>
+        </is>
+      </c>
+      <c r="B8" s="34" t="inlineStr">
+        <is>
+          <t>La arquitectura obligó a separar repositorios de BD y refactorizar controladores en FastAPI.</t>
+        </is>
+      </c>
+      <c r="C8" s="34" t="inlineStr">
+        <is>
+          <t>Curva de aprendizaje elevada para adaptar el código monolítico a un patrón segregado.</t>
+        </is>
+      </c>
+      <c r="D8" s="34" t="inlineStr">
+        <is>
+          <t>Implementación de inyección de dependencias y separación estricta en servicios (reserva_service vs disponibilidad_service).</t>
+        </is>
+      </c>
+      <c r="E8" s="34" t="inlineStr">
+        <is>
+          <t>Thiago Sossa</t>
+        </is>
+      </c>
+      <c r="F8" s="35" t="inlineStr">
+        <is>
+          <t>Resuelto</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="99.75" customHeight="1" s="1">
+      <c r="A9" s="34" t="inlineStr">
+        <is>
+          <t>Sin datos históricos de tráfico de campañas (Vuelos Azules).</t>
+        </is>
+      </c>
+      <c r="B9" s="34" t="inlineStr">
+        <is>
+          <t>Información interna y confidencial que BoA no publica.</t>
+        </is>
+      </c>
+      <c r="C9" s="34" t="inlineStr">
+        <is>
+          <t>Escenarios de prueba no tienen base de carga exacta local.</t>
+        </is>
+      </c>
+      <c r="D9" s="34" t="inlineStr">
+        <is>
+          <t>Modelar escenarios K6 con benchmarks de la industria (LATAM, Avianca) como proxy de carga técnica.</t>
+        </is>
+      </c>
+      <c r="E9" s="34" t="inlineStr">
+        <is>
+          <t>Wilson Gonzales</t>
+        </is>
+      </c>
+      <c r="F9" s="35" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="99.75" customHeight="1" s="1">
+      <c r="A10" s="34" t="inlineStr">
+        <is>
+          <t>Riesgo de inconsistencia temporal entre Caché (Valkey) y Base de Datos (Postgres).</t>
+        </is>
+      </c>
+      <c r="B10" s="34" t="inlineStr">
+        <is>
+          <t>La propagación de la disponibilidad tras una reserva requiere sincronización o invalidación rápida.</t>
+        </is>
+      </c>
+      <c r="C10" s="34" t="inlineStr">
+        <is>
+          <t>Podría mostrar asientos falsamente disponibles (falsos positivos) en consultas cacheadas.</t>
+        </is>
+      </c>
+      <c r="D10" s="34" t="inlineStr">
+        <is>
+          <t>Implementar TTL conservador y expiración bajo demanda de keys específicas por vuelo tras una reserva exitosa.</t>
+        </is>
+      </c>
+      <c r="E10" s="34" t="inlineStr">
+        <is>
+          <t>Nataly Crespo</t>
+        </is>
+      </c>
+      <c r="F10" s="35" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="37.5" customHeight="1" s="1">
+      <c r="A11" s="9" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+    </row>
+    <row r="21" ht="15.75" customHeight="1" s="1">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+    </row>
+    <row r="22" ht="15.75" customHeight="1" s="1">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+    </row>
+    <row r="23" ht="15.75" customHeight="1" s="1">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="1">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+    </row>
+    <row r="25" ht="15.75" customHeight="1" s="1">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+    </row>
+    <row r="26" ht="15.75" customHeight="1" s="1">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+    </row>
+    <row r="27" ht="15.75" customHeight="1" s="1">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+    </row>
+    <row r="28" ht="15.75" customHeight="1" s="1">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+    </row>
+    <row r="29" ht="15.75" customHeight="1" s="1">
+      <c r="A29" t="inlineStr"/>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+    </row>
+    <row r="30" ht="15.75" customHeight="1" s="1"/>
+    <row r="31" ht="15.75" customHeight="1" s="1"/>
+    <row r="32" ht="15.75" customHeight="1" s="1"/>
+    <row r="33" ht="15.75" customHeight="1" s="1"/>
+    <row r="34" ht="15.75" customHeight="1" s="1"/>
+    <row r="35" ht="15.75" customHeight="1" s="1"/>
+    <row r="36" ht="15.75" customHeight="1" s="1"/>
+    <row r="37" ht="15.75" customHeight="1" s="1"/>
+    <row r="38" ht="15.75" customHeight="1" s="1"/>
+    <row r="39" ht="15.75" customHeight="1" s="1"/>
+    <row r="40" ht="15.75" customHeight="1" s="1"/>
+    <row r="41" ht="15.75" customHeight="1" s="1"/>
+    <row r="42" ht="15.75" customHeight="1" s="1"/>
+    <row r="43" ht="15.75" customHeight="1" s="1"/>
+    <row r="44" ht="15.75" customHeight="1" s="1"/>
+    <row r="45" ht="15.75" customHeight="1" s="1"/>
+    <row r="46" ht="15.75" customHeight="1" s="1"/>
+    <row r="47" ht="15.75" customHeight="1" s="1"/>
+    <row r="48" ht="15.75" customHeight="1" s="1"/>
+    <row r="49" ht="15.75" customHeight="1" s="1"/>
+    <row r="50" ht="15.75" customHeight="1" s="1"/>
+    <row r="51" ht="15.75" customHeight="1" s="1"/>
+    <row r="52" ht="15.75" customHeight="1" s="1"/>
+    <row r="53" ht="15.75" customHeight="1" s="1"/>
+    <row r="54" ht="15.75" customHeight="1" s="1"/>
+    <row r="55" ht="15.75" customHeight="1" s="1"/>
+    <row r="56" ht="15.75" customHeight="1" s="1"/>
+    <row r="57" ht="15.75" customHeight="1" s="1"/>
+    <row r="58" ht="15.75" customHeight="1" s="1"/>
+    <row r="59" ht="15.75" customHeight="1" s="1"/>
+    <row r="60" ht="15.75" customHeight="1" s="1"/>
+    <row r="61" ht="15.75" customHeight="1" s="1"/>
+    <row r="62" ht="15.75" customHeight="1" s="1"/>
+    <row r="63" ht="15.75" customHeight="1" s="1"/>
+    <row r="64" ht="15.75" customHeight="1" s="1"/>
+    <row r="65" ht="15.75" customHeight="1" s="1"/>
+    <row r="66" ht="15.75" customHeight="1" s="1"/>
+    <row r="67" ht="15.75" customHeight="1" s="1"/>
+    <row r="68" ht="15.75" customHeight="1" s="1"/>
+    <row r="69" ht="15.75" customHeight="1" s="1"/>
+    <row r="70" ht="15.75" customHeight="1" s="1"/>
+    <row r="71" ht="15.75" customHeight="1" s="1"/>
+    <row r="72" ht="15.75" customHeight="1" s="1"/>
+    <row r="73" ht="15.75" customHeight="1" s="1"/>
+    <row r="74" ht="15.75" customHeight="1" s="1"/>
+    <row r="75" ht="15.75" customHeight="1" s="1"/>
+    <row r="76" ht="15.75" customHeight="1" s="1"/>
+    <row r="77" ht="15.75" customHeight="1" s="1"/>
+    <row r="78" ht="15.75" customHeight="1" s="1"/>
+    <row r="79" ht="15.75" customHeight="1" s="1"/>
+    <row r="80" ht="15.75" customHeight="1" s="1"/>
+    <row r="81" ht="15.75" customHeight="1" s="1"/>
+    <row r="82" ht="15.75" customHeight="1" s="1"/>
+    <row r="83" ht="15.75" customHeight="1" s="1"/>
+    <row r="84" ht="15.75" customHeight="1" s="1"/>
+    <row r="85" ht="15.75" customHeight="1" s="1"/>
+    <row r="86" ht="15.75" customHeight="1" s="1"/>
+    <row r="87" ht="15.75" customHeight="1" s="1"/>
+    <row r="88" ht="15.75" customHeight="1" s="1"/>
+    <row r="89" ht="15.75" customHeight="1" s="1"/>
+    <row r="90" ht="15.75" customHeight="1" s="1"/>
+    <row r="91" ht="15.75" customHeight="1" s="1"/>
+    <row r="92" ht="15.75" customHeight="1" s="1"/>
+    <row r="93" ht="15.75" customHeight="1" s="1"/>
+    <row r="94" ht="15.75" customHeight="1" s="1"/>
+    <row r="95" ht="15.75" customHeight="1" s="1"/>
+    <row r="96" ht="15.75" customHeight="1" s="1"/>
+    <row r="97" ht="15.75" customHeight="1" s="1"/>
+    <row r="98" ht="15.75" customHeight="1" s="1"/>
+    <row r="99" ht="15.75" customHeight="1" s="1"/>
+    <row r="100" ht="15.75" customHeight="1" s="1"/>
+    <row r="101" ht="15.75" customHeight="1" s="1"/>
+    <row r="102" ht="15.75" customHeight="1" s="1"/>
+    <row r="103" ht="15.75" customHeight="1" s="1"/>
+    <row r="104" ht="15.75" customHeight="1" s="1"/>
+    <row r="105" ht="15.75" customHeight="1" s="1"/>
+    <row r="106" ht="15.75" customHeight="1" s="1"/>
+    <row r="107" ht="15.75" customHeight="1" s="1"/>
+    <row r="108" ht="15.75" customHeight="1" s="1"/>
+    <row r="109" ht="15.75" customHeight="1" s="1"/>
+    <row r="110" ht="15.75" customHeight="1" s="1"/>
+    <row r="111" ht="15.75" customHeight="1" s="1"/>
+    <row r="112" ht="15.75" customHeight="1" s="1"/>
+    <row r="113" ht="15.75" customHeight="1" s="1"/>
+    <row r="114" ht="15.75" customHeight="1" s="1"/>
+    <row r="115" ht="15.75" customHeight="1" s="1"/>
+    <row r="116" ht="15.75" customHeight="1" s="1"/>
+    <row r="117" ht="15.75" customHeight="1" s="1"/>
+    <row r="118" ht="15.75" customHeight="1" s="1"/>
+    <row r="119" ht="15.75" customHeight="1" s="1"/>
+    <row r="120" ht="15.75" customHeight="1" s="1"/>
+    <row r="121" ht="15.75" customHeight="1" s="1"/>
+    <row r="122" ht="15.75" customHeight="1" s="1"/>
+    <row r="123" ht="15.75" customHeight="1" s="1"/>
+    <row r="124" ht="15.75" customHeight="1" s="1"/>
+    <row r="125" ht="15.75" customHeight="1" s="1"/>
+    <row r="126" ht="15.75" customHeight="1" s="1"/>
+    <row r="127" ht="15.75" customHeight="1" s="1"/>
+    <row r="128" ht="15.75" customHeight="1" s="1"/>
+    <row r="129" ht="15.75" customHeight="1" s="1"/>
+    <row r="130" ht="15.75" customHeight="1" s="1"/>
+    <row r="131" ht="15.75" customHeight="1" s="1"/>
+    <row r="132" ht="15.75" customHeight="1" s="1"/>
+    <row r="133" ht="15.75" customHeight="1" s="1"/>
+    <row r="134" ht="15.75" customHeight="1" s="1"/>
+    <row r="135" ht="15.75" customHeight="1" s="1"/>
+    <row r="136" ht="15.75" customHeight="1" s="1"/>
+    <row r="137" ht="15.75" customHeight="1" s="1"/>
+    <row r="138" ht="15.75" customHeight="1" s="1"/>
+    <row r="139" ht="15.75" customHeight="1" s="1"/>
+    <row r="140" ht="15.75" customHeight="1" s="1"/>
+    <row r="141" ht="15.75" customHeight="1" s="1"/>
+    <row r="142" ht="15.75" customHeight="1" s="1"/>
+    <row r="143" ht="15.75" customHeight="1" s="1"/>
+    <row r="144" ht="15.75" customHeight="1" s="1"/>
+    <row r="145" ht="15.75" customHeight="1" s="1"/>
+    <row r="146" ht="15.75" customHeight="1" s="1"/>
+    <row r="147" ht="15.75" customHeight="1" s="1"/>
+    <row r="148" ht="15.75" customHeight="1" s="1"/>
+    <row r="149" ht="15.75" customHeight="1" s="1"/>
+    <row r="150" ht="15.75" customHeight="1" s="1"/>
+    <row r="151" ht="15.75" customHeight="1" s="1"/>
+    <row r="152" ht="15.75" customHeight="1" s="1"/>
+    <row r="153" ht="15.75" customHeight="1" s="1"/>
+    <row r="154" ht="15.75" customHeight="1" s="1"/>
+    <row r="155" ht="15.75" customHeight="1" s="1"/>
+    <row r="156" ht="15.75" customHeight="1" s="1"/>
+    <row r="157" ht="15.75" customHeight="1" s="1"/>
+    <row r="158" ht="15.75" customHeight="1" s="1"/>
+    <row r="159" ht="15.75" customHeight="1" s="1"/>
+    <row r="160" ht="15.75" customHeight="1" s="1"/>
+    <row r="161" ht="15.75" customHeight="1" s="1"/>
+    <row r="162" ht="15.75" customHeight="1" s="1"/>
+    <row r="163" ht="15.75" customHeight="1" s="1"/>
+    <row r="164" ht="15.75" customHeight="1" s="1"/>
+    <row r="165" ht="15.75" customHeight="1" s="1"/>
+    <row r="166" ht="15.75" customHeight="1" s="1"/>
+    <row r="167" ht="15.75" customHeight="1" s="1"/>
+    <row r="168" ht="15.75" customHeight="1" s="1"/>
+    <row r="169" ht="15.75" customHeight="1" s="1"/>
+    <row r="170" ht="15.75" customHeight="1" s="1"/>
+    <row r="171" ht="15.75" customHeight="1" s="1"/>
+    <row r="172" ht="15.75" customHeight="1" s="1"/>
+    <row r="173" ht="15.75" customHeight="1" s="1"/>
+    <row r="174" ht="15.75" customHeight="1" s="1"/>
+    <row r="175" ht="15.75" customHeight="1" s="1"/>
+    <row r="176" ht="15.75" customHeight="1" s="1"/>
+    <row r="177" ht="15.75" customHeight="1" s="1"/>
+    <row r="178" ht="15.75" customHeight="1" s="1"/>
+    <row r="179" ht="15.75" customHeight="1" s="1"/>
+    <row r="180" ht="15.75" customHeight="1" s="1"/>
+    <row r="181" ht="15.75" customHeight="1" s="1"/>
+    <row r="182" ht="15.75" customHeight="1" s="1"/>
+    <row r="183" ht="15.75" customHeight="1" s="1"/>
+    <row r="184" ht="15.75" customHeight="1" s="1"/>
+    <row r="185" ht="15.75" customHeight="1" s="1"/>
+    <row r="186" ht="15.75" customHeight="1" s="1"/>
+    <row r="187" ht="15.75" customHeight="1" s="1"/>
+    <row r="188" ht="15.75" customHeight="1" s="1"/>
+    <row r="189" ht="15.75" customHeight="1" s="1"/>
+    <row r="190" ht="15.75" customHeight="1" s="1"/>
+    <row r="191" ht="15.75" customHeight="1" s="1"/>
+    <row r="192" ht="15.75" customHeight="1" s="1"/>
+    <row r="193" ht="15.75" customHeight="1" s="1"/>
+    <row r="194" ht="15.75" customHeight="1" s="1"/>
+    <row r="195" ht="15.75" customHeight="1" s="1"/>
+    <row r="196" ht="15.75" customHeight="1" s="1"/>
+    <row r="197" ht="15.75" customHeight="1" s="1"/>
+    <row r="198" ht="15.75" customHeight="1" s="1"/>
+    <row r="199" ht="15.75" customHeight="1" s="1"/>
+    <row r="200" ht="15.75" customHeight="1" s="1"/>
+    <row r="201" ht="15.75" customHeight="1" s="1"/>
+    <row r="202" ht="15.75" customHeight="1" s="1"/>
+    <row r="203" ht="15.75" customHeight="1" s="1"/>
+    <row r="204" ht="15.75" customHeight="1" s="1"/>
+    <row r="205" ht="15.75" customHeight="1" s="1"/>
+    <row r="206" ht="15.75" customHeight="1" s="1"/>
+    <row r="207" ht="15.75" customHeight="1" s="1"/>
+    <row r="208" ht="15.75" customHeight="1" s="1"/>
+    <row r="209" ht="15.75" customHeight="1" s="1"/>
+    <row r="210" ht="15.75" customHeight="1" s="1"/>
+    <row r="211" ht="15.75" customHeight="1" s="1"/>
+    <row r="212" ht="15.75" customHeight="1" s="1"/>
+    <row r="213" ht="15.75" customHeight="1" s="1"/>
+    <row r="214" ht="15.75" customHeight="1" s="1"/>
+    <row r="215" ht="15.75" customHeight="1" s="1"/>
+    <row r="216" ht="15.75" customHeight="1" s="1"/>
+    <row r="217" ht="15.75" customHeight="1" s="1"/>
+    <row r="218" ht="15.75" customHeight="1" s="1"/>
+    <row r="219" ht="15.75" customHeight="1" s="1"/>
+    <row r="220" ht="15.75" customHeight="1" s="1"/>
+    <row r="221" ht="15.75" customHeight="1" s="1"/>
+    <row r="222" ht="15.75" customHeight="1" s="1"/>
+    <row r="223" ht="15.75" customHeight="1" s="1"/>
+    <row r="224" ht="15.75" customHeight="1" s="1"/>
+    <row r="225" ht="15.75" customHeight="1" s="1"/>
+    <row r="226" ht="15.75" customHeight="1" s="1"/>
+    <row r="227" ht="15.75" customHeight="1" s="1"/>
+    <row r="228" ht="15.75" customHeight="1" s="1"/>
+    <row r="229" ht="15.75" customHeight="1" s="1"/>
+    <row r="230" ht="15.75" customHeight="1" s="1"/>
+    <row r="231" ht="15.75" customHeight="1" s="1"/>
+    <row r="232" ht="15.75" customHeight="1" s="1"/>
+    <row r="233" ht="15.75" customHeight="1" s="1"/>
+    <row r="234" ht="15.75" customHeight="1" s="1"/>
+    <row r="235" ht="15.75" customHeight="1" s="1"/>
+    <row r="236" ht="15.75" customHeight="1" s="1"/>
+    <row r="237" ht="15.75" customHeight="1" s="1"/>
+    <row r="238" ht="15.75" customHeight="1" s="1"/>
+    <row r="239" ht="15.75" customHeight="1" s="1"/>
+    <row r="240" ht="15.75" customHeight="1" s="1"/>
+    <row r="241" ht="15.75" customHeight="1" s="1"/>
+    <row r="242" ht="15.75" customHeight="1" s="1"/>
+    <row r="243" ht="15.75" customHeight="1" s="1"/>
+    <row r="244" ht="15.75" customHeight="1" s="1"/>
+    <row r="245" ht="15.75" customHeight="1" s="1"/>
+    <row r="246" ht="15.75" customHeight="1" s="1"/>
+    <row r="247" ht="15.75" customHeight="1" s="1"/>
+    <row r="248" ht="15.75" customHeight="1" s="1"/>
+    <row r="249" ht="15.75" customHeight="1" s="1"/>
+    <row r="250" ht="15.75" customHeight="1" s="1"/>
+    <row r="251" ht="15.75" customHeight="1" s="1"/>
+    <row r="252" ht="15.75" customHeight="1" s="1"/>
+    <row r="253" ht="15.75" customHeight="1" s="1"/>
+    <row r="254" ht="15.75" customHeight="1" s="1"/>
+    <row r="255" ht="15.75" customHeight="1" s="1"/>
+    <row r="256" ht="15.75" customHeight="1" s="1"/>
+    <row r="257" ht="15.75" customHeight="1" s="1"/>
+    <row r="258" ht="15.75" customHeight="1" s="1"/>
+    <row r="259" ht="15.75" customHeight="1" s="1"/>
+    <row r="260" ht="15.75" customHeight="1" s="1"/>
+    <row r="261" ht="15.75" customHeight="1" s="1"/>
+    <row r="262" ht="15.75" customHeight="1" s="1"/>
+    <row r="263" ht="15.75" customHeight="1" s="1"/>
+    <row r="264" ht="15.75" customHeight="1" s="1"/>
+    <row r="265" ht="15.75" customHeight="1" s="1"/>
+    <row r="266" ht="15.75" customHeight="1" s="1"/>
+    <row r="267" ht="15.75" customHeight="1" s="1"/>
+    <row r="268" ht="15.75" customHeight="1" s="1"/>
+    <row r="269" ht="15.75" customHeight="1" s="1"/>
+    <row r="270" ht="15.75" customHeight="1" s="1"/>
+    <row r="271" ht="15.75" customHeight="1" s="1"/>
+    <row r="272" ht="15.75" customHeight="1" s="1"/>
+    <row r="273" ht="15.75" customHeight="1" s="1"/>
+    <row r="274" ht="15.75" customHeight="1" s="1"/>
+    <row r="275" ht="15.75" customHeight="1" s="1"/>
+    <row r="276" ht="15.75" customHeight="1" s="1"/>
+    <row r="277" ht="15.75" customHeight="1" s="1"/>
+    <row r="278" ht="15.75" customHeight="1" s="1"/>
+    <row r="279" ht="15.75" customHeight="1" s="1"/>
+    <row r="280" ht="15.75" customHeight="1" s="1"/>
+    <row r="281" ht="15.75" customHeight="1" s="1"/>
+    <row r="282" ht="15.75" customHeight="1" s="1"/>
+    <row r="283" ht="15.75" customHeight="1" s="1"/>
+    <row r="284" ht="15.75" customHeight="1" s="1"/>
+    <row r="285" ht="15.75" customHeight="1" s="1"/>
+    <row r="286" ht="15.75" customHeight="1" s="1"/>
+    <row r="287" ht="15.75" customHeight="1" s="1"/>
+    <row r="288" ht="15.75" customHeight="1" s="1"/>
+    <row r="289" ht="15.75" customHeight="1" s="1"/>
+    <row r="290" ht="15.75" customHeight="1" s="1"/>
+    <row r="291" ht="15.75" customHeight="1" s="1"/>
+    <row r="292" ht="15.75" customHeight="1" s="1"/>
+    <row r="293" ht="15.75" customHeight="1" s="1"/>
+    <row r="294" ht="15.75" customHeight="1" s="1"/>
+    <row r="295" ht="15.75" customHeight="1" s="1"/>
+    <row r="296" ht="15.75" customHeight="1" s="1"/>
+    <row r="297" ht="15.75" customHeight="1" s="1"/>
+    <row r="298" ht="15.75" customHeight="1" s="1"/>
+    <row r="299" ht="15.75" customHeight="1" s="1"/>
+    <row r="300" ht="15.75" customHeight="1" s="1"/>
+    <row r="301" ht="15.75" customHeight="1" s="1"/>
+    <row r="302" ht="15.75" customHeight="1" s="1"/>
+    <row r="303" ht="15.75" customHeight="1" s="1"/>
+    <row r="304" ht="15.75" customHeight="1" s="1"/>
+    <row r="305" ht="15.75" customHeight="1" s="1"/>
+    <row r="306" ht="15.75" customHeight="1" s="1"/>
+    <row r="307" ht="15.75" customHeight="1" s="1"/>
+    <row r="308" ht="15.75" customHeight="1" s="1"/>
+    <row r="309" ht="15.75" customHeight="1" s="1"/>
+    <row r="310" ht="15.75" customHeight="1" s="1"/>
+    <row r="311" ht="15.75" customHeight="1" s="1"/>
+    <row r="312" ht="15.75" customHeight="1" s="1"/>
+    <row r="313" ht="15.75" customHeight="1" s="1"/>
+    <row r="314" ht="15.75" customHeight="1" s="1"/>
+    <row r="315" ht="15.75" customHeight="1" s="1"/>
+    <row r="316" ht="15.75" customHeight="1" s="1"/>
+    <row r="317" ht="15.75" customHeight="1" s="1"/>
+    <row r="318" ht="15.75" customHeight="1" s="1"/>
+    <row r="319" ht="15.75" customHeight="1" s="1"/>
+    <row r="320" ht="15.75" customHeight="1" s="1"/>
+    <row r="321" ht="15.75" customHeight="1" s="1"/>
+    <row r="322" ht="15.75" customHeight="1" s="1"/>
+    <row r="323" ht="15.75" customHeight="1" s="1"/>
+    <row r="324" ht="15.75" customHeight="1" s="1"/>
+    <row r="325" ht="15.75" customHeight="1" s="1"/>
+    <row r="326" ht="15.75" customHeight="1" s="1"/>
+    <row r="327" ht="15.75" customHeight="1" s="1"/>
+    <row r="328" ht="15.75" customHeight="1" s="1"/>
+    <row r="329" ht="15.75" customHeight="1" s="1"/>
+    <row r="330" ht="15.75" customHeight="1" s="1"/>
+    <row r="331" ht="15.75" customHeight="1" s="1"/>
+    <row r="332" ht="15.75" customHeight="1" s="1"/>
+    <row r="333" ht="15.75" customHeight="1" s="1"/>
+    <row r="334" ht="15.75" customHeight="1" s="1"/>
+    <row r="335" ht="15.75" customHeight="1" s="1"/>
+    <row r="336" ht="15.75" customHeight="1" s="1"/>
+    <row r="337" ht="15.75" customHeight="1" s="1"/>
+    <row r="338" ht="15.75" customHeight="1" s="1"/>
+    <row r="339" ht="15.75" customHeight="1" s="1"/>
+    <row r="340" ht="15.75" customHeight="1" s="1"/>
+    <row r="341" ht="15.75" customHeight="1" s="1"/>
+    <row r="342" ht="15.75" customHeight="1" s="1"/>
+    <row r="343" ht="15.75" customHeight="1" s="1"/>
+    <row r="344" ht="15.75" customHeight="1" s="1"/>
+    <row r="345" ht="15.75" customHeight="1" s="1"/>
+    <row r="346" ht="15.75" customHeight="1" s="1"/>
+    <row r="347" ht="15.75" customHeight="1" s="1"/>
+    <row r="348" ht="15.75" customHeight="1" s="1"/>
+    <row r="349" ht="15.75" customHeight="1" s="1"/>
+    <row r="350" ht="15.75" customHeight="1" s="1"/>
+    <row r="351" ht="15.75" customHeight="1" s="1"/>
+    <row r="352" ht="15.75" customHeight="1" s="1"/>
+    <row r="353" ht="15.75" customHeight="1" s="1"/>
+    <row r="354" ht="15.75" customHeight="1" s="1"/>
+    <row r="355" ht="15.75" customHeight="1" s="1"/>
+    <row r="356" ht="15.75" customHeight="1" s="1"/>
+    <row r="357" ht="15.75" customHeight="1" s="1"/>
+    <row r="358" ht="15.75" customHeight="1" s="1"/>
+    <row r="359" ht="15.75" customHeight="1" s="1"/>
+    <row r="360" ht="15.75" customHeight="1" s="1"/>
+    <row r="361" ht="15.75" customHeight="1" s="1"/>
+    <row r="362" ht="15.75" customHeight="1" s="1"/>
+    <row r="363" ht="15.75" customHeight="1" s="1"/>
+    <row r="364" ht="15.75" customHeight="1" s="1"/>
+    <row r="365" ht="15.75" customHeight="1" s="1"/>
+    <row r="366" ht="15.75" customHeight="1" s="1"/>
+    <row r="367" ht="15.75" customHeight="1" s="1"/>
+    <row r="368" ht="15.75" customHeight="1" s="1"/>
+    <row r="369" ht="15.75" customHeight="1" s="1"/>
+    <row r="370" ht="15.75" customHeight="1" s="1"/>
+    <row r="371" ht="15.75" customHeight="1" s="1"/>
+    <row r="372" ht="15.75" customHeight="1" s="1"/>
+    <row r="373" ht="15.75" customHeight="1" s="1"/>
+    <row r="374" ht="15.75" customHeight="1" s="1"/>
+    <row r="375" ht="15.75" customHeight="1" s="1"/>
+    <row r="376" ht="15.75" customHeight="1" s="1"/>
+    <row r="377" ht="15.75" customHeight="1" s="1"/>
+    <row r="378" ht="15.75" customHeight="1" s="1"/>
+    <row r="379" ht="15.75" customHeight="1" s="1"/>
+    <row r="380" ht="15.75" customHeight="1" s="1"/>
+    <row r="381" ht="15.75" customHeight="1" s="1"/>
+    <row r="382" ht="15.75" customHeight="1" s="1"/>
+    <row r="383" ht="15.75" customHeight="1" s="1"/>
+    <row r="384" ht="15.75" customHeight="1" s="1"/>
+    <row r="385" ht="15.75" customHeight="1" s="1"/>
+    <row r="386" ht="15.75" customHeight="1" s="1"/>
+    <row r="387" ht="15.75" customHeight="1" s="1"/>
+    <row r="388" ht="15.75" customHeight="1" s="1"/>
+    <row r="389" ht="15.75" customHeight="1" s="1"/>
+    <row r="390" ht="15.75" customHeight="1" s="1"/>
+    <row r="391" ht="15.75" customHeight="1" s="1"/>
+    <row r="392" ht="15.75" customHeight="1" s="1"/>
+    <row r="393" ht="15.75" customHeight="1" s="1"/>
+    <row r="394" ht="15.75" customHeight="1" s="1"/>
+    <row r="395" ht="15.75" customHeight="1" s="1"/>
+    <row r="396" ht="15.75" customHeight="1" s="1"/>
+    <row r="397" ht="15.75" customHeight="1" s="1"/>
+    <row r="398" ht="15.75" customHeight="1" s="1"/>
+    <row r="399" ht="15.75" customHeight="1" s="1"/>
+    <row r="400" ht="15.75" customHeight="1" s="1"/>
+    <row r="401" ht="15.75" customHeight="1" s="1"/>
+    <row r="402" ht="15.75" customHeight="1" s="1"/>
+    <row r="403" ht="15.75" customHeight="1" s="1"/>
+    <row r="404" ht="15.75" customHeight="1" s="1"/>
+    <row r="405" ht="15.75" customHeight="1" s="1"/>
+    <row r="406" ht="15.75" customHeight="1" s="1"/>
+    <row r="407" ht="15.75" customHeight="1" s="1"/>
+    <row r="408" ht="15.75" customHeight="1" s="1"/>
+    <row r="409" ht="15.75" customHeight="1" s="1"/>
+    <row r="410" ht="15.75" customHeight="1" s="1"/>
+    <row r="411" ht="15.75" customHeight="1" s="1"/>
+    <row r="412" ht="15.75" customHeight="1" s="1"/>
+    <row r="413" ht="15.75" customHeight="1" s="1"/>
+    <row r="414" ht="15.75" customHeight="1" s="1"/>
+    <row r="415" ht="15.75" customHeight="1" s="1"/>
+    <row r="416" ht="15.75" customHeight="1" s="1"/>
+    <row r="417" ht="15.75" customHeight="1" s="1"/>
+    <row r="418" ht="15.75" customHeight="1" s="1"/>
+    <row r="419" ht="15.75" customHeight="1" s="1"/>
+    <row r="420" ht="15.75" customHeight="1" s="1"/>
+    <row r="421" ht="15.75" customHeight="1" s="1"/>
+    <row r="422" ht="15.75" customHeight="1" s="1"/>
+    <row r="423" ht="15.75" customHeight="1" s="1"/>
+    <row r="424" ht="15.75" customHeight="1" s="1"/>
+    <row r="425" ht="15.75" customHeight="1" s="1"/>
+    <row r="426" ht="15.75" customHeight="1" s="1"/>
+    <row r="427" ht="15.75" customHeight="1" s="1"/>
+    <row r="428" ht="15.75" customHeight="1" s="1"/>
+    <row r="429" ht="15.75" customHeight="1" s="1"/>
+    <row r="430" ht="15.75" customHeight="1" s="1"/>
+    <row r="431" ht="15.75" customHeight="1" s="1"/>
+    <row r="432" ht="15.75" customHeight="1" s="1"/>
+    <row r="433" ht="15.75" customHeight="1" s="1"/>
+    <row r="434" ht="15.75" customHeight="1" s="1"/>
+    <row r="435" ht="15.75" customHeight="1" s="1"/>
+    <row r="436" ht="15.75" customHeight="1" s="1"/>
+    <row r="437" ht="15.75" customHeight="1" s="1"/>
+    <row r="438" ht="15.75" customHeight="1" s="1"/>
+    <row r="439" ht="15.75" customHeight="1" s="1"/>
+    <row r="440" ht="15.75" customHeight="1" s="1"/>
+    <row r="441" ht="15.75" customHeight="1" s="1"/>
+    <row r="442" ht="15.75" customHeight="1" s="1"/>
+    <row r="443" ht="15.75" customHeight="1" s="1"/>
+    <row r="444" ht="15.75" customHeight="1" s="1"/>
+    <row r="445" ht="15.75" customHeight="1" s="1"/>
+    <row r="446" ht="15.75" customHeight="1" s="1"/>
+    <row r="447" ht="15.75" customHeight="1" s="1"/>
+    <row r="448" ht="15.75" customHeight="1" s="1"/>
+    <row r="449" ht="15.75" customHeight="1" s="1"/>
+    <row r="450" ht="15.75" customHeight="1" s="1"/>
+    <row r="451" ht="15.75" customHeight="1" s="1"/>
+    <row r="452" ht="15.75" customHeight="1" s="1"/>
+    <row r="453" ht="15.75" customHeight="1" s="1"/>
+    <row r="454" ht="15.75" customHeight="1" s="1"/>
+    <row r="455" ht="15.75" customHeight="1" s="1"/>
+    <row r="456" ht="15.75" customHeight="1" s="1"/>
+    <row r="457" ht="15.75" customHeight="1" s="1"/>
+    <row r="458" ht="15.75" customHeight="1" s="1"/>
+    <row r="459" ht="15.75" customHeight="1" s="1"/>
+    <row r="460" ht="15.75" customHeight="1" s="1"/>
+    <row r="461" ht="15.75" customHeight="1" s="1"/>
+    <row r="462" ht="15.75" customHeight="1" s="1"/>
+    <row r="463" ht="15.75" customHeight="1" s="1"/>
+    <row r="464" ht="15.75" customHeight="1" s="1"/>
+    <row r="465" ht="15.75" customHeight="1" s="1"/>
+    <row r="466" ht="15.75" customHeight="1" s="1"/>
+    <row r="467" ht="15.75" customHeight="1" s="1"/>
+    <row r="468" ht="15.75" customHeight="1" s="1"/>
+    <row r="469" ht="15.75" customHeight="1" s="1"/>
+    <row r="470" ht="15.75" customHeight="1" s="1"/>
+    <row r="471" ht="15.75" customHeight="1" s="1"/>
+    <row r="472" ht="15.75" customHeight="1" s="1"/>
+    <row r="473" ht="15.75" customHeight="1" s="1"/>
+    <row r="474" ht="15.75" customHeight="1" s="1"/>
+    <row r="475" ht="15.75" customHeight="1" s="1"/>
+    <row r="476" ht="15.75" customHeight="1" s="1"/>
+    <row r="477" ht="15.75" customHeight="1" s="1"/>
+    <row r="478" ht="15.75" customHeight="1" s="1"/>
+    <row r="479" ht="15.75" customHeight="1" s="1"/>
+    <row r="480" ht="15.75" customHeight="1" s="1"/>
+    <row r="481" ht="15.75" customHeight="1" s="1"/>
+    <row r="482" ht="15.75" customHeight="1" s="1"/>
+    <row r="483" ht="15.75" customHeight="1" s="1"/>
+    <row r="484" ht="15.75" customHeight="1" s="1"/>
+    <row r="485" ht="15.75" customHeight="1" s="1"/>
+    <row r="486" ht="15.75" customHeight="1" s="1"/>
+    <row r="487" ht="15.75" customHeight="1" s="1"/>
+    <row r="488" ht="15.75" customHeight="1" s="1"/>
+    <row r="489" ht="15.75" customHeight="1" s="1"/>
+    <row r="490" ht="15.75" customHeight="1" s="1"/>
+    <row r="491" ht="15.75" customHeight="1" s="1"/>
+    <row r="492" ht="15.75" customHeight="1" s="1"/>
+    <row r="493" ht="15.75" customHeight="1" s="1"/>
+    <row r="494" ht="15.75" customHeight="1" s="1"/>
+    <row r="495" ht="15.75" customHeight="1" s="1"/>
+    <row r="496" ht="15.75" customHeight="1" s="1"/>
+    <row r="497" ht="15.75" customHeight="1" s="1"/>
+    <row r="498" ht="15.75" customHeight="1" s="1"/>
+    <row r="499" ht="15.75" customHeight="1" s="1"/>
+    <row r="500" ht="15.75" customHeight="1" s="1"/>
+    <row r="501" ht="15.75" customHeight="1" s="1"/>
+    <row r="502" ht="15.75" customHeight="1" s="1"/>
+    <row r="503" ht="15.75" customHeight="1" s="1"/>
+    <row r="504" ht="15.75" customHeight="1" s="1"/>
+    <row r="505" ht="15.75" customHeight="1" s="1"/>
+    <row r="506" ht="15.75" customHeight="1" s="1"/>
+    <row r="507" ht="15.75" customHeight="1" s="1"/>
+    <row r="508" ht="15.75" customHeight="1" s="1"/>
+    <row r="509" ht="15.75" customHeight="1" s="1"/>
+    <row r="510" ht="15.75" customHeight="1" s="1"/>
+    <row r="511" ht="15.75" customHeight="1" s="1"/>
+    <row r="512" ht="15.75" customHeight="1" s="1"/>
+    <row r="513" ht="15.75" customHeight="1" s="1"/>
+    <row r="514" ht="15.75" customHeight="1" s="1"/>
+    <row r="515" ht="15.75" customHeight="1" s="1"/>
+    <row r="516" ht="15.75" customHeight="1" s="1"/>
+    <row r="517" ht="15.75" customHeight="1" s="1"/>
+    <row r="518" ht="15.75" customHeight="1" s="1"/>
+    <row r="519" ht="15.75" customHeight="1" s="1"/>
+    <row r="520" ht="15.75" customHeight="1" s="1"/>
+    <row r="521" ht="15.75" customHeight="1" s="1"/>
+    <row r="522" ht="15.75" customHeight="1" s="1"/>
+    <row r="523" ht="15.75" customHeight="1" s="1"/>
+    <row r="524" ht="15.75" customHeight="1" s="1"/>
+    <row r="525" ht="15.75" customHeight="1" s="1"/>
+    <row r="526" ht="15.75" customHeight="1" s="1"/>
+    <row r="527" ht="15.75" customHeight="1" s="1"/>
+    <row r="528" ht="15.75" customHeight="1" s="1"/>
+    <row r="529" ht="15.75" customHeight="1" s="1"/>
+    <row r="530" ht="15.75" customHeight="1" s="1"/>
+    <row r="531" ht="15.75" customHeight="1" s="1"/>
+    <row r="532" ht="15.75" customHeight="1" s="1"/>
+    <row r="533" ht="15.75" customHeight="1" s="1"/>
+    <row r="534" ht="15.75" customHeight="1" s="1"/>
+    <row r="535" ht="15.75" customHeight="1" s="1"/>
+    <row r="536" ht="15.75" customHeight="1" s="1"/>
+    <row r="537" ht="15.75" customHeight="1" s="1"/>
+    <row r="538" ht="15.75" customHeight="1" s="1"/>
+    <row r="539" ht="15.75" customHeight="1" s="1"/>
+    <row r="540" ht="15.75" customHeight="1" s="1"/>
+    <row r="541" ht="15.75" customHeight="1" s="1"/>
+    <row r="542" ht="15.75" customHeight="1" s="1"/>
+    <row r="543" ht="15.75" customHeight="1" s="1"/>
+    <row r="544" ht="15.75" customHeight="1" s="1"/>
+    <row r="545" ht="15.75" customHeight="1" s="1"/>
+    <row r="546" ht="15.75" customHeight="1" s="1"/>
+    <row r="547" ht="15.75" customHeight="1" s="1"/>
+    <row r="548" ht="15.75" customHeight="1" s="1"/>
+    <row r="549" ht="15.75" customHeight="1" s="1"/>
+    <row r="550" ht="15.75" customHeight="1" s="1"/>
+    <row r="551" ht="15.75" customHeight="1" s="1"/>
+    <row r="552" ht="15.75" customHeight="1" s="1"/>
+    <row r="553" ht="15.75" customHeight="1" s="1"/>
+    <row r="554" ht="15.75" customHeight="1" s="1"/>
+    <row r="555" ht="15.75" customHeight="1" s="1"/>
+    <row r="556" ht="15.75" customHeight="1" s="1"/>
+    <row r="557" ht="15.75" customHeight="1" s="1"/>
+    <row r="558" ht="15.75" customHeight="1" s="1"/>
+    <row r="559" ht="15.75" customHeight="1" s="1"/>
+    <row r="560" ht="15.75" customHeight="1" s="1"/>
+    <row r="561" ht="15.75" customHeight="1" s="1"/>
+    <row r="562" ht="15.75" customHeight="1" s="1"/>
+    <row r="563" ht="15.75" customHeight="1" s="1"/>
+    <row r="564" ht="15.75" customHeight="1" s="1"/>
+    <row r="565" ht="15.75" customHeight="1" s="1"/>
+    <row r="566" ht="15.75" customHeight="1" s="1"/>
+    <row r="567" ht="15.75" customHeight="1" s="1"/>
+    <row r="568" ht="15.75" customHeight="1" s="1"/>
+    <row r="569" ht="15.75" customHeight="1" s="1"/>
+    <row r="570" ht="15.75" customHeight="1" s="1"/>
+    <row r="571" ht="15.75" customHeight="1" s="1"/>
+    <row r="572" ht="15.75" customHeight="1" s="1"/>
+    <row r="573" ht="15.75" customHeight="1" s="1"/>
+    <row r="574" ht="15.75" customHeight="1" s="1"/>
+    <row r="575" ht="15.75" customHeight="1" s="1"/>
+    <row r="576" ht="15.75" customHeight="1" s="1"/>
+    <row r="577" ht="15.75" customHeight="1" s="1"/>
+    <row r="578" ht="15.75" customHeight="1" s="1"/>
+    <row r="579" ht="15.75" customHeight="1" s="1"/>
+    <row r="580" ht="15.75" customHeight="1" s="1"/>
+    <row r="581" ht="15.75" customHeight="1" s="1"/>
+    <row r="582" ht="15.75" customHeight="1" s="1"/>
+    <row r="583" ht="15.75" customHeight="1" s="1"/>
+    <row r="584" ht="15.75" customHeight="1" s="1"/>
+    <row r="585" ht="15.75" customHeight="1" s="1"/>
+    <row r="586" ht="15.75" customHeight="1" s="1"/>
+    <row r="587" ht="15.75" customHeight="1" s="1"/>
+    <row r="588" ht="15.75" customHeight="1" s="1"/>
+    <row r="589" ht="15.75" customHeight="1" s="1"/>
+    <row r="590" ht="15.75" customHeight="1" s="1"/>
+    <row r="591" ht="15.75" customHeight="1" s="1"/>
+    <row r="592" ht="15.75" customHeight="1" s="1"/>
+    <row r="593" ht="15.75" customHeight="1" s="1"/>
+    <row r="594" ht="15.75" customHeight="1" s="1"/>
+    <row r="595" ht="15.75" customHeight="1" s="1"/>
+    <row r="596" ht="15.75" customHeight="1" s="1"/>
+    <row r="597" ht="15.75" customHeight="1" s="1"/>
+    <row r="598" ht="15.75" customHeight="1" s="1"/>
+    <row r="599" ht="15.75" customHeight="1" s="1"/>
+    <row r="600" ht="15.75" customHeight="1" s="1"/>
+    <row r="601" ht="15.75" customHeight="1" s="1"/>
+    <row r="602" ht="15.75" customHeight="1" s="1"/>
+    <row r="603" ht="15.75" customHeight="1" s="1"/>
+    <row r="604" ht="15.75" customHeight="1" s="1"/>
+    <row r="605" ht="15.75" customHeight="1" s="1"/>
+    <row r="606" ht="15.75" customHeight="1" s="1"/>
+    <row r="607" ht="15.75" customHeight="1" s="1"/>
+    <row r="608" ht="15.75" customHeight="1" s="1"/>
+    <row r="609" ht="15.75" customHeight="1" s="1"/>
+    <row r="610" ht="15.75" customHeight="1" s="1"/>
+    <row r="611" ht="15.75" customHeight="1" s="1"/>
+    <row r="612" ht="15.75" customHeight="1" s="1"/>
+    <row r="613" ht="15.75" customHeight="1" s="1"/>
+    <row r="614" ht="15.75" customHeight="1" s="1"/>
+    <row r="615" ht="15.75" customHeight="1" s="1"/>
+    <row r="616" ht="15.75" customHeight="1" s="1"/>
+    <row r="617" ht="15.75" customHeight="1" s="1"/>
+    <row r="618" ht="15.75" customHeight="1" s="1"/>
+    <row r="619" ht="15.75" customHeight="1" s="1"/>
+    <row r="620" ht="15.75" customHeight="1" s="1"/>
+    <row r="621" ht="15.75" customHeight="1" s="1"/>
+    <row r="622" ht="15.75" customHeight="1" s="1"/>
+    <row r="623" ht="15.75" customHeight="1" s="1"/>
+    <row r="624" ht="15.75" customHeight="1" s="1"/>
+    <row r="625" ht="15.75" customHeight="1" s="1"/>
+    <row r="626" ht="15.75" customHeight="1" s="1"/>
+    <row r="627" ht="15.75" customHeight="1" s="1"/>
+    <row r="628" ht="15.75" customHeight="1" s="1"/>
+    <row r="629" ht="15.75" customHeight="1" s="1"/>
+    <row r="630" ht="15.75" customHeight="1" s="1"/>
+    <row r="631" ht="15.75" customHeight="1" s="1"/>
+    <row r="632" ht="15.75" customHeight="1" s="1"/>
+    <row r="633" ht="15.75" customHeight="1" s="1"/>
+    <row r="634" ht="15.75" customHeight="1" s="1"/>
+    <row r="635" ht="15.75" customHeight="1" s="1"/>
+    <row r="636" ht="15.75" customHeight="1" s="1"/>
+    <row r="637" ht="15.75" customHeight="1" s="1"/>
+    <row r="638" ht="15.75" customHeight="1" s="1"/>
+    <row r="639" ht="15.75" customHeight="1" s="1"/>
+    <row r="640" ht="15.75" customHeight="1" s="1"/>
+    <row r="641" ht="15.75" customHeight="1" s="1"/>
+    <row r="642" ht="15.75" customHeight="1" s="1"/>
+    <row r="643" ht="15.75" customHeight="1" s="1"/>
+    <row r="644" ht="15.75" customHeight="1" s="1"/>
+    <row r="645" ht="15.75" customHeight="1" s="1"/>
+    <row r="646" ht="15.75" customHeight="1" s="1"/>
+    <row r="647" ht="15.75" customHeight="1" s="1"/>
+    <row r="648" ht="15.75" customHeight="1" s="1"/>
+    <row r="649" ht="15.75" customHeight="1" s="1"/>
+    <row r="650" ht="15.75" customHeight="1" s="1"/>
+    <row r="651" ht="15.75" customHeight="1" s="1"/>
+    <row r="652" ht="15.75" customHeight="1" s="1"/>
+    <row r="653" ht="15.75" customHeight="1" s="1"/>
+    <row r="654" ht="15.75" customHeight="1" s="1"/>
+    <row r="655" ht="15.75" customHeight="1" s="1"/>
+    <row r="656" ht="15.75" customHeight="1" s="1"/>
+    <row r="657" ht="15.75" customHeight="1" s="1"/>
+    <row r="658" ht="15.75" customHeight="1" s="1"/>
+    <row r="659" ht="15.75" customHeight="1" s="1"/>
+    <row r="660" ht="15.75" customHeight="1" s="1"/>
+    <row r="661" ht="15.75" customHeight="1" s="1"/>
+    <row r="662" ht="15.75" customHeight="1" s="1"/>
+    <row r="663" ht="15.75" customHeight="1" s="1"/>
+    <row r="664" ht="15.75" customHeight="1" s="1"/>
+    <row r="665" ht="15.75" customHeight="1" s="1"/>
+    <row r="666" ht="15.75" customHeight="1" s="1"/>
+    <row r="667" ht="15.75" customHeight="1" s="1"/>
+    <row r="668" ht="15.75" customHeight="1" s="1"/>
+    <row r="669" ht="15.75" customHeight="1" s="1"/>
+    <row r="670" ht="15.75" customHeight="1" s="1"/>
+    <row r="671" ht="15.75" customHeight="1" s="1"/>
+    <row r="672" ht="15.75" customHeight="1" s="1"/>
+    <row r="673" ht="15.75" customHeight="1" s="1"/>
+    <row r="674" ht="15.75" customHeight="1" s="1"/>
+    <row r="675" ht="15.75" customHeight="1" s="1"/>
+    <row r="676" ht="15.75" customHeight="1" s="1"/>
+    <row r="677" ht="15.75" customHeight="1" s="1"/>
+    <row r="678" ht="15.75" customHeight="1" s="1"/>
+    <row r="679" ht="15.75" customHeight="1" s="1"/>
+    <row r="680" ht="15.75" customHeight="1" s="1"/>
+    <row r="681" ht="15.75" customHeight="1" s="1"/>
+    <row r="682" ht="15.75" customHeight="1" s="1"/>
+    <row r="683" ht="15.75" customHeight="1" s="1"/>
+    <row r="684" ht="15.75" customHeight="1" s="1"/>
+    <row r="685" ht="15.75" customHeight="1" s="1"/>
+    <row r="686" ht="15.75" customHeight="1" s="1"/>
+    <row r="687" ht="15.75" customHeight="1" s="1"/>
+    <row r="688" ht="15.75" customHeight="1" s="1"/>
+    <row r="689" ht="15.75" customHeight="1" s="1"/>
+    <row r="690" ht="15.75" customHeight="1" s="1"/>
+    <row r="691" ht="15.75" customHeight="1" s="1"/>
+    <row r="692" ht="15.75" customHeight="1" s="1"/>
+    <row r="693" ht="15.75" customHeight="1" s="1"/>
+    <row r="694" ht="15.75" customHeight="1" s="1"/>
+    <row r="695" ht="15.75" customHeight="1" s="1"/>
+    <row r="696" ht="15.75" customHeight="1" s="1"/>
+    <row r="697" ht="15.75" customHeight="1" s="1"/>
+    <row r="698" ht="15.75" customHeight="1" s="1"/>
+    <row r="699" ht="15.75" customHeight="1" s="1"/>
+    <row r="700" ht="15.75" customHeight="1" s="1"/>
+    <row r="701" ht="15.75" customHeight="1" s="1"/>
+    <row r="702" ht="15.75" customHeight="1" s="1"/>
+    <row r="703" ht="15.75" customHeight="1" s="1"/>
+    <row r="704" ht="15.75" customHeight="1" s="1"/>
+    <row r="705" ht="15.75" customHeight="1" s="1"/>
+    <row r="706" ht="15.75" customHeight="1" s="1"/>
+    <row r="707" ht="15.75" customHeight="1" s="1"/>
+    <row r="708" ht="15.75" customHeight="1" s="1"/>
+    <row r="709" ht="15.75" customHeight="1" s="1"/>
+    <row r="710" ht="15.75" customHeight="1" s="1"/>
+    <row r="711" ht="15.75" customHeight="1" s="1"/>
+    <row r="712" ht="15.75" customHeight="1" s="1"/>
+    <row r="713" ht="15.75" customHeight="1" s="1"/>
+    <row r="714" ht="15.75" customHeight="1" s="1"/>
+    <row r="715" ht="15.75" customHeight="1" s="1"/>
+    <row r="716" ht="15.75" customHeight="1" s="1"/>
+    <row r="717" ht="15.75" customHeight="1" s="1"/>
+    <row r="718" ht="15.75" customHeight="1" s="1"/>
+    <row r="719" ht="15.75" customHeight="1" s="1"/>
+    <row r="720" ht="15.75" customHeight="1" s="1"/>
+    <row r="721" ht="15.75" customHeight="1" s="1"/>
+    <row r="722" ht="15.75" customHeight="1" s="1"/>
+    <row r="723" ht="15.75" customHeight="1" s="1"/>
+    <row r="724" ht="15.75" customHeight="1" s="1"/>
+    <row r="725" ht="15.75" customHeight="1" s="1"/>
+    <row r="726" ht="15.75" customHeight="1" s="1"/>
+    <row r="727" ht="15.75" customHeight="1" s="1"/>
+    <row r="728" ht="15.75" customHeight="1" s="1"/>
+    <row r="729" ht="15.75" customHeight="1" s="1"/>
+    <row r="730" ht="15.75" customHeight="1" s="1"/>
+    <row r="731" ht="15.75" customHeight="1" s="1"/>
+    <row r="732" ht="15.75" customHeight="1" s="1"/>
+    <row r="733" ht="15.75" customHeight="1" s="1"/>
+    <row r="734" ht="15.75" customHeight="1" s="1"/>
+    <row r="735" ht="15.75" customHeight="1" s="1"/>
+    <row r="736" ht="15.75" customHeight="1" s="1"/>
+    <row r="737" ht="15.75" customHeight="1" s="1"/>
+    <row r="738" ht="15.75" customHeight="1" s="1"/>
+    <row r="739" ht="15.75" customHeight="1" s="1"/>
+    <row r="740" ht="15.75" customHeight="1" s="1"/>
+    <row r="741" ht="15.75" customHeight="1" s="1"/>
+    <row r="742" ht="15.75" customHeight="1" s="1"/>
+    <row r="743" ht="15.75" customHeight="1" s="1"/>
+    <row r="744" ht="15.75" customHeight="1" s="1"/>
+    <row r="745" ht="15.75" customHeight="1" s="1"/>
+    <row r="746" ht="15.75" customHeight="1" s="1"/>
+    <row r="747" ht="15.75" customHeight="1" s="1"/>
+    <row r="748" ht="15.75" customHeight="1" s="1"/>
+    <row r="749" ht="15.75" customHeight="1" s="1"/>
+    <row r="750" ht="15.75" customHeight="1" s="1"/>
+    <row r="751" ht="15.75" customHeight="1" s="1"/>
+    <row r="752" ht="15.75" customHeight="1" s="1"/>
+    <row r="753" ht="15.75" customHeight="1" s="1"/>
+    <row r="754" ht="15.75" customHeight="1" s="1"/>
+    <row r="755" ht="15.75" customHeight="1" s="1"/>
+    <row r="756" ht="15.75" customHeight="1" s="1"/>
+    <row r="757" ht="15.75" customHeight="1" s="1"/>
+    <row r="758" ht="15.75" customHeight="1" s="1"/>
+    <row r="759" ht="15.75" customHeight="1" s="1"/>
+    <row r="760" ht="15.75" customHeight="1" s="1"/>
+    <row r="761" ht="15.75" customHeight="1" s="1"/>
+    <row r="762" ht="15.75" customHeight="1" s="1"/>
+    <row r="763" ht="15.75" customHeight="1" s="1"/>
+    <row r="764" ht="15.75" customHeight="1" s="1"/>
+    <row r="765" ht="15.75" customHeight="1" s="1"/>
+    <row r="766" ht="15.75" customHeight="1" s="1"/>
+    <row r="767" ht="15.75" customHeight="1" s="1"/>
+    <row r="768" ht="15.75" customHeight="1" s="1"/>
+    <row r="769" ht="15.75" customHeight="1" s="1"/>
+    <row r="770" ht="15.75" customHeight="1" s="1"/>
+    <row r="771" ht="15.75" customHeight="1" s="1"/>
+    <row r="772" ht="15.75" customHeight="1" s="1"/>
+    <row r="773" ht="15.75" customHeight="1" s="1"/>
+    <row r="774" ht="15.75" customHeight="1" s="1"/>
+    <row r="775" ht="15.75" customHeight="1" s="1"/>
+    <row r="776" ht="15.75" customHeight="1" s="1"/>
+    <row r="777" ht="15.75" customHeight="1" s="1"/>
+    <row r="778" ht="15.75" customHeight="1" s="1"/>
+    <row r="779" ht="15.75" customHeight="1" s="1"/>
+    <row r="780" ht="15.75" customHeight="1" s="1"/>
+    <row r="781" ht="15.75" customHeight="1" s="1"/>
+    <row r="782" ht="15.75" customHeight="1" s="1"/>
+    <row r="783" ht="15.75" customHeight="1" s="1"/>
+    <row r="784" ht="15.75" customHeight="1" s="1"/>
+    <row r="785" ht="15.75" customHeight="1" s="1"/>
+    <row r="786" ht="15.75" customHeight="1" s="1"/>
+    <row r="787" ht="15.75" customHeight="1" s="1"/>
+    <row r="788" ht="15.75" customHeight="1" s="1"/>
+    <row r="789" ht="15.75" customHeight="1" s="1"/>
+    <row r="790" ht="15.75" customHeight="1" s="1"/>
+    <row r="791" ht="15.75" customHeight="1" s="1"/>
+    <row r="792" ht="15.75" customHeight="1" s="1"/>
+    <row r="793" ht="15.75" customHeight="1" s="1"/>
+    <row r="794" ht="15.75" customHeight="1" s="1"/>
+    <row r="795" ht="15.75" customHeight="1" s="1"/>
+    <row r="796" ht="15.75" customHeight="1" s="1"/>
+    <row r="797" ht="15.75" customHeight="1" s="1"/>
+    <row r="798" ht="15.75" customHeight="1" s="1"/>
+    <row r="799" ht="15.75" customHeight="1" s="1"/>
+    <row r="800" ht="15.75" customHeight="1" s="1"/>
+    <row r="801" ht="15.75" customHeight="1" s="1"/>
+    <row r="802" ht="15.75" customHeight="1" s="1"/>
+    <row r="803" ht="15.75" customHeight="1" s="1"/>
+    <row r="804" ht="15.75" customHeight="1" s="1"/>
+    <row r="805" ht="15.75" customHeight="1" s="1"/>
+    <row r="806" ht="15.75" customHeight="1" s="1"/>
+    <row r="807" ht="15.75" customHeight="1" s="1"/>
+    <row r="808" ht="15.75" customHeight="1" s="1"/>
+    <row r="809" ht="15.75" customHeight="1" s="1"/>
+    <row r="810" ht="15.75" customHeight="1" s="1"/>
+    <row r="811" ht="15.75" customHeight="1" s="1"/>
+    <row r="812" ht="15.75" customHeight="1" s="1"/>
+    <row r="813" ht="15.75" customHeight="1" s="1"/>
+    <row r="814" ht="15.75" customHeight="1" s="1"/>
+    <row r="815" ht="15.75" customHeight="1" s="1"/>
+    <row r="816" ht="15.75" customHeight="1" s="1"/>
+    <row r="817" ht="15.75" customHeight="1" s="1"/>
+    <row r="818" ht="15.75" customHeight="1" s="1"/>
+    <row r="819" ht="15.75" customHeight="1" s="1"/>
+    <row r="820" ht="15.75" customHeight="1" s="1"/>
+    <row r="821" ht="15.75" customHeight="1" s="1"/>
+    <row r="822" ht="15.75" customHeight="1" s="1"/>
+    <row r="823" ht="15.75" customHeight="1" s="1"/>
+    <row r="824" ht="15.75" customHeight="1" s="1"/>
+    <row r="825" ht="15.75" customHeight="1" s="1"/>
+    <row r="826" ht="15.75" customHeight="1" s="1"/>
+    <row r="827" ht="15.75" customHeight="1" s="1"/>
+    <row r="828" ht="15.75" customHeight="1" s="1"/>
+    <row r="829" ht="15.75" customHeight="1" s="1"/>
+    <row r="830" ht="15.75" customHeight="1" s="1"/>
+    <row r="831" ht="15.75" customHeight="1" s="1"/>
+    <row r="832" ht="15.75" customHeight="1" s="1"/>
+    <row r="833" ht="15.75" customHeight="1" s="1"/>
+    <row r="834" ht="15.75" customHeight="1" s="1"/>
+    <row r="835" ht="15.75" customHeight="1" s="1"/>
+    <row r="836" ht="15.75" customHeight="1" s="1"/>
+    <row r="837" ht="15.75" customHeight="1" s="1"/>
+    <row r="838" ht="15.75" customHeight="1" s="1"/>
+    <row r="839" ht="15.75" customHeight="1" s="1"/>
+    <row r="840" ht="15.75" customHeight="1" s="1"/>
+    <row r="841" ht="15.75" customHeight="1" s="1"/>
+    <row r="842" ht="15.75" customHeight="1" s="1"/>
+    <row r="843" ht="15.75" customHeight="1" s="1"/>
+    <row r="844" ht="15.75" customHeight="1" s="1"/>
+    <row r="845" ht="15.75" customHeight="1" s="1"/>
+    <row r="846" ht="15.75" customHeight="1" s="1"/>
+    <row r="847" ht="15.75" customHeight="1" s="1"/>
+    <row r="848" ht="15.75" customHeight="1" s="1"/>
+    <row r="849" ht="15.75" customHeight="1" s="1"/>
+    <row r="850" ht="15.75" customHeight="1" s="1"/>
+    <row r="851" ht="15.75" customHeight="1" s="1"/>
+    <row r="852" ht="15.75" customHeight="1" s="1"/>
+    <row r="853" ht="15.75" customHeight="1" s="1"/>
+    <row r="854" ht="15.75" customHeight="1" s="1"/>
+    <row r="855" ht="15.75" customHeight="1" s="1"/>
+    <row r="856" ht="15.75" customHeight="1" s="1"/>
+    <row r="857" ht="15.75" customHeight="1" s="1"/>
+    <row r="858" ht="15.75" customHeight="1" s="1"/>
+    <row r="859" ht="15.75" customHeight="1" s="1"/>
+    <row r="860" ht="15.75" customHeight="1" s="1"/>
+    <row r="861" ht="15.75" customHeight="1" s="1"/>
+    <row r="862" ht="15.75" customHeight="1" s="1"/>
+    <row r="863" ht="15.75" customHeight="1" s="1"/>
+    <row r="864" ht="15.75" customHeight="1" s="1"/>
+    <row r="865" ht="15.75" customHeight="1" s="1"/>
+    <row r="866" ht="15.75" customHeight="1" s="1"/>
+    <row r="867" ht="15.75" customHeight="1" s="1"/>
+    <row r="868" ht="15.75" customHeight="1" s="1"/>
+    <row r="869" ht="15.75" customHeight="1" s="1"/>
+    <row r="870" ht="15.75" customHeight="1" s="1"/>
+    <row r="871" ht="15.75" customHeight="1" s="1"/>
+    <row r="872" ht="15.75" customHeight="1" s="1"/>
+    <row r="873" ht="15.75" customHeight="1" s="1"/>
+    <row r="874" ht="15.75" customHeight="1" s="1"/>
+    <row r="875" ht="15.75" customHeight="1" s="1"/>
+    <row r="876" ht="15.75" customHeight="1" s="1"/>
+    <row r="877" ht="15.75" customHeight="1" s="1"/>
+    <row r="878" ht="15.75" customHeight="1" s="1"/>
+    <row r="879" ht="15.75" customHeight="1" s="1"/>
+    <row r="880" ht="15.75" customHeight="1" s="1"/>
+    <row r="881" ht="15.75" customHeight="1" s="1"/>
+    <row r="882" ht="15.75" customHeight="1" s="1"/>
+    <row r="883" ht="15.75" customHeight="1" s="1"/>
+    <row r="884" ht="15.75" customHeight="1" s="1"/>
+    <row r="885" ht="15.75" customHeight="1" s="1"/>
+    <row r="886" ht="15.75" customHeight="1" s="1"/>
+    <row r="887" ht="15.75" customHeight="1" s="1"/>
+    <row r="888" ht="15.75" customHeight="1" s="1"/>
+    <row r="889" ht="15.75" customHeight="1" s="1"/>
+    <row r="890" ht="15.75" customHeight="1" s="1"/>
+    <row r="891" ht="15.75" customHeight="1" s="1"/>
+    <row r="892" ht="15.75" customHeight="1" s="1"/>
+    <row r="893" ht="15.75" customHeight="1" s="1"/>
+    <row r="894" ht="15.75" customHeight="1" s="1"/>
+    <row r="895" ht="15.75" customHeight="1" s="1"/>
+    <row r="896" ht="15.75" customHeight="1" s="1"/>
+    <row r="897" ht="15.75" customHeight="1" s="1"/>
+    <row r="898" ht="15.75" customHeight="1" s="1"/>
+    <row r="899" ht="15.75" customHeight="1" s="1"/>
+    <row r="900" ht="15.75" customHeight="1" s="1"/>
+    <row r="901" ht="15.75" customHeight="1" s="1"/>
+    <row r="902" ht="15.75" customHeight="1" s="1"/>
+    <row r="903" ht="15.75" customHeight="1" s="1"/>
+    <row r="904" ht="15.75" customHeight="1" s="1"/>
+    <row r="905" ht="15.75" customHeight="1" s="1"/>
+    <row r="906" ht="15.75" customHeight="1" s="1"/>
+    <row r="907" ht="15.75" customHeight="1" s="1"/>
+    <row r="908" ht="15.75" customHeight="1" s="1"/>
+    <row r="909" ht="15.75" customHeight="1" s="1"/>
+    <row r="910" ht="15.75" customHeight="1" s="1"/>
+    <row r="911" ht="15.75" customHeight="1" s="1"/>
+    <row r="912" ht="15.75" customHeight="1" s="1"/>
+    <row r="913" ht="15.75" customHeight="1" s="1"/>
+    <row r="914" ht="15.75" customHeight="1" s="1"/>
+    <row r="915" ht="15.75" customHeight="1" s="1"/>
+    <row r="916" ht="15.75" customHeight="1" s="1"/>
+    <row r="917" ht="15.75" customHeight="1" s="1"/>
+    <row r="918" ht="15.75" customHeight="1" s="1"/>
+    <row r="919" ht="15.75" customHeight="1" s="1"/>
+    <row r="920" ht="15.75" customHeight="1" s="1"/>
+    <row r="921" ht="15.75" customHeight="1" s="1"/>
+    <row r="922" ht="15.75" customHeight="1" s="1"/>
+    <row r="923" ht="15.75" customHeight="1" s="1"/>
+    <row r="924" ht="15.75" customHeight="1" s="1"/>
+    <row r="925" ht="15.75" customHeight="1" s="1"/>
+    <row r="926" ht="15.75" customHeight="1" s="1"/>
+    <row r="927" ht="15.75" customHeight="1" s="1"/>
+    <row r="928" ht="15.75" customHeight="1" s="1"/>
+    <row r="929" ht="15.75" customHeight="1" s="1"/>
+    <row r="930" ht="15.75" customHeight="1" s="1"/>
+    <row r="931" ht="15.75" customHeight="1" s="1"/>
+    <row r="932" ht="15.75" customHeight="1" s="1"/>
+    <row r="933" ht="15.75" customHeight="1" s="1"/>
+    <row r="934" ht="15.75" customHeight="1" s="1"/>
+    <row r="935" ht="15.75" customHeight="1" s="1"/>
+    <row r="936" ht="15.75" customHeight="1" s="1"/>
+    <row r="937" ht="15.75" customHeight="1" s="1"/>
+    <row r="938" ht="15.75" customHeight="1" s="1"/>
+    <row r="939" ht="15.75" customHeight="1" s="1"/>
+    <row r="940" ht="15.75" customHeight="1" s="1"/>
+    <row r="941" ht="15.75" customHeight="1" s="1"/>
+    <row r="942" ht="15.75" customHeight="1" s="1"/>
+    <row r="943" ht="15.75" customHeight="1" s="1"/>
+    <row r="944" ht="15.75" customHeight="1" s="1"/>
+    <row r="945" ht="15.75" customHeight="1" s="1"/>
+    <row r="946" ht="15.75" customHeight="1" s="1"/>
+    <row r="947" ht="15.75" customHeight="1" s="1"/>
+    <row r="948" ht="15.75" customHeight="1" s="1"/>
+    <row r="949" ht="15.75" customHeight="1" s="1"/>
+    <row r="950" ht="15.75" customHeight="1" s="1"/>
+    <row r="951" ht="15.75" customHeight="1" s="1"/>
+    <row r="952" ht="15.75" customHeight="1" s="1"/>
+    <row r="953" ht="15.75" customHeight="1" s="1"/>
+    <row r="954" ht="15.75" customHeight="1" s="1"/>
+    <row r="955" ht="15.75" customHeight="1" s="1"/>
+    <row r="956" ht="15.75" customHeight="1" s="1"/>
+    <row r="957" ht="15.75" customHeight="1" s="1"/>
+    <row r="958" ht="15.75" customHeight="1" s="1"/>
+    <row r="959" ht="15.75" customHeight="1" s="1"/>
+    <row r="960" ht="15.75" customHeight="1" s="1"/>
+    <row r="961" ht="15.75" customHeight="1" s="1"/>
+    <row r="962" ht="15.75" customHeight="1" s="1"/>
+    <row r="963" ht="15.75" customHeight="1" s="1"/>
+    <row r="964" ht="15.75" customHeight="1" s="1"/>
+    <row r="965" ht="15.75" customHeight="1" s="1"/>
+    <row r="966" ht="15.75" customHeight="1" s="1"/>
+    <row r="967" ht="15.75" customHeight="1" s="1"/>
+    <row r="968" ht="15.75" customHeight="1" s="1"/>
+    <row r="969" ht="15.75" customHeight="1" s="1"/>
+    <row r="970" ht="15.75" customHeight="1" s="1"/>
+    <row r="971" ht="15.75" customHeight="1" s="1"/>
+    <row r="972" ht="15.75" customHeight="1" s="1"/>
+    <row r="973" ht="15.75" customHeight="1" s="1"/>
+    <row r="974" ht="15.75" customHeight="1" s="1"/>
+    <row r="975" ht="15.75" customHeight="1" s="1"/>
+    <row r="976" ht="15.75" customHeight="1" s="1"/>
+    <row r="977" ht="15.75" customHeight="1" s="1"/>
+    <row r="978" ht="15.75" customHeight="1" s="1"/>
+    <row r="979" ht="15.75" customHeight="1" s="1"/>
+    <row r="980" ht="15.75" customHeight="1" s="1"/>
+    <row r="981" ht="15.75" customHeight="1" s="1"/>
+    <row r="982" ht="15.75" customHeight="1" s="1"/>
+    <row r="983" ht="15.75" customHeight="1" s="1"/>
+    <row r="984" ht="15.75" customHeight="1" s="1"/>
+    <row r="985" ht="15.75" customHeight="1" s="1"/>
+    <row r="986" ht="15.75" customHeight="1" s="1"/>
+    <row r="987" ht="15.75" customHeight="1" s="1"/>
+    <row r="988" ht="15.75" customHeight="1" s="1"/>
+    <row r="989" ht="15.75" customHeight="1" s="1"/>
+    <row r="990" ht="15.75" customHeight="1" s="1"/>
+    <row r="991" ht="15.75" customHeight="1" s="1"/>
+    <row r="992" ht="15.75" customHeight="1" s="1"/>
+    <row r="993" ht="15.75" customHeight="1" s="1"/>
+    <row r="994" ht="15.75" customHeight="1" s="1"/>
+    <row r="995" ht="15.75" customHeight="1" s="1"/>
+    <row r="996" ht="15.75" customHeight="1" s="1"/>
+    <row r="997" ht="15.75" customHeight="1" s="1"/>
+    <row r="998" ht="15.75" customHeight="1" s="1"/>
+    <row r="999" ht="15.75" customHeight="1" s="1"/>
+    <row r="1000" ht="15.75" customHeight="1" s="1"/>
+  </sheetData>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" useFirstPageNumber="0" pageOrder="downThenOver" usePrinterDefaults="1" blackAndWhite="0" draft="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>

</xml_diff>

<commit_message>
docs: ajustar espaciado y altura de celdas en el excel para mejor legibilidad
</commit_message>
<xml_diff>
--- a/docs/entregables/PRACTICA EMPRESARIAL/GRUPO2_FIREFOX_MATRICES_COMPLETAS.xlsx
+++ b/docs/entregables/PRACTICA EMPRESARIAL/GRUPO2_FIREFOX_MATRICES_COMPLETAS.xlsx
@@ -1961,11 +1961,11 @@
   <dimension ref="A1:E199"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="36" customWidth="1" style="1" min="1" max="1"/>
-    <col width="26" customWidth="1" style="1" min="2" max="2"/>
-    <col width="44" customWidth="1" style="1" min="3" max="3"/>
-    <col width="34" customWidth="1" style="1" min="4" max="4"/>
-    <col width="28" customWidth="1" style="1" min="5" max="5"/>
+    <col width="35" customWidth="1" style="1" min="1" max="1"/>
+    <col width="25" customWidth="1" style="1" min="2" max="2"/>
+    <col width="45" customWidth="1" style="1" min="3" max="3"/>
+    <col width="35" customWidth="1" style="1" min="4" max="4"/>
+    <col width="15" customWidth="1" style="1" min="5" max="5"/>
     <col width="8.710000000000001" customWidth="1" style="1" min="6" max="26"/>
   </cols>
   <sheetData>
@@ -2032,7 +2032,7 @@
       <c r="D7" s="18" t="n"/>
       <c r="E7" s="18" t="n"/>
     </row>
-    <row r="8" ht="49.5" customHeight="1" s="1">
+    <row r="8" ht="45" customHeight="1" s="1">
       <c r="A8" s="29" t="inlineStr">
         <is>
           <t>Archivo de Documentación Global (README.md)</t>
@@ -2059,7 +2059,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="49.5" customHeight="1" s="1">
+    <row r="9" ht="45" customHeight="1" s="1">
       <c r="A9" s="29" t="inlineStr">
         <is>
           <t>Integración Continua CI/CD (GitHub Actions)</t>
@@ -2086,7 +2086,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="49.5" customHeight="1" s="1">
+    <row r="10" ht="45" customHeight="1" s="1">
       <c r="A10" s="29" t="inlineStr">
         <is>
           <t>Automatización de Comandos (Makefile)</t>
@@ -2113,7 +2113,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="49.5" customHeight="1" s="1">
+    <row r="11" ht="45" customHeight="1" s="1">
       <c r="A11" s="29" t="inlineStr">
         <is>
           <t>Configuración Centralizada (Pydantic Settings)</t>
@@ -2140,7 +2140,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="49.5" customHeight="1" s="1">
+    <row r="12" ht="45" customHeight="1" s="1">
       <c r="A12" s="29" t="inlineStr">
         <is>
           <t>Script Seeder de Datos de Prueba</t>
@@ -2167,7 +2167,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="49.5" customHeight="1" s="1">
+    <row r="13" ht="45" customHeight="1" s="1">
       <c r="A13" s="29" t="inlineStr">
         <is>
           <t>Esquema Inicial de Base de Datos</t>
@@ -2194,7 +2194,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="30.75" customHeight="1" s="1">
+    <row r="14" ht="45" customHeight="1" s="1">
       <c r="A14" s="29" t="inlineStr">
         <is>
           <t>Diagrama de Entidad-Relación (DER)</t>
@@ -2221,7 +2221,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="39.75" customHeight="1" s="1">
+    <row r="15" ht="45" customHeight="1" s="1">
       <c r="A15" s="32" t="inlineStr">
         <is>
           <t>Diagrama de Secuencia: Reservas y Bloqueo</t>
@@ -2248,7 +2248,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="51.75" customHeight="1" s="1">
+    <row r="16" ht="45" customHeight="1" s="1">
       <c r="A16" s="29" t="inlineStr">
         <is>
           <t>Diagrama de Secuencia: Check-in</t>
@@ -2275,7 +2275,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="51.75" customHeight="1" s="1">
+    <row r="17" ht="45" customHeight="1" s="1">
       <c r="A17" s="29" t="inlineStr">
         <is>
           <t>Diagrama de Secuencia: Cancelación</t>
@@ -2302,7 +2302,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="51.75" customHeight="1" s="1">
+    <row r="18" ht="45" customHeight="1" s="1">
       <c r="A18" s="29" t="inlineStr">
         <is>
           <t>Modelos de Base de Datos (SQLAlchemy)</t>
@@ -2329,7 +2329,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="51.75" customHeight="1" s="1">
+    <row r="19" ht="45" customHeight="1" s="1">
       <c r="A19" s="29" t="inlineStr">
         <is>
           <t>Validadores de Datos y Especificación OpenAPI</t>
@@ -2356,7 +2356,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="51.75" customHeight="1" s="1">
+    <row r="20" ht="45" customHeight="1" s="1">
       <c r="A20" s="29" t="inlineStr">
         <is>
           <t>Lógica de Negocio y Bloqueo Pesimista</t>
@@ -2383,7 +2383,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="51.75" customHeight="1" s="1">
+    <row r="21" ht="45" customHeight="1" s="1">
       <c r="A21" s="29" t="inlineStr">
         <is>
           <t>Endpoints Transaccionales REST</t>
@@ -2410,7 +2410,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="51.75" customHeight="1" s="1">
+    <row r="22" ht="45" customHeight="1" s="1">
       <c r="A22" s="29" t="inlineStr">
         <is>
           <t>Endpoints Administrativos</t>
@@ -2437,7 +2437,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="51.75" customHeight="1" s="1">
+    <row r="23" ht="45" customHeight="1" s="1">
       <c r="A23" s="29" t="inlineStr">
         <is>
           <t>Manejo de Sesiones DB (Dependency Injection)</t>
@@ -2464,7 +2464,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="51.75" customHeight="1" s="1">
+    <row r="24" ht="45" customHeight="1" s="1">
       <c r="A24" s="29" t="inlineStr">
         <is>
           <t>Test Automatizado de Concurrencia</t>
@@ -2491,7 +2491,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="51.75" customHeight="1" s="1">
+    <row r="25" ht="45" customHeight="1" s="1">
       <c r="A25" s="29" t="inlineStr">
         <is>
           <t>Test End-to-End (E2E) Viaje del Usuario</t>
@@ -2518,7 +2518,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="51.75" customHeight="1" s="1">
+    <row r="26" ht="45" customHeight="1" s="1">
       <c r="A26" s="29" t="inlineStr">
         <is>
           <t>Tests Unitarios de Modelos</t>
@@ -2545,7 +2545,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="51.75" customHeight="1" s="1">
+    <row r="27" ht="45" customHeight="1" s="1">
       <c r="A27" s="29" t="inlineStr">
         <is>
           <t>Configuración de Tests (Fixtures)</t>
@@ -2572,7 +2572,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="31.5" customHeight="1" s="1">
+    <row r="28" ht="45" customHeight="1" s="1">
       <c r="A28" s="33" t="inlineStr">
         <is>
           <t>Diagrama de Arquitectura de Sistemas (C4)</t>
@@ -2599,7 +2599,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="15.75" customHeight="1" s="1">
+    <row r="29" ht="45" customHeight="1" s="1">
       <c r="A29" s="31" t="inlineStr">
         <is>
           <t>Documento Técnico de Justificación CQRS</t>
@@ -2626,7 +2626,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="15.75" customHeight="1" s="1">
+    <row r="30" ht="45" customHeight="1" s="1">
       <c r="A30" s="31" t="inlineStr">
         <is>
           <t>Servicio Desacoplado de Disponibilidad</t>
@@ -2653,7 +2653,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="15.75" customHeight="1" s="1">
+    <row r="31" ht="45" customHeight="1" s="1">
       <c r="A31" s="31" t="inlineStr">
         <is>
           <t>Endpoints Optimizados de Búsqueda (API)</t>
@@ -2680,7 +2680,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="15.75" customHeight="1" s="1">
+    <row r="32" ht="45" customHeight="1" s="1">
       <c r="A32" s="31" t="inlineStr">
         <is>
           <t>Monitoreo de Salud del Sistema (Healthcheck)</t>
@@ -2707,7 +2707,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="15.75" customHeight="1" s="1">
+    <row r="33" ht="45" customHeight="1" s="1">
       <c r="A33" s="31" t="inlineStr">
         <is>
           <t>Dockerfile de Aplicación API</t>
@@ -2734,7 +2734,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="15.75" customHeight="1" s="1">
+    <row r="34" ht="45" customHeight="1" s="1">
       <c r="A34" s="31" t="inlineStr">
         <is>
           <t>Orquestación de Infraestructura (Docker Compose)</t>
@@ -2761,7 +2761,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="15.75" customHeight="1" s="1">
+    <row r="35" ht="45" customHeight="1" s="1">
       <c r="A35" s="31" t="inlineStr">
         <is>
           <t>Cliente y Configuración Caché (Valkey)</t>
@@ -2788,7 +2788,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="15.75" customHeight="1" s="1">
+    <row r="36" ht="45" customHeight="1" s="1">
       <c r="A36" s="31" t="inlineStr">
         <is>
           <t>Inyección de Caché en Disponibilidad</t>
@@ -2815,7 +2815,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="15.75" customHeight="1" s="1">
+    <row r="37" ht="45" customHeight="1" s="1">
       <c r="A37" s="31" t="inlineStr">
         <is>
           <t>Servidor Valkey en Infraestructura</t>
@@ -2842,7 +2842,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="15.75" customHeight="1" s="1">
+    <row r="38" ht="45" customHeight="1" s="1">
       <c r="A38" s="31" t="inlineStr">
         <is>
           <t>Políticas de Invalidación y TTL</t>
@@ -2869,7 +2869,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="15.75" customHeight="1" s="1">
+    <row r="39" ht="45" customHeight="1" s="1">
       <c r="A39" s="31" t="inlineStr">
         <is>
           <t>Pruebas de Resiliencia de Caché</t>
@@ -2896,7 +2896,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="15.75" customHeight="1" s="1">
+    <row r="40" ht="45" customHeight="1" s="1">
       <c r="A40" s="31" t="inlineStr">
         <is>
           <t>Documento Protocolo Pruebas de Estrés K6</t>
@@ -2923,7 +2923,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="15.75" customHeight="1" s="1">
+    <row r="41" ht="45" customHeight="1" s="1">
       <c r="A41" s="31" t="inlineStr">
         <is>
           <t>Guía de Generación de Logs de Auditoría</t>
@@ -2950,7 +2950,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="15.75" customHeight="1" s="1">
+    <row r="42" ht="45" customHeight="1" s="1">
       <c r="A42" s="31" t="inlineStr">
         <is>
           <t>Script de Carga Masiva Automatizada (K6)</t>
@@ -2977,7 +2977,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="15.75" customHeight="1" s="1">
+    <row r="43" ht="45" customHeight="1" s="1">
       <c r="A43" s="31" t="inlineStr">
         <is>
           <t>Plan Maestro de Ejecución BoA</t>
@@ -4910,15 +4910,15 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="33" customWidth="1" style="1" min="1" max="1"/>
-    <col width="26" customWidth="1" style="1" min="2" max="2"/>
-    <col width="30" customWidth="1" style="1" min="3" max="3"/>
-    <col width="38" customWidth="1" style="1" min="4" max="4"/>
-    <col width="22" customWidth="1" style="1" min="5" max="5"/>
-    <col width="16" customWidth="1" style="1" min="6" max="6"/>
+    <col width="35" customWidth="1" style="1" min="1" max="1"/>
+    <col width="35" customWidth="1" style="1" min="2" max="2"/>
+    <col width="35" customWidth="1" style="1" min="3" max="3"/>
+    <col width="35" customWidth="1" style="1" min="4" max="4"/>
+    <col width="15" customWidth="1" style="1" min="5" max="5"/>
+    <col width="15" customWidth="1" style="1" min="6" max="6"/>
     <col width="8.710000000000001" customWidth="1" style="1" min="7" max="26"/>
   </cols>
   <sheetData>
@@ -4978,7 +4978,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="99.75" customHeight="1" s="1">
+    <row r="6" ht="60" customHeight="1" s="1">
       <c r="A6" s="25" t="inlineStr">
         <is>
           <t>Sin acceso al código fuente, base de datos ni entorno de producción de BoA.</t>
@@ -5010,7 +5010,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="99.75" customHeight="1" s="1">
+    <row r="7" ht="60" customHeight="1" s="1">
       <c r="A7" s="25" t="inlineStr">
         <is>
           <t>Complejidad de orquestar múltiples servicios (Postgres, Valkey, API) localmente.</t>
@@ -5042,7 +5042,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="99.75" customHeight="1" s="1">
+    <row r="8" ht="60" customHeight="1" s="1">
       <c r="A8" s="27" t="inlineStr">
         <is>
           <t>Desacoplamiento complejo de operaciones de Lectura y Escritura (CQRS).</t>
@@ -5074,7 +5074,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="99.75" customHeight="1" s="1">
+    <row r="9" ht="60" customHeight="1" s="1">
       <c r="A9" s="27" t="inlineStr">
         <is>
           <t>Sin datos históricos de tráfico de campañas (Vuelos Azules).</t>
@@ -5106,7 +5106,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="99.75" customHeight="1" s="1">
+    <row r="10" ht="60" customHeight="1" s="1">
       <c r="A10" s="27" t="inlineStr">
         <is>
           <t>Riesgo de inconsistencia temporal entre Caché (Valkey) y Base de Datos (Postgres).</t>
@@ -5149,7 +5149,6 @@
     <row r="17"/>
     <row r="18"/>
     <row r="19"/>
-    <row r="20"/>
     <row r="21" ht="15.75" customHeight="1" s="1"/>
     <row r="22" ht="15.75" customHeight="1" s="1"/>
     <row r="23" ht="15.75" customHeight="1" s="1"/>

</xml_diff>

<commit_message>
docs: agregar 6 diagramas profesionales nuevos y documentarlos en matriz 2
</commit_message>
<xml_diff>
--- a/docs/entregables/PRACTICA EMPRESARIAL/GRUPO2_FIREFOX_MATRICES_COMPLETAS.xlsx
+++ b/docs/entregables/PRACTICA EMPRESARIAL/GRUPO2_FIREFOX_MATRICES_COMPLETAS.xlsx
@@ -3004,47 +3004,167 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="15.75" customHeight="1" s="1">
-      <c r="A44" s="35" t="inlineStr"/>
-      <c r="B44" s="35" t="inlineStr"/>
-      <c r="C44" s="35" t="inlineStr"/>
-      <c r="D44" s="35" t="inlineStr"/>
-      <c r="E44" s="35" t="inlineStr"/>
-    </row>
-    <row r="45" ht="15.75" customHeight="1" s="1">
-      <c r="A45" s="35" t="inlineStr"/>
-      <c r="B45" s="35" t="inlineStr"/>
-      <c r="C45" s="35" t="inlineStr"/>
-      <c r="D45" s="35" t="inlineStr"/>
-      <c r="E45" s="35" t="inlineStr"/>
-    </row>
-    <row r="46" ht="15.75" customHeight="1" s="1">
-      <c r="A46" s="35" t="inlineStr"/>
-      <c r="B46" s="35" t="inlineStr"/>
-      <c r="C46" s="35" t="inlineStr"/>
-      <c r="D46" s="35" t="inlineStr"/>
-      <c r="E46" s="35" t="inlineStr"/>
-    </row>
-    <row r="47" ht="15.75" customHeight="1" s="1">
-      <c r="A47" s="35" t="inlineStr"/>
-      <c r="B47" s="35" t="inlineStr"/>
-      <c r="C47" s="35" t="inlineStr"/>
-      <c r="D47" s="35" t="inlineStr"/>
-      <c r="E47" s="35" t="inlineStr"/>
-    </row>
-    <row r="48" ht="15.75" customHeight="1" s="1">
-      <c r="A48" s="35" t="inlineStr"/>
-      <c r="B48" s="35" t="inlineStr"/>
-      <c r="C48" s="35" t="inlineStr"/>
-      <c r="D48" s="35" t="inlineStr"/>
-      <c r="E48" s="35" t="inlineStr"/>
-    </row>
-    <row r="49" ht="15.75" customHeight="1" s="1">
-      <c r="A49" s="35" t="inlineStr"/>
-      <c r="B49" s="35" t="inlineStr"/>
-      <c r="C49" s="35" t="inlineStr"/>
-      <c r="D49" s="35" t="inlineStr"/>
-      <c r="E49" s="35" t="inlineStr"/>
+    <row r="44" ht="45" customHeight="1" s="1">
+      <c r="A44" s="31" t="inlineStr">
+        <is>
+          <t>Diagrama de Estados del Asiento (Máquina de Estados)</t>
+        </is>
+      </c>
+      <c r="B44" s="31" t="inlineStr">
+        <is>
+          <t>Obj. 1 - Bloqueo transaccional</t>
+        </is>
+      </c>
+      <c r="C44" s="31" t="inlineStr">
+        <is>
+          <t>Evolución lógica de un asiento desde LIBRE hasta ABORDADO o CANCELADO.</t>
+        </is>
+      </c>
+      <c r="D44" s="31" t="inlineStr">
+        <is>
+          <t>docs/diagramas/diagrama_estados_asiento.md</t>
+        </is>
+      </c>
+      <c r="E44" s="30" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="45" customHeight="1" s="1">
+      <c r="A45" s="31" t="inlineStr">
+        <is>
+          <t>Diagrama de Flujo: Sincronización CQRS</t>
+        </is>
+      </c>
+      <c r="B45" s="31" t="inlineStr">
+        <is>
+          <t>Obj. 2 - Validación de disponibilidad</t>
+        </is>
+      </c>
+      <c r="C45" s="31" t="inlineStr">
+        <is>
+          <t>Propagación de eventos de la Write API hacia la Read API.</t>
+        </is>
+      </c>
+      <c r="D45" s="31" t="inlineStr">
+        <is>
+          <t>docs/diagramas/diagrama_sincronizacion_cqrs.md</t>
+        </is>
+      </c>
+      <c r="E45" s="30" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="45" customHeight="1" s="1">
+      <c r="A46" s="31" t="inlineStr">
+        <is>
+          <t>Diagrama de Componentes de Backend</t>
+        </is>
+      </c>
+      <c r="B46" s="31" t="inlineStr">
+        <is>
+          <t>Obj. 2 - Validación de disponibilidad</t>
+        </is>
+      </c>
+      <c r="C46" s="31" t="inlineStr">
+        <is>
+          <t>Mapeo interno de routers, servicios y repositorios en FastAPI.</t>
+        </is>
+      </c>
+      <c r="D46" s="31" t="inlineStr">
+        <is>
+          <t>docs/diagramas/diagrama_componentes_backend.md</t>
+        </is>
+      </c>
+      <c r="E46" s="30" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="45" customHeight="1" s="1">
+      <c r="A47" s="31" t="inlineStr">
+        <is>
+          <t>Diagrama de Secuencia: Flujo Cache-Aside</t>
+        </is>
+      </c>
+      <c r="B47" s="31" t="inlineStr">
+        <is>
+          <t>Obj. 3 - Capa de caché</t>
+        </is>
+      </c>
+      <c r="C47" s="31" t="inlineStr">
+        <is>
+          <t>Decisión del sistema entre recuperar de RAM o calcular desde BD.</t>
+        </is>
+      </c>
+      <c r="D47" s="31" t="inlineStr">
+        <is>
+          <t>docs/diagramas/diagrama_flujo_cache.md</t>
+        </is>
+      </c>
+      <c r="E47" s="34" t="inlineStr">
+        <is>
+          <t>○ Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="45" customHeight="1" s="1">
+      <c r="A48" s="31" t="inlineStr">
+        <is>
+          <t>Diagrama de Topología: Entorno K6</t>
+        </is>
+      </c>
+      <c r="B48" s="31" t="inlineStr">
+        <is>
+          <t>Obj. 4 - Protocolo de estrés</t>
+        </is>
+      </c>
+      <c r="C48" s="31" t="inlineStr">
+        <is>
+          <t>Ubicación del Load Generator K6 y el clúster atacado.</t>
+        </is>
+      </c>
+      <c r="D48" s="31" t="inlineStr">
+        <is>
+          <t>docs/diagramas/diagrama_topologia_k6.md</t>
+        </is>
+      </c>
+      <c r="E48" s="34" t="inlineStr">
+        <is>
+          <t>○ Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="45" customHeight="1" s="1">
+      <c r="A49" s="31" t="inlineStr">
+        <is>
+          <t>Gráfico Perfil de Rampas de Estrés K6</t>
+        </is>
+      </c>
+      <c r="B49" s="31" t="inlineStr">
+        <is>
+          <t>Obj. 4 - Protocolo de estrés</t>
+        </is>
+      </c>
+      <c r="C49" s="31" t="inlineStr">
+        <is>
+          <t>Evolución de Usuarios Concurrentes (VUs) durante la prueba.</t>
+        </is>
+      </c>
+      <c r="D49" s="31" t="inlineStr">
+        <is>
+          <t>docs/diagramas/diagrama_rampas_estres.md</t>
+        </is>
+      </c>
+      <c r="E49" s="34" t="inlineStr">
+        <is>
+          <t>○ Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="1">
       <c r="A50" s="35" t="inlineStr"/>
@@ -4910,7 +5030,7 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="35" customWidth="1" style="1" min="1" max="1"/>
@@ -5141,14 +5261,6 @@
     <row r="11" ht="37.5" customHeight="1" s="1">
       <c r="A11" s="9" t="n"/>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
     <row r="21" ht="15.75" customHeight="1" s="1"/>
     <row r="22" ht="15.75" customHeight="1" s="1"/>
     <row r="23" ht="15.75" customHeight="1" s="1"/>

</xml_diff>

<commit_message>
docs: reordenar matriz 2 por objetivos de forma ascendente
</commit_message>
<xml_diff>
--- a/docs/entregables/PRACTICA EMPRESARIAL/GRUPO2_FIREFOX_MATRICES_COMPLETAS.xlsx
+++ b/docs/entregables/PRACTICA EMPRESARIAL/GRUPO2_FIREFOX_MATRICES_COMPLETAS.xlsx
@@ -180,7 +180,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -254,11 +254,12 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -357,6 +358,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2575,22 +2577,22 @@
     <row r="28" ht="45" customHeight="1" s="1">
       <c r="A28" s="33" t="inlineStr">
         <is>
-          <t>Diagrama de Arquitectura de Sistemas (C4)</t>
+          <t>Diagrama de Estados del Asiento (Máquina de Estados)</t>
         </is>
       </c>
       <c r="B28" s="31" t="inlineStr">
         <is>
-          <t>Obj. 2 - Validación de disponibilidad</t>
+          <t>Obj. 1 - Bloqueo transaccional</t>
         </is>
       </c>
       <c r="C28" s="31" t="inlineStr">
         <is>
-          <t>Visión arquitectónica de nivel Sistema, Contenedores y Componentes.</t>
+          <t>Evolución lógica de un asiento desde LIBRE hasta ABORDADO o CANCELADO.</t>
         </is>
       </c>
       <c r="D28" s="31" t="inlineStr">
         <is>
-          <t>docs/arquitectura/arquitectura_sistema.md</t>
+          <t>docs/diagramas/diagrama_estados_asiento.md</t>
         </is>
       </c>
       <c r="E28" s="30" t="inlineStr">
@@ -2602,7 +2604,7 @@
     <row r="29" ht="45" customHeight="1" s="1">
       <c r="A29" s="31" t="inlineStr">
         <is>
-          <t>Documento Técnico de Justificación CQRS</t>
+          <t>Diagrama de Arquitectura de Sistemas (C4)</t>
         </is>
       </c>
       <c r="B29" s="31" t="inlineStr">
@@ -2612,12 +2614,12 @@
       </c>
       <c r="C29" s="31" t="inlineStr">
         <is>
-          <t>Explicación del patrón de Separación de Responsabilidades para alta carga.</t>
+          <t>Visión arquitectónica de nivel Sistema, Contenedores y Componentes.</t>
         </is>
       </c>
       <c r="D29" s="31" t="inlineStr">
         <is>
-          <t>docs/arquitectura/arquitectura_cqrs_objetivo_2.md</t>
+          <t>docs/arquitectura/arquitectura_sistema.md</t>
         </is>
       </c>
       <c r="E29" s="30" t="inlineStr">
@@ -2629,7 +2631,7 @@
     <row r="30" ht="45" customHeight="1" s="1">
       <c r="A30" s="31" t="inlineStr">
         <is>
-          <t>Servicio Desacoplado de Disponibilidad</t>
+          <t>Documento Técnico de Justificación CQRS</t>
         </is>
       </c>
       <c r="B30" s="31" t="inlineStr">
@@ -2639,12 +2641,12 @@
       </c>
       <c r="C30" s="31" t="inlineStr">
         <is>
-          <t>Lógica de negocio aislada puramente para consultas masivas de vuelos (Read-Model).</t>
+          <t>Explicación del patrón de Separación de Responsabilidades para alta carga.</t>
         </is>
       </c>
       <c r="D30" s="31" t="inlineStr">
         <is>
-          <t>app/services/disponibilidad_service.py</t>
+          <t>docs/arquitectura/arquitectura_cqrs_objetivo_2.md</t>
         </is>
       </c>
       <c r="E30" s="30" t="inlineStr">
@@ -2656,7 +2658,7 @@
     <row r="31" ht="45" customHeight="1" s="1">
       <c r="A31" s="31" t="inlineStr">
         <is>
-          <t>Endpoints Optimizados de Búsqueda (API)</t>
+          <t>Servicio Desacoplado de Disponibilidad</t>
         </is>
       </c>
       <c r="B31" s="31" t="inlineStr">
@@ -2666,12 +2668,12 @@
       </c>
       <c r="C31" s="31" t="inlineStr">
         <is>
-          <t>Rutas HTTP (GET) exclusivas para alimentar sistemas de frontend rápidamente.</t>
+          <t>Lógica de negocio aislada puramente para consultas masivas de vuelos (Read-Model).</t>
         </is>
       </c>
       <c r="D31" s="31" t="inlineStr">
         <is>
-          <t>app/api/v1/disponibilidad.py</t>
+          <t>app/services/disponibilidad_service.py</t>
         </is>
       </c>
       <c r="E31" s="30" t="inlineStr">
@@ -2683,7 +2685,7 @@
     <row r="32" ht="45" customHeight="1" s="1">
       <c r="A32" s="31" t="inlineStr">
         <is>
-          <t>Monitoreo de Salud del Sistema (Healthcheck)</t>
+          <t>Endpoints Optimizados de Búsqueda (API)</t>
         </is>
       </c>
       <c r="B32" s="31" t="inlineStr">
@@ -2693,12 +2695,12 @@
       </c>
       <c r="C32" s="31" t="inlineStr">
         <is>
-          <t>Endpoint de verificación de estado para balanceadores de carga.</t>
+          <t>Rutas HTTP (GET) exclusivas para alimentar sistemas de frontend rápidamente.</t>
         </is>
       </c>
       <c r="D32" s="31" t="inlineStr">
         <is>
-          <t>app/api/v1/health.py</t>
+          <t>app/api/v1/disponibilidad.py</t>
         </is>
       </c>
       <c r="E32" s="30" t="inlineStr">
@@ -2710,7 +2712,7 @@
     <row r="33" ht="45" customHeight="1" s="1">
       <c r="A33" s="31" t="inlineStr">
         <is>
-          <t>Dockerfile de Aplicación API</t>
+          <t>Monitoreo de Salud del Sistema (Healthcheck)</t>
         </is>
       </c>
       <c r="B33" s="31" t="inlineStr">
@@ -2720,12 +2722,12 @@
       </c>
       <c r="C33" s="31" t="inlineStr">
         <is>
-          <t>Imagen de contenedor optimizada para el entorno de ejecución Python.</t>
+          <t>Endpoint de verificación de estado para balanceadores de carga.</t>
         </is>
       </c>
       <c r="D33" s="31" t="inlineStr">
         <is>
-          <t>docker/Dockerfile</t>
+          <t>app/api/v1/health.py</t>
         </is>
       </c>
       <c r="E33" s="30" t="inlineStr">
@@ -2737,7 +2739,7 @@
     <row r="34" ht="45" customHeight="1" s="1">
       <c r="A34" s="31" t="inlineStr">
         <is>
-          <t>Orquestación de Infraestructura (Docker Compose)</t>
+          <t>Dockerfile de Aplicación API</t>
         </is>
       </c>
       <c r="B34" s="31" t="inlineStr">
@@ -2747,12 +2749,12 @@
       </c>
       <c r="C34" s="31" t="inlineStr">
         <is>
-          <t>Topología de servicios que incluye DB, App y futuras expansiones de Caché.</t>
+          <t>Imagen de contenedor optimizada para el entorno de ejecución Python.</t>
         </is>
       </c>
       <c r="D34" s="31" t="inlineStr">
         <is>
-          <t>docker/docker-compose.yml</t>
+          <t>docker/Dockerfile</t>
         </is>
       </c>
       <c r="E34" s="30" t="inlineStr">
@@ -2764,88 +2766,88 @@
     <row r="35" ht="45" customHeight="1" s="1">
       <c r="A35" s="31" t="inlineStr">
         <is>
-          <t>Cliente y Configuración Caché (Valkey)</t>
+          <t>Orquestación de Infraestructura (Docker Compose)</t>
         </is>
       </c>
       <c r="B35" s="31" t="inlineStr">
         <is>
-          <t>Obj. 3 - Capa de caché</t>
+          <t>Obj. 2 - Validación de disponibilidad</t>
         </is>
       </c>
       <c r="C35" s="31" t="inlineStr">
         <is>
-          <t>Lógica de conexión, seteo y lectura rápida desde memoria RAM.</t>
+          <t>Topología de servicios que incluye DB, App y futuras expansiones de Caché.</t>
         </is>
       </c>
       <c r="D35" s="31" t="inlineStr">
         <is>
-          <t>app/db/cache.py</t>
-        </is>
-      </c>
-      <c r="E35" s="34" t="inlineStr">
-        <is>
-          <t>○ Pendiente</t>
+          <t>docker/docker-compose.yml</t>
+        </is>
+      </c>
+      <c r="E35" s="30" t="inlineStr">
+        <is>
+          <t>Disponible</t>
         </is>
       </c>
     </row>
     <row r="36" ht="45" customHeight="1" s="1">
       <c r="A36" s="31" t="inlineStr">
         <is>
-          <t>Inyección de Caché en Disponibilidad</t>
+          <t>Diagrama de Flujo: Sincronización CQRS</t>
         </is>
       </c>
       <c r="B36" s="31" t="inlineStr">
         <is>
-          <t>Obj. 3 - Capa de caché</t>
+          <t>Obj. 2 - Validación de disponibilidad</t>
         </is>
       </c>
       <c r="C36" s="31" t="inlineStr">
         <is>
-          <t>El servicio leerá primero de Valkey antes de saturar Postgres.</t>
+          <t>Propagación de eventos de la Write API hacia la Read API.</t>
         </is>
       </c>
       <c r="D36" s="31" t="inlineStr">
         <is>
-          <t>app/services/disponibilidad_service.py</t>
-        </is>
-      </c>
-      <c r="E36" s="34" t="inlineStr">
-        <is>
-          <t>○ Pendiente</t>
+          <t>docs/diagramas/diagrama_sincronizacion_cqrs.md</t>
+        </is>
+      </c>
+      <c r="E36" s="30" t="inlineStr">
+        <is>
+          <t>Disponible</t>
         </is>
       </c>
     </row>
     <row r="37" ht="45" customHeight="1" s="1">
       <c r="A37" s="31" t="inlineStr">
         <is>
-          <t>Servidor Valkey en Infraestructura</t>
+          <t>Diagrama de Componentes de Backend</t>
         </is>
       </c>
       <c r="B37" s="31" t="inlineStr">
         <is>
-          <t>Obj. 3 - Capa de caché</t>
+          <t>Obj. 2 - Validación de disponibilidad</t>
         </is>
       </c>
       <c r="C37" s="31" t="inlineStr">
         <is>
-          <t>El nodo de caché dentro de Docker Compose listo para usarse.</t>
+          <t>Mapeo interno de routers, servicios y repositorios en FastAPI.</t>
         </is>
       </c>
       <c r="D37" s="31" t="inlineStr">
         <is>
-          <t>docker/docker-compose.yml</t>
-        </is>
-      </c>
-      <c r="E37" s="34" t="inlineStr">
-        <is>
-          <t>○ Pendiente</t>
+          <t>docs/diagramas/diagrama_componentes_backend.md</t>
+        </is>
+      </c>
+      <c r="E37" s="30" t="inlineStr">
+        <is>
+          <t>Disponible</t>
         </is>
       </c>
     </row>
     <row r="38" ht="45" customHeight="1" s="1">
       <c r="A38" s="31" t="inlineStr">
         <is>
-          <t>Políticas de Invalidación y TTL</t>
+          <t>Cliente y Configuración Caché (Valkey)</t>
         </is>
       </c>
       <c r="B38" s="31" t="inlineStr">
@@ -2855,12 +2857,12 @@
       </c>
       <c r="C38" s="31" t="inlineStr">
         <is>
-          <t>Documentación y reglas técnicas sobre cuándo expira el caché de vuelos.</t>
+          <t>Lógica de conexión, seteo y lectura rápida desde memoria RAM.</t>
         </is>
       </c>
       <c r="D38" s="31" t="inlineStr">
         <is>
-          <t>docs/arquitectura/politicas_cache.md</t>
+          <t>app/db/cache.py</t>
         </is>
       </c>
       <c r="E38" s="34" t="inlineStr">
@@ -2872,7 +2874,7 @@
     <row r="39" ht="45" customHeight="1" s="1">
       <c r="A39" s="31" t="inlineStr">
         <is>
-          <t>Pruebas de Resiliencia de Caché</t>
+          <t>Inyección de Caché en Disponibilidad</t>
         </is>
       </c>
       <c r="B39" s="31" t="inlineStr">
@@ -2882,12 +2884,12 @@
       </c>
       <c r="C39" s="31" t="inlineStr">
         <is>
-          <t>Pruebas de Circuit Breaker (si Valkey cae, el sistema sobrevive usando Postgres).</t>
+          <t>El servicio leerá primero de Valkey antes de saturar Postgres.</t>
         </is>
       </c>
       <c r="D39" s="31" t="inlineStr">
         <is>
-          <t>tests/test_cache_resilience.py</t>
+          <t>app/services/disponibilidad_service.py</t>
         </is>
       </c>
       <c r="E39" s="34" t="inlineStr">
@@ -2899,22 +2901,22 @@
     <row r="40" ht="45" customHeight="1" s="1">
       <c r="A40" s="31" t="inlineStr">
         <is>
-          <t>Documento Protocolo Pruebas de Estrés K6</t>
+          <t>Servidor Valkey en Infraestructura</t>
         </is>
       </c>
       <c r="B40" s="31" t="inlineStr">
         <is>
-          <t>Obj. 4 - Protocolo de estrés</t>
+          <t>Obj. 3 - Capa de caché</t>
         </is>
       </c>
       <c r="C40" s="31" t="inlineStr">
         <is>
-          <t>Definición formal de SLAs, umbrales de fallo y escenarios (ej. Vuelos Azules).</t>
+          <t>El nodo de caché dentro de Docker Compose listo para usarse.</t>
         </is>
       </c>
       <c r="D40" s="31" t="inlineStr">
         <is>
-          <t>docs/testing/protocolo_pruebas_estres.md</t>
+          <t>docker/docker-compose.yml</t>
         </is>
       </c>
       <c r="E40" s="34" t="inlineStr">
@@ -2926,22 +2928,22 @@
     <row r="41" ht="45" customHeight="1" s="1">
       <c r="A41" s="31" t="inlineStr">
         <is>
-          <t>Guía de Generación de Logs de Auditoría</t>
+          <t>Políticas de Invalidación y TTL</t>
         </is>
       </c>
       <c r="B41" s="31" t="inlineStr">
         <is>
-          <t>Obj. 4 - Protocolo de estrés</t>
+          <t>Obj. 3 - Capa de caché</t>
         </is>
       </c>
       <c r="C41" s="31" t="inlineStr">
         <is>
-          <t>Instrucciones precisas para capturar evidencias de caídas de latencia.</t>
+          <t>Documentación y reglas técnicas sobre cuándo expira el caché de vuelos.</t>
         </is>
       </c>
       <c r="D41" s="31" t="inlineStr">
         <is>
-          <t>docs/testing/como_generar_logs.md</t>
+          <t>docs/arquitectura/politicas_cache.md</t>
         </is>
       </c>
       <c r="E41" s="34" t="inlineStr">
@@ -2953,22 +2955,22 @@
     <row r="42" ht="45" customHeight="1" s="1">
       <c r="A42" s="31" t="inlineStr">
         <is>
-          <t>Script de Carga Masiva Automatizada (K6)</t>
+          <t>Pruebas de Resiliencia de Caché</t>
         </is>
       </c>
       <c r="B42" s="31" t="inlineStr">
         <is>
-          <t>Obj. 4 - Protocolo de estrés</t>
+          <t>Obj. 3 - Capa de caché</t>
         </is>
       </c>
       <c r="C42" s="31" t="inlineStr">
         <is>
-          <t>El archivo JS que dispara miles de requests concurrentes al servidor.</t>
+          <t>Pruebas de Circuit Breaker (si Valkey cae, el sistema sobrevive usando Postgres).</t>
         </is>
       </c>
       <c r="D42" s="31" t="inlineStr">
         <is>
-          <t>scripts/load_test_k6.js</t>
+          <t>tests/test_cache_resilience.py</t>
         </is>
       </c>
       <c r="E42" s="34" t="inlineStr">
@@ -2980,22 +2982,22 @@
     <row r="43" ht="45" customHeight="1" s="1">
       <c r="A43" s="31" t="inlineStr">
         <is>
-          <t>Plan Maestro de Ejecución BoA</t>
+          <t>Diagrama de Secuencia: Flujo Cache-Aside</t>
         </is>
       </c>
       <c r="B43" s="31" t="inlineStr">
         <is>
-          <t>Obj. 4 - Protocolo de estrés</t>
+          <t>Obj. 3 - Capa de caché</t>
         </is>
       </c>
       <c r="C43" s="31" t="inlineStr">
         <is>
-          <t>Cronograma, roles y plan general que sustenta la ejecución del proyecto.</t>
+          <t>Decisión del sistema entre recuperar de RAM o calcular desde BD.</t>
         </is>
       </c>
       <c r="D43" s="31" t="inlineStr">
         <is>
-          <t>docs/planificacion/plan_maestro_boa.md</t>
+          <t>docs/diagramas/diagrama_flujo_cache.md</t>
         </is>
       </c>
       <c r="E43" s="34" t="inlineStr">
@@ -3007,103 +3009,103 @@
     <row r="44" ht="45" customHeight="1" s="1">
       <c r="A44" s="31" t="inlineStr">
         <is>
-          <t>Diagrama de Estados del Asiento (Máquina de Estados)</t>
+          <t>Documento Protocolo Pruebas de Estrés K6</t>
         </is>
       </c>
       <c r="B44" s="31" t="inlineStr">
         <is>
-          <t>Obj. 1 - Bloqueo transaccional</t>
+          <t>Obj. 4 - Protocolo de estrés</t>
         </is>
       </c>
       <c r="C44" s="31" t="inlineStr">
         <is>
-          <t>Evolución lógica de un asiento desde LIBRE hasta ABORDADO o CANCELADO.</t>
+          <t>Definición formal de SLAs, umbrales de fallo y escenarios (ej. Vuelos Azules).</t>
         </is>
       </c>
       <c r="D44" s="31" t="inlineStr">
         <is>
-          <t>docs/diagramas/diagrama_estados_asiento.md</t>
-        </is>
-      </c>
-      <c r="E44" s="30" t="inlineStr">
-        <is>
-          <t>Disponible</t>
+          <t>docs/testing/protocolo_pruebas_estres.md</t>
+        </is>
+      </c>
+      <c r="E44" s="34" t="inlineStr">
+        <is>
+          <t>○ Pendiente</t>
         </is>
       </c>
     </row>
     <row r="45" ht="45" customHeight="1" s="1">
       <c r="A45" s="31" t="inlineStr">
         <is>
-          <t>Diagrama de Flujo: Sincronización CQRS</t>
+          <t>Guía de Generación de Logs de Auditoría</t>
         </is>
       </c>
       <c r="B45" s="31" t="inlineStr">
         <is>
-          <t>Obj. 2 - Validación de disponibilidad</t>
+          <t>Obj. 4 - Protocolo de estrés</t>
         </is>
       </c>
       <c r="C45" s="31" t="inlineStr">
         <is>
-          <t>Propagación de eventos de la Write API hacia la Read API.</t>
+          <t>Instrucciones precisas para capturar evidencias de caídas de latencia.</t>
         </is>
       </c>
       <c r="D45" s="31" t="inlineStr">
         <is>
-          <t>docs/diagramas/diagrama_sincronizacion_cqrs.md</t>
-        </is>
-      </c>
-      <c r="E45" s="30" t="inlineStr">
-        <is>
-          <t>Disponible</t>
+          <t>docs/testing/como_generar_logs.md</t>
+        </is>
+      </c>
+      <c r="E45" s="34" t="inlineStr">
+        <is>
+          <t>○ Pendiente</t>
         </is>
       </c>
     </row>
     <row r="46" ht="45" customHeight="1" s="1">
       <c r="A46" s="31" t="inlineStr">
         <is>
-          <t>Diagrama de Componentes de Backend</t>
+          <t>Script de Carga Masiva Automatizada (K6)</t>
         </is>
       </c>
       <c r="B46" s="31" t="inlineStr">
         <is>
-          <t>Obj. 2 - Validación de disponibilidad</t>
+          <t>Obj. 4 - Protocolo de estrés</t>
         </is>
       </c>
       <c r="C46" s="31" t="inlineStr">
         <is>
-          <t>Mapeo interno de routers, servicios y repositorios en FastAPI.</t>
+          <t>El archivo JS que dispara miles de requests concurrentes al servidor.</t>
         </is>
       </c>
       <c r="D46" s="31" t="inlineStr">
         <is>
-          <t>docs/diagramas/diagrama_componentes_backend.md</t>
-        </is>
-      </c>
-      <c r="E46" s="30" t="inlineStr">
-        <is>
-          <t>Disponible</t>
+          <t>scripts/load_test_k6.js</t>
+        </is>
+      </c>
+      <c r="E46" s="34" t="inlineStr">
+        <is>
+          <t>○ Pendiente</t>
         </is>
       </c>
     </row>
     <row r="47" ht="45" customHeight="1" s="1">
       <c r="A47" s="31" t="inlineStr">
         <is>
-          <t>Diagrama de Secuencia: Flujo Cache-Aside</t>
+          <t>Plan Maestro de Ejecución BoA</t>
         </is>
       </c>
       <c r="B47" s="31" t="inlineStr">
         <is>
-          <t>Obj. 3 - Capa de caché</t>
+          <t>Obj. 4 - Protocolo de estrés</t>
         </is>
       </c>
       <c r="C47" s="31" t="inlineStr">
         <is>
-          <t>Decisión del sistema entre recuperar de RAM o calcular desde BD.</t>
+          <t>Cronograma, roles y plan general que sustenta la ejecución del proyecto.</t>
         </is>
       </c>
       <c r="D47" s="31" t="inlineStr">
         <is>
-          <t>docs/diagramas/diagrama_flujo_cache.md</t>
+          <t>docs/planificacion/plan_maestro_boa.md</t>
         </is>
       </c>
       <c r="E47" s="34" t="inlineStr">
@@ -3167,74 +3169,74 @@
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="1">
-      <c r="A50" s="35" t="inlineStr"/>
-      <c r="B50" s="35" t="inlineStr"/>
-      <c r="C50" s="35" t="inlineStr"/>
-      <c r="D50" s="35" t="inlineStr"/>
-      <c r="E50" s="35" t="inlineStr"/>
+      <c r="A50" s="36" t="inlineStr"/>
+      <c r="B50" s="36" t="inlineStr"/>
+      <c r="C50" s="36" t="inlineStr"/>
+      <c r="D50" s="36" t="inlineStr"/>
+      <c r="E50" s="36" t="inlineStr"/>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="1">
-      <c r="A51" s="35" t="inlineStr"/>
-      <c r="B51" s="35" t="inlineStr"/>
-      <c r="C51" s="35" t="inlineStr"/>
-      <c r="D51" s="35" t="inlineStr"/>
-      <c r="E51" s="35" t="inlineStr"/>
+      <c r="A51" s="36" t="inlineStr"/>
+      <c r="B51" s="36" t="inlineStr"/>
+      <c r="C51" s="36" t="inlineStr"/>
+      <c r="D51" s="36" t="inlineStr"/>
+      <c r="E51" s="36" t="inlineStr"/>
     </row>
     <row r="52" ht="15.75" customHeight="1" s="1">
-      <c r="A52" s="35" t="inlineStr"/>
-      <c r="B52" s="35" t="inlineStr"/>
-      <c r="C52" s="35" t="inlineStr"/>
-      <c r="D52" s="35" t="inlineStr"/>
-      <c r="E52" s="35" t="inlineStr"/>
+      <c r="A52" s="36" t="inlineStr"/>
+      <c r="B52" s="36" t="inlineStr"/>
+      <c r="C52" s="36" t="inlineStr"/>
+      <c r="D52" s="36" t="inlineStr"/>
+      <c r="E52" s="36" t="inlineStr"/>
     </row>
     <row r="53" ht="15.75" customHeight="1" s="1">
-      <c r="A53" s="35" t="inlineStr"/>
-      <c r="B53" s="35" t="inlineStr"/>
-      <c r="C53" s="35" t="inlineStr"/>
-      <c r="D53" s="35" t="inlineStr"/>
-      <c r="E53" s="35" t="inlineStr"/>
+      <c r="A53" s="36" t="inlineStr"/>
+      <c r="B53" s="36" t="inlineStr"/>
+      <c r="C53" s="36" t="inlineStr"/>
+      <c r="D53" s="36" t="inlineStr"/>
+      <c r="E53" s="36" t="inlineStr"/>
     </row>
     <row r="54" ht="15.75" customHeight="1" s="1">
-      <c r="A54" s="35" t="inlineStr"/>
-      <c r="B54" s="35" t="inlineStr"/>
-      <c r="C54" s="35" t="inlineStr"/>
-      <c r="D54" s="35" t="inlineStr"/>
-      <c r="E54" s="35" t="inlineStr"/>
+      <c r="A54" s="36" t="inlineStr"/>
+      <c r="B54" s="36" t="inlineStr"/>
+      <c r="C54" s="36" t="inlineStr"/>
+      <c r="D54" s="36" t="inlineStr"/>
+      <c r="E54" s="36" t="inlineStr"/>
     </row>
     <row r="55" ht="15.75" customHeight="1" s="1">
-      <c r="A55" s="35" t="inlineStr"/>
-      <c r="B55" s="35" t="inlineStr"/>
-      <c r="C55" s="35" t="inlineStr"/>
-      <c r="D55" s="35" t="inlineStr"/>
-      <c r="E55" s="35" t="inlineStr"/>
+      <c r="A55" s="36" t="inlineStr"/>
+      <c r="B55" s="36" t="inlineStr"/>
+      <c r="C55" s="36" t="inlineStr"/>
+      <c r="D55" s="36" t="inlineStr"/>
+      <c r="E55" s="36" t="inlineStr"/>
     </row>
     <row r="56" ht="15.75" customHeight="1" s="1">
-      <c r="A56" s="35" t="inlineStr"/>
-      <c r="B56" s="35" t="inlineStr"/>
-      <c r="C56" s="35" t="inlineStr"/>
-      <c r="D56" s="35" t="inlineStr"/>
-      <c r="E56" s="35" t="inlineStr"/>
+      <c r="A56" s="36" t="inlineStr"/>
+      <c r="B56" s="36" t="inlineStr"/>
+      <c r="C56" s="36" t="inlineStr"/>
+      <c r="D56" s="36" t="inlineStr"/>
+      <c r="E56" s="36" t="inlineStr"/>
     </row>
     <row r="57" ht="15.75" customHeight="1" s="1">
-      <c r="A57" s="35" t="inlineStr"/>
-      <c r="B57" s="35" t="inlineStr"/>
-      <c r="C57" s="35" t="inlineStr"/>
-      <c r="D57" s="35" t="inlineStr"/>
-      <c r="E57" s="35" t="inlineStr"/>
+      <c r="A57" s="36" t="inlineStr"/>
+      <c r="B57" s="36" t="inlineStr"/>
+      <c r="C57" s="36" t="inlineStr"/>
+      <c r="D57" s="36" t="inlineStr"/>
+      <c r="E57" s="36" t="inlineStr"/>
     </row>
     <row r="58" ht="15.75" customHeight="1" s="1">
-      <c r="A58" s="35" t="inlineStr"/>
-      <c r="B58" s="35" t="inlineStr"/>
-      <c r="C58" s="35" t="inlineStr"/>
-      <c r="D58" s="35" t="inlineStr"/>
-      <c r="E58" s="35" t="inlineStr"/>
+      <c r="A58" s="36" t="inlineStr"/>
+      <c r="B58" s="36" t="inlineStr"/>
+      <c r="C58" s="36" t="inlineStr"/>
+      <c r="D58" s="36" t="inlineStr"/>
+      <c r="E58" s="36" t="inlineStr"/>
     </row>
     <row r="59" ht="15.75" customHeight="1" s="1">
-      <c r="A59" s="35" t="inlineStr"/>
-      <c r="B59" s="35" t="inlineStr"/>
-      <c r="C59" s="35" t="inlineStr"/>
-      <c r="D59" s="35" t="inlineStr"/>
-      <c r="E59" s="35" t="inlineStr"/>
+      <c r="A59" s="36" t="inlineStr"/>
+      <c r="B59" s="36" t="inlineStr"/>
+      <c r="C59" s="36" t="inlineStr"/>
+      <c r="D59" s="36" t="inlineStr"/>
+      <c r="E59" s="36" t="inlineStr"/>
     </row>
     <row r="60" ht="15.75" customHeight="1" s="1">
       <c r="A60" s="35" t="inlineStr"/>

</xml_diff>